<commit_message>
removed grey text and updated spreadsheet
</commit_message>
<xml_diff>
--- a/bec/TA_Exfil_logs_BEC_projvictoria_final.xlsx
+++ b/bec/TA_Exfil_logs_BEC_projvictoria_final.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kris\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F27755D7-BDCB-455B-BFEA-55941A72B8AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2ABEF4E-8DA0-4658-AD53-82217B14BC6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{51077852-24B8-4DBB-BC98-89EBBD13A684}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{51077852-24B8-4DBB-BC98-89EBBD13A684}"/>
   </bookViews>
   <sheets>
     <sheet name="Key Events" sheetId="5" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3312" uniqueCount="752">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3142" uniqueCount="696">
   <si>
     <t>TenantId</t>
   </si>
@@ -1609,183 +1609,15 @@
     <t>AdditionalDetails</t>
   </si>
   <si>
-    <t>2/28/2026, 11:56:26.727 PM</t>
-  </si>
-  <si>
     <t>Update user</t>
   </si>
   <si>
-    <t>[{"id":"9ebb7bc1-ad39-486e-9bf5-056f352fed91","displayName":null,"type":"User","modifiedProperties":[{"displayName":"StrongAuthenticationPhoneAppDetail","oldValue":"[{\"DeviceName\":\"NO_DEVICE\",\"DeviceToken\":\"NO_DEVICE_TOKEN\",\"DeviceTag\":\"SoftwareTokenActivated\",\"PhoneAppVersion\":\"NO_PHONE_APP_VERSION\",\"OathTokenTimeDrift\":0,\"DeviceId\":\"00000000-0000-0000-0000-000000000000\",\"Id\":\"1378ded7-887e-417d-9f8c-0535c94eae5b\",\"TimeInterval\":0,\"AuthenticationType\":2,\"NotificationType\":1,\"LastAuthenticatedTimestamp\":\"2026-02-25T21:17:48.8656208Z\",\"AuthenticatorFlavor\":\"Authenticator\",\"HashFunction\":\"hmacsha1\",\"TenantDeviceId\":null,\"SecuredPartitionId\":20102,\"SecuredKeyId\":7}]","newValue":"[{\"DeviceName\":\"NO_DEVICE\",\"DeviceToken\":\"NO_DEVICE_TOKEN\",\"DeviceTag\":\"SoftwareTokenActivated\",\"PhoneAppVersion\":\"NO_PHONE_APP_VERSION\",\"OathTokenTimeDrift\":0,\"DeviceId\":\"00000000-0000-0000-0000-000000000000\",\"Id\":\"1378ded7-887e-417d-9f8c-0535c94eae5b\",\"TimeInterval\":0,\"AuthenticationType\":2,\"NotificationType\":1,\"LastAuthenticatedTimestamp\":\"2026-02-28T23:56:26.5933494Z\",\"AuthenticatorFlavor\":\"Authenticator\",\"HashFunction\":\"hmacsha1\",\"TenantDeviceId\":null,\"SecuredPartitionId\":20102,\"SecuredKeyId\":7}]"},{"displayName":"Included Updated Properties","oldValue":null,"newValue":"\"StrongAuthenticationPhoneAppDetail\""},{"displayName":"TargetId.UserType","oldValue":null,"newValue":"\"Member\""}],"administrativeUnits":[],"agentType":"notAgentic","userPrincipalName":"donald.anderson@wdlabs.com.au"}]</t>
-  </si>
-  <si>
     <t>success</t>
   </si>
   <si>
-    <t>[{"key":"UserType","value":"Member"}]</t>
-  </si>
-  <si>
-    <t>3/1/2026, 5:19:54.677 AM</t>
-  </si>
-  <si>
-    <t>[{"id":"9ebb7bc1-ad39-486e-9bf5-056f352fed91","displayName":null,"type":"User","modifiedProperties":[],"administrativeUnits":[],"agentType":"notAgentic","userPrincipalName":"donald.anderson@wdlabs.com.au"}]</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"5d931786-8141-4696-963e-487cf1663b83"},{"key":"seq","value":"1"},{"key":"b","value":"{\"targetUpdatedProperties\":\"[{\\\"Name\\\":\\\"AssignedLicense\\\",\\\"OldValue\\\":[\\\"[SkuName=EXCHANGESTANDARD, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=4b9405b0-7788-4568-add1-99614e613b69, DisabledPlans=[]]\\\",\\\"[SkuName=AAD_PREMIUM_P2, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=84a661c4-e949-4bd2-a560-ed7766fcaf2b, DisabledPlans=[]]\\\",\\\"[SkuName=Microsoft_Teams_Exploratory_Dept, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=e0dfc8b9-9531-4ec8-94b4-9fec23b05fc8, DisabledPlans=[EXCHANGE_S_STANDARD]]\\\"],\\\"NewValue\\\":[\\\"[SkuName=Microsoft_Teams_Exploratory_Dept, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=e0dfc8b9-9531-4ec8-94b4-9fec23b05fc8, DisabledPlans=[EXCHANGE_S_STANDARD]]\\\",\\\"[SkuName=AAD_PREMIUM_P2, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=84a661c4-e949-4bd2-a560-ed7766fcaf2b, DisabledPlans=[]]\\\",\\\"[SkuName=EXCHANGESTANDARD, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=4b9405b0-7788-4568-add1-99614e613b69, DisabledPlans=[]]\\\",\\\"[SkuName=SPB, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=cbdc14ab-d96c-4c30-b9f4-6ada7cdc1d46, DisabledPlans=[]]\\\"]},{\\\"Name\\\":\\\"AssignedPlan\\\",\\\"OldValue\\\":[{\\\"SubscribedPlanId\\\":\\\"0dfd484c-cc3b-4cd7-be8e-e51c1b4bc0ea\\\",\\\"ServiceInstance\\\":\\\"Sway/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a23b959c-7ce8-4e57-9140-b90eb88a9e97\\\"},{\\\"SubscribedPlanId\\\":\\\"0e6e1ecc-f9bf-4414-9e6f-1828660fd975\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"40b010bb-0b69-4654-ac5e-ba161433f4b4\\\"},{\\\"SubscribedPlanId\\\":\\\"11013c80-c192-4862-bbb5-7b86a741c83a\\\",\\\"ServiceInstance\\\":\\\"WhiteboardServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b8afc642-032e-4de5-8c0a-507a7bba7e5d\\\"},{\\\"SubscribedPlanId\\\":\\\"11b27917-6674-453b-9913-cba7aba6883a\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"dcf9d2f4-772e-4434-b757-77a453cfbc02\\\"},{\\\"SubscribedPlanId\\\":\\\"177b15ab-51b1-47d1-b213-f0e968822a83\\\",\\\"ServiceInstance\\\":\\\"MultiFactorService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8a256a2b-b617-496d-b51b-e76466e88db0\\\"},{\\\"SubscribedPlanId\\\":\\\"1a6d321c-ebe3-4198-8527-0d14340c3009\\\",\\\"ServiceInstance\\\":\\\"ProcessSimple/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0f9b09cb-62d1-4ff4-9129-43f4996f83f4\\\"},{\\\"SubscribedPlanId\\\":\\\"1b044c1d-0c69-4b8d-8b93-03c2ef1fd3da\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c7699d2e-19aa-44de-8edf-1736da088ca1\\\"},{\\\"SubscribedPlanId\\\":\\\"2287b27a-b6ec-40e6-bb03-35170aa2c846\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"41781fb2-bc02-4b7c-bd55-b576c07bb09d\\\"},{\\\"SubscribedPlanId\\\":\\\"3ef79a81-ae21-49b8-8fa7-dc1d795d9671\\\",\\\"ServiceInstance\\\":\\\"ProjectProgramsAndPortfolios/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a55dfd10-0864-46d9-a3cd-da5991a3e0e2\\\"},{\\\"SubscribedPlanId\\\":\\\"449a3874-a6a4-498d-905d-662cfc611bea\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"f0ff6ac6-297d-49cd-be34-6dfef97f0c28\\\"},{\\\"SubscribedPlanId\\\":\\\"529909ed-7627-4843-bb53-3556b852c9d9\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T20:21:00Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9aaf7827-d63c-4b61-89c3-182f06f82e5c\\\"},{\\\"SubscribedPlanId\\\":\\\"53ac6e25-a8f6-44bf-b402-9f56b8eecfd9\\\",\\\"ServiceInstance\\\":\\\"To-Do/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5e62787c-c316-451f-b873-1d05acd4d12c\\\"},{\\\"SubscribedPlanId\\\":\\\"6f907b14-cb0b-4a3a-9bb9-4f951739e103\\\",\\\"ServiceInstance\\\":\\\"Deskless/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8c7d2df8-86f0-4902-b2ed-a0458298f3b3\\\"},{\\\"SubscribedPlanId\\\":\\\"71ac5b1a-e1dc-4ced-ba2d-059d74e89acf\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"3efbd4ed-8958-4824-8389-1321f8730af8\\\"},{\\\"SubscribedPlanId\\\":\\\"85ff92c3-df66-4ccc-ba0b-38683b60b371\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"33c4f319-9bdd-48d6-9c4d-410b750a4a5a\\\"},{\\\"SubscribedPlanId\\\":\\\"88ae6c56-fccc-497d-9e45-c0ea113b9406\\\",\\\"ServiceInstance\\\":\\\"PowerAppsService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"92f7a6f3-b89b-4bbd-8c30-809e6da5ad1c\\\"},{\\\"SubscribedPlanId\\\":\\\"956ea907-9a03-46cd-8699-95667e82355a\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c63d4d19-e8cb-460e-b37c-4d6c34603745\\\"},{\\\"SubscribedPlanId\\\":\\\"a22189d7-70fa-482b-9d57-ada39f5e0872\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"eec0eb4f-6444-4f95-aba0-50c24d67f998\\\"},{\\\"SubscribedPlanId\\\":\\\"a5d43ea2-3323-489d-a579-068f683b41f7\\\",\\\"ServiceInstance\\\":\\\"ccibotsprod/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0683001c-0492-4d59-9515-d9a6426b5813\\\"},{\\\"SubscribedPlanId\\\":\\\"a83d2db3-81e2-45ee-bf0e-c1088b24bb96\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"e95bec33-7c88-4a70-8e19-b10bd9d0c014\\\"},{\\\"SubscribedPlanId\\\":\\\"b3ae2021-9f74-4a09-9845-42accad7b182\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bed136c6-b799-4462-824d-fc045d3a9d25\\\"},{\\\"SubscribedPlanId\\\":\\\"b7b9220c-a3f0-437e-b99a-0e925b312c86\\\",\\\"ServiceInstance\\\":\\\"YammerEnterprise/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"7547a3fe-08ee-4ccb-b430-5077c5041653\\\"},{\\\"SubscribedPlanId\\\":\\\"c73a8c4e-f6b6-4998-bf41-862fdea05abd\\\",\\\"ServiceInstance\\\":\\\"ProjectWorkManagement/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b737dad2-2f6c-4c65-90e3-ca563267e8b9\\\"},{\\\"SubscribedPlanId\\\":\\\"d1c57312-4814-4818-a991-38bb7429b211\\\",\\\"ServiceInstance\\\":\\\"TeamspaceAPI/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"57ff2da0-773e-42df-b2af-ffb7a2317929\\\"},{\\\"SubscribedPlanId\\\":\\\"dddc5824-34a0-4b85-b6b8-0fafe67a57b0\\\",\\\"ServiceInstance\\\":\\\"OfficeForms/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"159f4cd6-e380-449f-a816-af1a9ef76344\\\"},{\\\"SubscribedPlanId\\\":\\\"e039cc95-628d-4ade-80ce-f77a46135dde\\\",\\\"ServiceInstance\\\":\\\"MicrosoftStream/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"743dd19e-1ce3-4c62-a3ad-49ba8f63a2f6\\\"},{\\\"SubscribedPlanId\\\":\\\"e7733084-cf3d-4d56-9cfd-1cd9ea183052\\\",\\\"ServiceInstance\\\":\\\"Adallom/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"932ad362-64a8-4783-9106-97849a1a30b9\\\"},{\\\"SubscribedPlanId\\\":\\\"ea16e50b-9303-4b92-9e45-0c4c4f2482be\\\",\\\"ServiceInstance\\\":\\\"MicrosoftCommunicationsOnline/APAC-AU1-S1\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"42a3ec34-28ba-46b6-992f-db53a675ac5b\\\"}],\\\"NewValue\\\":[{\\\"SubscribedPlanId\\\":\\\"529909ed-7627-4843-bb53-3556b852c9d9\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6131188Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9aaf7827-d63c-4b61-89c3-182f06f82e5c\\\"},{\\\"SubscribedPlanId\\\":\\\"ea16e50b-9303-4b92-9e45-0c4c4f2482be\\\",\\\"ServiceInstance\\\":\\\"MicrosoftCommunicationsOnline/APAC-AU1-S1\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"42a3ec34-28ba-46b6-992f-db53a675ac5b\\\"},{\\\"SubscribedPlanId\\\":\\\"e039cc95-628d-4ade-80ce-f77a46135dde\\\",\\\"ServiceInstance\\\":\\\"MicrosoftStream/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"743dd19e-1ce3-4c62-a3ad-49ba8f63a2f6\\\"},{\\\"SubscribedPlanId\\\":\\\"dddc5824-34a0"},{"key":"c","value":"3"}]</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"5d931786-8141-4696-963e-487cf1663b83"},{"key":"seq","value":"2"},{"key":"b","value":"-4b85-b6b8-0fafe67a57b0\\\",\\\"ServiceInstance\\\":\\\"OfficeForms/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"159f4cd6-e380-449f-a816-af1a9ef76344\\\"},{\\\"SubscribedPlanId\\\":\\\"d1c57312-4814-4818-a991-38bb7429b211\\\",\\\"ServiceInstance\\\":\\\"TeamspaceAPI/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"57ff2da0-773e-42df-b2af-ffb7a2317929\\\"},{\\\"SubscribedPlanId\\\":\\\"c73a8c4e-f6b6-4998-bf41-862fdea05abd\\\",\\\"ServiceInstance\\\":\\\"ProjectWorkManagement/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b737dad2-2f6c-4c65-90e3-ca563267e8b9\\\"},{\\\"SubscribedPlanId\\\":\\\"b7b9220c-a3f0-437e-b99a-0e925b312c86\\\",\\\"ServiceInstance\\\":\\\"YammerEnterprise/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"7547a3fe-08ee-4ccb-b430-5077c5041653\\\"},{\\\"SubscribedPlanId\\\":\\\"b3ae2021-9f74-4a09-9845-42accad7b182\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bed136c6-b799-4462-824d-fc045d3a9d25\\\"},{\\\"SubscribedPlanId\\\":\\\"a83d2db3-81e2-45ee-bf0e-c1088b24bb96\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"e95bec33-7c88-4a70-8e19-b10bd9d0c014\\\"},{\\\"SubscribedPlanId\\\":\\\"a5d43ea2-3323-489d-a579-068f683b41f7\\\",\\\"ServiceInstance\\\":\\\"ccibotsprod/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0683001c-0492-4d59-9515-d9a6426b5813\\\"},{\\\"SubscribedPlanId\\\":\\\"956ea907-9a03-46cd-8699-95667e82355a\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c63d4d19-e8cb-460e-b37c-4d6c34603745\\\"},{\\\"SubscribedPlanId\\\":\\\"88ae6c56-fccc-497d-9e45-c0ea113b9406\\\",\\\"ServiceInstance\\\":\\\"PowerAppsService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"92f7a6f3-b89b-4bbd-8c30-809e6da5ad1c\\\"},{\\\"SubscribedPlanId\\\":\\\"85ff92c3-df66-4ccc-ba0b-38683b60b371\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"33c4f319-9bdd-48d6-9c4d-410b750a4a5a\\\"},{\\\"SubscribedPlanId\\\":\\\"71ac5b1a-e1dc-4ced-ba2d-059d74e89acf\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"3efbd4ed-8958-4824-8389-1321f8730af8\\\"},{\\\"SubscribedPlanId\\\":\\\"6f907b14-cb0b-4a3a-9bb9-4f951739e103\\\",\\\"ServiceInstance\\\":\\\"Deskless/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8c7d2df8-86f0-4902-b2ed-a0458298f3b3\\\"},{\\\"SubscribedPlanId\\\":\\\"53ac6e25-a8f6-44bf-b402-9f56b8eecfd9\\\",\\\"ServiceInstance\\\":\\\"To-Do/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5e62787c-c316-451f-b873-1d05acd4d12c\\\"},{\\\"SubscribedPlanId\\\":\\\"449a3874-a6a4-498d-905d-662cfc611bea\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"f0ff6ac6-297d-49cd-be34-6dfef97f0c28\\\"},{\\\"SubscribedPlanId\\\":\\\"3ef79a81-ae21-49b8-8fa7-dc1d795d9671\\\",\\\"ServiceInstance\\\":\\\"ProjectProgramsAndPortfolios/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a55dfd10-0864-46d9-a3cd-da5991a3e0e2\\\"},{\\\"SubscribedPlanId\\\":\\\"1b044c1d-0c69-4b8d-8b93-03c2ef1fd3da\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c7699d2e-19aa-44de-8edf-1736da088ca1\\\"},{\\\"SubscribedPlanId\\\":\\\"1a6d321c-ebe3-4198-8527-0d14340c3009\\\",\\\"ServiceInstance\\\":\\\"ProcessSimple/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0f9b09cb-62d1-4ff4-9129-43f4996f83f4\\\"},{\\\"SubscribedPlanId\\\":\\\"11b27917-6674-453b-9913-cba7aba6883a\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"dcf9d2f4-772e-4434-b757-77a453cfbc02\\\"},{\\\"SubscribedPlanId\\\":\\\"11013c80-c192-4862-bbb5-7b86a741c83a\\\",\\\"ServiceInstance\\\":\\\"WhiteboardServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b8afc642-032e-4de5-8c0a-507a7bba7e5d\\\"},{\\\"SubscribedPlanId\\\":\\\"0e6e1ecc-f9bf-4414-9e6f-1828660fd975\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"40b010bb-0b69-4654-ac5e-ba161433f4b4\\\"},{\\\"SubscribedPlanId\\\":\\\"0dfd484c-cc3b-4cd7-be8e-e51c1b4bc0ea\\\",\\\"ServiceInstance\\\":\\\"Sway/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a23b959c-7ce8-4e57-9140-b90eb88a9e97\\\"},{\\\"SubscribedPlanId\\\":\\\"e7733084-cf3d-4d56-9cfd-1cd9ea183052\\\",\\\"ServiceInstance\\\":\\\"Adallom/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"932ad362-64a8-4783-9106-97849a1a30b9\\\"},{\\\"SubscribedPlanId\\\":\\\"a22189d7-70fa-482b-9d57-ada39f5e0872\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"eec0eb4f-6444-4f95-aba0-50c24d67f998\\\"},{\\\"SubscribedPlanId\\\":\\\"2287b27a-b6ec-40e6-bb03-35170aa2c846\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"41781fb2-bc02-4b7c-bd55-b576c07bb09d\\\"},{\\\"SubscribedPlanId\\\":\\\"177b15ab-51b1-47d1-b213-f0e968822a83\\\",\\\"ServiceInstance\\\":\\\"MultiFactorService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8a256a2b-b617-496d-b51b-e76466e88db0\\\"},{\\\"SubscribedPlanId\\\":\\\"020805e7-7d5f-4bb3-b898-a3b1259a976f\\\",\\\"ServiceInstance\\\":\\\"VivaSkills/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6131188Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"13b6da2c-0d84-450e-9f69-a33e221387ca\\\"},{\\\"SubscribedPlanId\\\":\\\"694b4e1c-079c-4afe-9d08-f38537955130\\\",\\\"ServiceInstance\\\":\\\"OnlineService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6131188Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"1fe6227d-3e01-46d0-9510-0acad4ff6e94\\\"},{\\\"SubscribedPlanId\\\":\\\"f16c6e89-93cc-4fd6-b474-59b2cea0231b\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6141167Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a6520331-d7d4-4276-95f5-15c0933bc757\\\"},{\\\"SubscribedPlanId\\\":\\\"b7f56b27-f5ea-45fb-8884-1a5357c41c37\\\",\\\"ServiceInstance\\\":\\\"Microsoft.ProjectBabylon/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6141167Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c948ea65-2053-4a5a-8a62-9eaaaf11b522\\\"},{\\\"SubscribedPlanId\\\":\\\"22b5463b-d360-473f-80c2-be8e42afcc71\\\",\\\"ServiceInstance\\\":\\\"Chapter5FluidApp/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6141167Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c4b8c31a-fb44-4c65-9837-a21f55fcabda\\\"},{\\\"SubscribedPlanId\\\":\\\"c4031b28-43f8-42d9-b1f4-06f5b955074c\\\",\\\"ServiceInstance\\\":\\\"Bing/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6141167Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0d0c0d31-fae7-41f2-b909-eaf4d7f26dba\\\"},{\\\"SubscribedPlanId\\\":\\\"36e41faa-1e78-4c8b-8453-6b3ca38ab4c1\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6141167Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a1ace008-72f3-4ea0-8dac-33b3a23a2472\\\"},{\\\"SubscribedPlanId\\\":\\\"02e3d1d6-4434-4d5c-88b7-a35a509cce87\\\",\\\"ServiceInstance\\\":\\\"YammerEnterprise/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6141167Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a82fbf69-b4d7-49f4-83a6-915b2cf354f4\\\"},{\\\"SubscribedPlanId\\\":\\\"630b8d82-59e4-446a-9abe-48485d643257\\\",\\\"ServiceInstance\\\":\\\"WindowsDefenderATP/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6141167Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bfc1bbd9-981b-4f71-9b82-17c35fd0e2a4\\\"},{\\\"SubscribedPlanId\\\":\\\"0a80e2cd-b1e9-477d-829b-95dd228dd66a\\\",\\\"ServiceInstance\\\":\\\"LearningAppServiceInTeams/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6141167Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b76fb638-6ba6-402a-b9f9-83d28acb3d86\\\"},{\\\"SubscribedPlanId\\\":\\\"1e9fdb53-be7c-4185-8d79-17a4c14f96ea\\\",\\\"ServiceInstance\\\":\\\"WindowsUpdateforB"},{"key":"c","value":"3"}]</t>
-  </si>
-  <si>
-    <t>3/1/2026, 5:19:54.678 AM</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"5d931786-8141-4696-963e-487cf1663b83"},{"key":"seq","value":"3"},{"key":"b","value":"usinessCloudExtensions/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6141167Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"7bf960f6-2cd9-443a-8046-5dbff9558365\\\"},{\\\"SubscribedPlanId\\\":\\\"021ef71f-ddbf-4cfb-92fc-cc2c079d8025\\\",\\\"ServiceInstance\\\":\\\"MicrosoftPrint/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6141167Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"795f6fe0-cc4d-4773-b050-5dde4dc704c9\\\"},{\\\"SubscribedPlanId\\\":\\\"79a085f9-a0a5-47f8-87f4-aac406fd96e5\\\",\\\"ServiceInstance\\\":\\\"ccibotsprod/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6141167Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"ded3d325-1bdc-453e-8432-5bac26d7a014\\\"},{\\\"SubscribedPlanId\\\":\\\"7ff00ebf-2122-4a90-a21b-2dd8d91f47d0\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6151178Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"afa73018-811e-46e9-988f-f75d2b1b8430\\\"},{\\\"SubscribedPlanId\\\":\\\"a60c7542-c074-4479-af90-4af6caea7a57\\\",\\\"ServiceInstance\\\":\\\"ProjectProgramsAndPortfolios/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6151178Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b21a6b06-1988-436e-a07b-51ec6d9f52ad\\\"},{\\\"SubscribedPlanId\\\":\\\"3fe538b9-ba8a-451d-a33d-531f60dc7176\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6151178Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"28b0fa46-c39a-4188-89e2-58e979a6b014\\\"},{\\\"SubscribedPlanId\\\":\\\"161014a9-b8bc-4869-85e0-38e0137851e1\\\",\\\"ServiceInstance\\\":\\\"MicrosoftKaizala/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6151178Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"54fc630f-5a40-48ee-8965-af0503c1386e\\\"},{\\\"SubscribedPlanId\\\":\\\"0ab4aba1-516c-4f2e-ab1d-4d251481d78b\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6151178Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"276d6e8a-f056-4f70-b7e8-4fc27f79f809\\\"},{\\\"SubscribedPlanId\\\":\\\"108288ea-660d-4d4e-98ac-a651b4f33745\\\",\\\"ServiceInstance\\\":\\\"DynamicsNAV/OCN\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6151178Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"39b5c996-467e-4e60-bd62-46066f572726\\\"},{\\\"SubscribedPlanId\\\":\\\"4352e4d1-8707-4b5f-bede-d27d1ba5ae13\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6151178Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9bec7e34-c9fa-40b7-a9d1-bd6d1165c7ed\\\"},{\\\"SubscribedPlanId\\\":\\\"eeed2477-7994-4b39-a03f-181c64c7f7fa\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6151178Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bea4c11e-220a-4e6d-8eb8-8ea15d019f90\\\"},{\\\"SubscribedPlanId\\\":\\\"f6ef49c3-1a30-4a87-81bb-33eee7bba192\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6151178Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"6c57d4b6-3b23-47a5-9bc9-69f17b4947b3\\\"},{\\\"SubscribedPlanId\\\":\\\"33797a9f-7ebf-4160-b3dd-01b418e7fad8\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6151178Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"176a09a6-7ec5-4039-ac02-b2791c6ba793\\\"},{\\\"SubscribedPlanId\\\":\\\"29ff02e7-b9a1-4c7c-84a8-50aed2f7760d\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6161179Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"199a5c09-e0ca-4e37-8f7c-b05d533e1ea2\\\"},{\\\"SubscribedPlanId\\\":\\\"eaf152c0-4eeb-4f3c-8501-39ae7fe6989e\\\",\\\"ServiceInstance\\\":\\\"SCO/PROD_AMSUD0101_01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6161179Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c1ec4a95-1f05-45b3-a911-aa3fa01094f5\\\"},{\\\"SubscribedPlanId\\\":\\\"7ed1f528-4e3a-4770-bbd1-fc1e8c5ed421\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6161179Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"094e7854-93fc-4d55-b2c0-3ab5369ebdc1\\\"},{\\\"SubscribedPlanId\\\":\\\"a09cb9c4-8e21-4801-8aa3-a841705b1497\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6161179Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5bfe124c-bbdc-4494-8835-f1297d457d79\\\"},{\\\"SubscribedPlanId\\\":\\\"6bd8d315-6527-4b5e-af48-a682cf93421a\\\",\\\"ServiceInstance\\\":\\\"MicrosoftCommunicationsOnline/APAC-AU1-S1\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6161179Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0feaeb32-d00e-4d66-bd5a-43b5b83db82c\\\"},{\\\"SubscribedPlanId\\\":\\\"7c3a406a-7181-4717-a008-00e2b758651b\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6161179Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"de377cbc-0019-4ec2-b77c-3f223947e102\\\"},{\\\"SubscribedPlanId\\\":\\\"7aedce94-4e81-4a47-94fc-a18af8012419\\\",\\\"ServiceInstance\\\":\\\"SCO/PROD_AMSUD0101_01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6161179Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8e9ff0ff-aa7a-4b20-83c1-2f636b600ac2\\\"},{\\\"SubscribedPlanId\\\":\\\"dbae48d1-a0ef-497b-b857-608ffb8a0035\\\",\\\"ServiceInstance\\\":\\\"Windows/SDF\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6161179Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8e229017-d77b-43d5-9305-903395523b99\\\"}]},{\\\"Name\\\":\\\"LicenseAssignmentDetail\\\",\\\"OldValue\\\":[{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"4b9405b0-7788-4568-add1-99614e613b69\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-02-02T20:21:00.6859872Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"84a661c4-e949-4bd2-a560-ed7766fcaf2b\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-02-02T20:21:00.6859872Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"e0dfc8b9-9531-4ec8-94b4-9fec23b05fc8\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-02-02T20:21:00.6859872Z\\\",\\\"DisabledPlans\\\":[\\\"9aaf7827-d63c-4b61-89c3-182f06f82e5c\\\"],\\\"EncodingVersion\\\":2}],\\\"NewValue\\\":[{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"e0dfc8b9-9531-4ec8-94b4-9fec23b05fc8\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:19:54.5991182Z\\\",\\\"DisabledPlans\\\":[\\\"9aaf7827-d63c-4b61-89c3-182f06f82e5c\\\"],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"84a661c4-e949-4bd2-a560-ed7766fcaf2b\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:19:54.5991182Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"4b9405b0-7788-4568-add1-99614e613b69\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:19:54.5991182Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"cbdc14ab-d96c-4c30-b9f4-6ada7cdc1d46\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:19:54.5991182Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2}]},{\\\"Name\\\":\\\"Included Updated Properties\\\",\\\"OldValue\\\":null,\\\"NewValue\\\":\\\"AssignedLicense, AssignedPlan, LicenseAssignmentDetail\\\"},{\\\"Name\\\":\\\"TargetId.UserType\\\",\\\"OldValue\\\":null,\\\"NewValue\\\":\\\"Member\\\"}]\",\"additionalTargets\":\"\",\"additionalDetails\":\"{\\\"UserType\\\":\\\"Member\\\",\\\"User-Agent\\\":\\\"MCAPICommercialProductLicensing\\\"}\"}"},{"key":"c","value":"3"}]</t>
-  </si>
-  <si>
-    <t>3/1/2026, 5:19:54.681 AM</t>
-  </si>
-  <si>
-    <t>Change user license</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"ee1d45a3-54c6-49b4-83a8-4820cddc043f"},{"key":"seq","value":"1"},{"key":"b","value":"{\"targetUpdatedProperties\":\"[{\\\"Name\\\":\\\"AssignedLicense\\\",\\\"OldValue\\\":[\\\"[SkuName=EXCHANGESTANDARD, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=4b9405b0-7788-4568-add1-99614e613b69, DisabledPlans=[]]\\\",\\\"[SkuName=AAD_PREMIUM_P2, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=84a661c4-e949-4bd2-a560-ed7766fcaf2b, DisabledPlans=[]]\\\",\\\"[SkuName=Microsoft_Teams_Exploratory_Dept, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=e0dfc8b9-9531-4ec8-94b4-9fec23b05fc8, DisabledPlans=[EXCHANGE_S_STANDARD]]\\\"],\\\"NewValue\\\":[\\\"[SkuName=Microsoft_Teams_Exploratory_Dept, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=e0dfc8b9-9531-4ec8-94b4-9fec23b05fc8, DisabledPlans=[EXCHANGE_S_STANDARD]]\\\",\\\"[SkuName=AAD_PREMIUM_P2, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=84a661c4-e949-4bd2-a560-ed7766fcaf2b, DisabledPlans=[]]\\\",\\\"[SkuName=EXCHANGESTANDARD, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=4b9405b0-7788-4568-add1-99614e613b69, DisabledPlans=[]]\\\",\\\"[SkuName=SPB, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=cbdc14ab-d96c-4c30-b9f4-6ada7cdc1d46, DisabledPlans=[]]\\\"]},{\\\"Name\\\":\\\"AssignedPlan\\\",\\\"OldValue\\\":[{\\\"SubscribedPlanId\\\":\\\"0dfd484c-cc3b-4cd7-be8e-e51c1b4bc0ea\\\",\\\"ServiceInstance\\\":\\\"Sway/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a23b959c-7ce8-4e57-9140-b90eb88a9e97\\\"},{\\\"SubscribedPlanId\\\":\\\"0e6e1ecc-f9bf-4414-9e6f-1828660fd975\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"40b010bb-0b69-4654-ac5e-ba161433f4b4\\\"},{\\\"SubscribedPlanId\\\":\\\"11013c80-c192-4862-bbb5-7b86a741c83a\\\",\\\"ServiceInstance\\\":\\\"WhiteboardServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b8afc642-032e-4de5-8c0a-507a7bba7e5d\\\"},{\\\"SubscribedPlanId\\\":\\\"11b27917-6674-453b-9913-cba7aba6883a\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"dcf9d2f4-772e-4434-b757-77a453cfbc02\\\"},{\\\"SubscribedPlanId\\\":\\\"177b15ab-51b1-47d1-b213-f0e968822a83\\\",\\\"ServiceInstance\\\":\\\"MultiFactorService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8a256a2b-b617-496d-b51b-e76466e88db0\\\"},{\\\"SubscribedPlanId\\\":\\\"1a6d321c-ebe3-4198-8527-0d14340c3009\\\",\\\"ServiceInstance\\\":\\\"ProcessSimple/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0f9b09cb-62d1-4ff4-9129-43f4996f83f4\\\"},{\\\"SubscribedPlanId\\\":\\\"1b044c1d-0c69-4b8d-8b93-03c2ef1fd3da\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c7699d2e-19aa-44de-8edf-1736da088ca1\\\"},{\\\"SubscribedPlanId\\\":\\\"2287b27a-b6ec-40e6-bb03-35170aa2c846\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"41781fb2-bc02-4b7c-bd55-b576c07bb09d\\\"},{\\\"SubscribedPlanId\\\":\\\"3ef79a81-ae21-49b8-8fa7-dc1d795d9671\\\",\\\"ServiceInstance\\\":\\\"ProjectProgramsAndPortfolios/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a55dfd10-0864-46d9-a3cd-da5991a3e0e2\\\"},{\\\"SubscribedPlanId\\\":\\\"449a3874-a6a4-498d-905d-662cfc611bea\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"f0ff6ac6-297d-49cd-be34-6dfef97f0c28\\\"},{\\\"SubscribedPlanId\\\":\\\"529909ed-7627-4843-bb53-3556b852c9d9\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T20:21:00Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9aaf7827-d63c-4b61-89c3-182f06f82e5c\\\"},{\\\"SubscribedPlanId\\\":\\\"53ac6e25-a8f6-44bf-b402-9f56b8eecfd9\\\",\\\"ServiceInstance\\\":\\\"To-Do/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5e62787c-c316-451f-b873-1d05acd4d12c\\\"},{\\\"SubscribedPlanId\\\":\\\"6f907b14-cb0b-4a3a-9bb9-4f951739e103\\\",\\\"ServiceInstance\\\":\\\"Deskless/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8c7d2df8-86f0-4902-b2ed-a0458298f3b3\\\"},{\\\"SubscribedPlanId\\\":\\\"71ac5b1a-e1dc-4ced-ba2d-059d74e89acf\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"3efbd4ed-8958-4824-8389-1321f8730af8\\\"},{\\\"SubscribedPlanId\\\":\\\"85ff92c3-df66-4ccc-ba0b-38683b60b371\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"33c4f319-9bdd-48d6-9c4d-410b750a4a5a\\\"},{\\\"SubscribedPlanId\\\":\\\"88ae6c56-fccc-497d-9e45-c0ea113b9406\\\",\\\"ServiceInstance\\\":\\\"PowerAppsService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"92f7a6f3-b89b-4bbd-8c30-809e6da5ad1c\\\"},{\\\"SubscribedPlanId\\\":\\\"956ea907-9a03-46cd-8699-95667e82355a\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c63d4d19-e8cb-460e-b37c-4d6c34603745\\\"},{\\\"SubscribedPlanId\\\":\\\"a22189d7-70fa-482b-9d57-ada39f5e0872\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"eec0eb4f-6444-4f95-aba0-50c24d67f998\\\"},{\\\"SubscribedPlanId\\\":\\\"a5d43ea2-3323-489d-a579-068f683b41f7\\\",\\\"ServiceInstance\\\":\\\"ccibotsprod/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0683001c-0492-4d59-9515-d9a6426b5813\\\"},{\\\"SubscribedPlanId\\\":\\\"a83d2db3-81e2-45ee-bf0e-c1088b24bb96\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"e95bec33-7c88-4a70-8e19-b10bd9d0c014\\\"},{\\\"SubscribedPlanId\\\":\\\"b3ae2021-9f74-4a09-9845-42accad7b182\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bed136c6-b799-4462-824d-fc045d3a9d25\\\"},{\\\"SubscribedPlanId\\\":\\\"b7b9220c-a3f0-437e-b99a-0e925b312c86\\\",\\\"ServiceInstance\\\":\\\"YammerEnterprise/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"7547a3fe-08ee-4ccb-b430-5077c5041653\\\"},{\\\"SubscribedPlanId\\\":\\\"c73a8c4e-f6b6-4998-bf41-862fdea05abd\\\",\\\"ServiceInstance\\\":\\\"ProjectWorkManagement/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b737dad2-2f6c-4c65-90e3-ca563267e8b9\\\"},{\\\"SubscribedPlanId\\\":\\\"d1c57312-4814-4818-a991-38bb7429b211\\\",\\\"ServiceInstance\\\":\\\"TeamspaceAPI/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"57ff2da0-773e-42df-b2af-ffb7a2317929\\\"},{\\\"SubscribedPlanId\\\":\\\"dddc5824-34a0-4b85-b6b8-0fafe67a57b0\\\",\\\"ServiceInstance\\\":\\\"OfficeForms/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"159f4cd6-e380-449f-a816-af1a9ef76344\\\"},{\\\"SubscribedPlanId\\\":\\\"e039cc95-628d-4ade-80ce-f77a46135dde\\\",\\\"ServiceInstance\\\":\\\"MicrosoftStream/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"743dd19e-1ce3-4c62-a3ad-49ba8f63a2f6\\\"},{\\\"SubscribedPlanId\\\":\\\"e7733084-cf3d-4d56-9cfd-1cd9ea183052\\\",\\\"ServiceInstance\\\":\\\"Adallom/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"932ad362-64a8-4783-9106-97849a1a30b9\\\"},{\\\"SubscribedPlanId\\\":\\\"ea16e50b-9303-4b92-9e45-0c4c4f2482be\\\",\\\"ServiceInstance\\\":\\\"MicrosoftCommunicationsOnline/APAC-AU1-S1\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"42a3ec34-28ba-46b6-992f-db53a675ac5b\\\"}],\\\"NewValue\\\":[{\\\"SubscribedPlanId\\\":\\\"529909ed-7627-4843-bb53-3556b852c9d9\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6131188Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9aaf7827-d63c-4b61-89c3-182f06f82e5c\\\"},{\\\"SubscribedPlanId\\\":\\\"ea16e50b-9303-4b92-9e45-0c4c4f2482be\\\",\\\"ServiceInstance\\\":\\\"MicrosoftCommunicationsOnline/APAC-AU1-S1\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"42a3ec34-28ba-46b6-992f-db53a675ac5b\\\"},{\\\"SubscribedPlanId\\\":\\\"e039cc95-628d-4ade-80ce-f77a46135dde\\\",\\\"ServiceInstance\\\":\\\"MicrosoftStream/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"743dd19e-1ce3-4c62-a3ad-49ba8f63a2f6\\\"},{\\\"SubscribedPlanId\\\":\\\"dddc5824-34a0"},{"key":"c","value":"3"}]</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"ee1d45a3-54c6-49b4-83a8-4820cddc043f"},{"key":"seq","value":"2"},{"key":"b","value":"-4b85-b6b8-0fafe67a57b0\\\",\\\"ServiceInstance\\\":\\\"OfficeForms/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"159f4cd6-e380-449f-a816-af1a9ef76344\\\"},{\\\"SubscribedPlanId\\\":\\\"d1c57312-4814-4818-a991-38bb7429b211\\\",\\\"ServiceInstance\\\":\\\"TeamspaceAPI/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"57ff2da0-773e-42df-b2af-ffb7a2317929\\\"},{\\\"SubscribedPlanId\\\":\\\"c73a8c4e-f6b6-4998-bf41-862fdea05abd\\\",\\\"ServiceInstance\\\":\\\"ProjectWorkManagement/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b737dad2-2f6c-4c65-90e3-ca563267e8b9\\\"},{\\\"SubscribedPlanId\\\":\\\"b7b9220c-a3f0-437e-b99a-0e925b312c86\\\",\\\"ServiceInstance\\\":\\\"YammerEnterprise/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"7547a3fe-08ee-4ccb-b430-5077c5041653\\\"},{\\\"SubscribedPlanId\\\":\\\"b3ae2021-9f74-4a09-9845-42accad7b182\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bed136c6-b799-4462-824d-fc045d3a9d25\\\"},{\\\"SubscribedPlanId\\\":\\\"a83d2db3-81e2-45ee-bf0e-c1088b24bb96\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"e95bec33-7c88-4a70-8e19-b10bd9d0c014\\\"},{\\\"SubscribedPlanId\\\":\\\"a5d43ea2-3323-489d-a579-068f683b41f7\\\",\\\"ServiceInstance\\\":\\\"ccibotsprod/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0683001c-0492-4d59-9515-d9a6426b5813\\\"},{\\\"SubscribedPlanId\\\":\\\"956ea907-9a03-46cd-8699-95667e82355a\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c63d4d19-e8cb-460e-b37c-4d6c34603745\\\"},{\\\"SubscribedPlanId\\\":\\\"88ae6c56-fccc-497d-9e45-c0ea113b9406\\\",\\\"ServiceInstance\\\":\\\"PowerAppsService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"92f7a6f3-b89b-4bbd-8c30-809e6da5ad1c\\\"},{\\\"SubscribedPlanId\\\":\\\"85ff92c3-df66-4ccc-ba0b-38683b60b371\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"33c4f319-9bdd-48d6-9c4d-410b750a4a5a\\\"},{\\\"SubscribedPlanId\\\":\\\"71ac5b1a-e1dc-4ced-ba2d-059d74e89acf\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"3efbd4ed-8958-4824-8389-1321f8730af8\\\"},{\\\"SubscribedPlanId\\\":\\\"6f907b14-cb0b-4a3a-9bb9-4f951739e103\\\",\\\"ServiceInstance\\\":\\\"Deskless/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8c7d2df8-86f0-4902-b2ed-a0458298f3b3\\\"},{\\\"SubscribedPlanId\\\":\\\"53ac6e25-a8f6-44bf-b402-9f56b8eecfd9\\\",\\\"ServiceInstance\\\":\\\"To-Do/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5e62787c-c316-451f-b873-1d05acd4d12c\\\"},{\\\"SubscribedPlanId\\\":\\\"449a3874-a6a4-498d-905d-662cfc611bea\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"f0ff6ac6-297d-49cd-be34-6dfef97f0c28\\\"},{\\\"SubscribedPlanId\\\":\\\"3ef79a81-ae21-49b8-8fa7-dc1d795d9671\\\",\\\"ServiceInstance\\\":\\\"ProjectProgramsAndPortfolios/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a55dfd10-0864-46d9-a3cd-da5991a3e0e2\\\"},{\\\"SubscribedPlanId\\\":\\\"1b044c1d-0c69-4b8d-8b93-03c2ef1fd3da\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c7699d2e-19aa-44de-8edf-1736da088ca1\\\"},{\\\"SubscribedPlanId\\\":\\\"1a6d321c-ebe3-4198-8527-0d14340c3009\\\",\\\"ServiceInstance\\\":\\\"ProcessSimple/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0f9b09cb-62d1-4ff4-9129-43f4996f83f4\\\"},{\\\"SubscribedPlanId\\\":\\\"11b27917-6674-453b-9913-cba7aba6883a\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"dcf9d2f4-772e-4434-b757-77a453cfbc02\\\"},{\\\"SubscribedPlanId\\\":\\\"11013c80-c192-4862-bbb5-7b86a741c83a\\\",\\\"ServiceInstance\\\":\\\"WhiteboardServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b8afc642-032e-4de5-8c0a-507a7bba7e5d\\\"},{\\\"SubscribedPlanId\\\":\\\"0e6e1ecc-f9bf-4414-9e6f-1828660fd975\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"40b010bb-0b69-4654-ac5e-ba161433f4b4\\\"},{\\\"SubscribedPlanId\\\":\\\"0dfd484c-cc3b-4cd7-be8e-e51c1b4bc0ea\\\",\\\"ServiceInstance\\\":\\\"Sway/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a23b959c-7ce8-4e57-9140-b90eb88a9e97\\\"},{\\\"SubscribedPlanId\\\":\\\"e7733084-cf3d-4d56-9cfd-1cd9ea183052\\\",\\\"ServiceInstance\\\":\\\"Adallom/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"932ad362-64a8-4783-9106-97849a1a30b9\\\"},{\\\"SubscribedPlanId\\\":\\\"a22189d7-70fa-482b-9d57-ada39f5e0872\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"eec0eb4f-6444-4f95-aba0-50c24d67f998\\\"},{\\\"SubscribedPlanId\\\":\\\"2287b27a-b6ec-40e6-bb03-35170aa2c846\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"41781fb2-bc02-4b7c-bd55-b576c07bb09d\\\"},{\\\"SubscribedPlanId\\\":\\\"177b15ab-51b1-47d1-b213-f0e968822a83\\\",\\\"ServiceInstance\\\":\\\"MultiFactorService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8a256a2b-b617-496d-b51b-e76466e88db0\\\"},{\\\"SubscribedPlanId\\\":\\\"020805e7-7d5f-4bb3-b898-a3b1259a976f\\\",\\\"ServiceInstance\\\":\\\"VivaSkills/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6131188Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"13b6da2c-0d84-450e-9f69-a33e221387ca\\\"},{\\\"SubscribedPlanId\\\":\\\"694b4e1c-079c-4afe-9d08-f38537955130\\\",\\\"ServiceInstance\\\":\\\"OnlineService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6131188Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"1fe6227d-3e01-46d0-9510-0acad4ff6e94\\\"},{\\\"SubscribedPlanId\\\":\\\"f16c6e89-93cc-4fd6-b474-59b2cea0231b\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6141167Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a6520331-d7d4-4276-95f5-15c0933bc757\\\"},{\\\"SubscribedPlanId\\\":\\\"b7f56b27-f5ea-45fb-8884-1a5357c41c37\\\",\\\"ServiceInstance\\\":\\\"Microsoft.ProjectBabylon/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6141167Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c948ea65-2053-4a5a-8a62-9eaaaf11b522\\\"},{\\\"SubscribedPlanId\\\":\\\"22b5463b-d360-473f-80c2-be8e42afcc71\\\",\\\"ServiceInstance\\\":\\\"Chapter5FluidApp/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6141167Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c4b8c31a-fb44-4c65-9837-a21f55fcabda\\\"},{\\\"SubscribedPlanId\\\":\\\"c4031b28-43f8-42d9-b1f4-06f5b955074c\\\",\\\"ServiceInstance\\\":\\\"Bing/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6141167Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0d0c0d31-fae7-41f2-b909-eaf4d7f26dba\\\"},{\\\"SubscribedPlanId\\\":\\\"36e41faa-1e78-4c8b-8453-6b3ca38ab4c1\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6141167Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a1ace008-72f3-4ea0-8dac-33b3a23a2472\\\"},{\\\"SubscribedPlanId\\\":\\\"02e3d1d6-4434-4d5c-88b7-a35a509cce87\\\",\\\"ServiceInstance\\\":\\\"YammerEnterprise/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6141167Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a82fbf69-b4d7-49f4-83a6-915b2cf354f4\\\"},{\\\"SubscribedPlanId\\\":\\\"630b8d82-59e4-446a-9abe-48485d643257\\\",\\\"ServiceInstance\\\":\\\"WindowsDefenderATP/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6141167Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bfc1bbd9-981b-4f71-9b82-17c35fd0e2a4\\\"},{\\\"SubscribedPlanId\\\":\\\"0a80e2cd-b1e9-477d-829b-95dd228dd66a\\\",\\\"ServiceInstance\\\":\\\"LearningAppServiceInTeams/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6141167Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b76fb638-6ba6-402a-b9f9-83d28acb3d86\\\"},{\\\"SubscribedPlanId\\\":\\\"1e9fdb53-be7c-4185-8d79-17a4c14f96ea\\\",\\\"ServiceInstance\\\":\\\"WindowsUpdateforB"},{"key":"c","value":"3"}]</t>
-  </si>
-  <si>
-    <t>3/1/2026, 5:19:54.682 AM</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"ee1d45a3-54c6-49b4-83a8-4820cddc043f"},{"key":"seq","value":"3"},{"key":"b","value":"usinessCloudExtensions/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6141167Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"7bf960f6-2cd9-443a-8046-5dbff9558365\\\"},{\\\"SubscribedPlanId\\\":\\\"021ef71f-ddbf-4cfb-92fc-cc2c079d8025\\\",\\\"ServiceInstance\\\":\\\"MicrosoftPrint/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6141167Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"795f6fe0-cc4d-4773-b050-5dde4dc704c9\\\"},{\\\"SubscribedPlanId\\\":\\\"79a085f9-a0a5-47f8-87f4-aac406fd96e5\\\",\\\"ServiceInstance\\\":\\\"ccibotsprod/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6141167Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"ded3d325-1bdc-453e-8432-5bac26d7a014\\\"},{\\\"SubscribedPlanId\\\":\\\"7ff00ebf-2122-4a90-a21b-2dd8d91f47d0\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6151178Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"afa73018-811e-46e9-988f-f75d2b1b8430\\\"},{\\\"SubscribedPlanId\\\":\\\"a60c7542-c074-4479-af90-4af6caea7a57\\\",\\\"ServiceInstance\\\":\\\"ProjectProgramsAndPortfolios/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6151178Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b21a6b06-1988-436e-a07b-51ec6d9f52ad\\\"},{\\\"SubscribedPlanId\\\":\\\"3fe538b9-ba8a-451d-a33d-531f60dc7176\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6151178Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"28b0fa46-c39a-4188-89e2-58e979a6b014\\\"},{\\\"SubscribedPlanId\\\":\\\"161014a9-b8bc-4869-85e0-38e0137851e1\\\",\\\"ServiceInstance\\\":\\\"MicrosoftKaizala/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6151178Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"54fc630f-5a40-48ee-8965-af0503c1386e\\\"},{\\\"SubscribedPlanId\\\":\\\"0ab4aba1-516c-4f2e-ab1d-4d251481d78b\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6151178Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"276d6e8a-f056-4f70-b7e8-4fc27f79f809\\\"},{\\\"SubscribedPlanId\\\":\\\"108288ea-660d-4d4e-98ac-a651b4f33745\\\",\\\"ServiceInstance\\\":\\\"DynamicsNAV/OCN\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6151178Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"39b5c996-467e-4e60-bd62-46066f572726\\\"},{\\\"SubscribedPlanId\\\":\\\"4352e4d1-8707-4b5f-bede-d27d1ba5ae13\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6151178Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9bec7e34-c9fa-40b7-a9d1-bd6d1165c7ed\\\"},{\\\"SubscribedPlanId\\\":\\\"eeed2477-7994-4b39-a03f-181c64c7f7fa\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6151178Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bea4c11e-220a-4e6d-8eb8-8ea15d019f90\\\"},{\\\"SubscribedPlanId\\\":\\\"f6ef49c3-1a30-4a87-81bb-33eee7bba192\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6151178Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"6c57d4b6-3b23-47a5-9bc9-69f17b4947b3\\\"},{\\\"SubscribedPlanId\\\":\\\"33797a9f-7ebf-4160-b3dd-01b418e7fad8\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6151178Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"176a09a6-7ec5-4039-ac02-b2791c6ba793\\\"},{\\\"SubscribedPlanId\\\":\\\"29ff02e7-b9a1-4c7c-84a8-50aed2f7760d\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6161179Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"199a5c09-e0ca-4e37-8f7c-b05d533e1ea2\\\"},{\\\"SubscribedPlanId\\\":\\\"eaf152c0-4eeb-4f3c-8501-39ae7fe6989e\\\",\\\"ServiceInstance\\\":\\\"SCO/PROD_AMSUD0101_01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6161179Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c1ec4a95-1f05-45b3-a911-aa3fa01094f5\\\"},{\\\"SubscribedPlanId\\\":\\\"7ed1f528-4e3a-4770-bbd1-fc1e8c5ed421\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6161179Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"094e7854-93fc-4d55-b2c0-3ab5369ebdc1\\\"},{\\\"SubscribedPlanId\\\":\\\"a09cb9c4-8e21-4801-8aa3-a841705b1497\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6161179Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5bfe124c-bbdc-4494-8835-f1297d457d79\\\"},{\\\"SubscribedPlanId\\\":\\\"6bd8d315-6527-4b5e-af48-a682cf93421a\\\",\\\"ServiceInstance\\\":\\\"MicrosoftCommunicationsOnline/APAC-AU1-S1\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6161179Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0feaeb32-d00e-4d66-bd5a-43b5b83db82c\\\"},{\\\"SubscribedPlanId\\\":\\\"7c3a406a-7181-4717-a008-00e2b758651b\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6161179Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"de377cbc-0019-4ec2-b77c-3f223947e102\\\"},{\\\"SubscribedPlanId\\\":\\\"7aedce94-4e81-4a47-94fc-a18af8012419\\\",\\\"ServiceInstance\\\":\\\"SCO/PROD_AMSUD0101_01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6161179Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8e9ff0ff-aa7a-4b20-83c1-2f636b600ac2\\\"},{\\\"SubscribedPlanId\\\":\\\"dbae48d1-a0ef-497b-b857-608ffb8a0035\\\",\\\"ServiceInstance\\\":\\\"Windows/SDF\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54.6161179Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8e229017-d77b-43d5-9305-903395523b99\\\"}]},{\\\"Name\\\":\\\"LicenseAssignmentDetail\\\",\\\"OldValue\\\":[{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"4b9405b0-7788-4568-add1-99614e613b69\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-02-02T20:21:00.6859872Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"84a661c4-e949-4bd2-a560-ed7766fcaf2b\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-02-02T20:21:00.6859872Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"e0dfc8b9-9531-4ec8-94b4-9fec23b05fc8\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-02-02T20:21:00.6859872Z\\\",\\\"DisabledPlans\\\":[\\\"9aaf7827-d63c-4b61-89c3-182f06f82e5c\\\"],\\\"EncodingVersion\\\":2}],\\\"NewValue\\\":[{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"e0dfc8b9-9531-4ec8-94b4-9fec23b05fc8\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:19:54.5991182Z\\\",\\\"DisabledPlans\\\":[\\\"9aaf7827-d63c-4b61-89c3-182f06f82e5c\\\"],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"84a661c4-e949-4bd2-a560-ed7766fcaf2b\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:19:54.5991182Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"4b9405b0-7788-4568-add1-99614e613b69\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:19:54.5991182Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"cbdc14ab-d96c-4c30-b9f4-6ada7cdc1d46\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:19:54.5991182Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2}]},{\\\"Name\\\":\\\"Included Updated Properties\\\",\\\"OldValue\\\":null,\\\"NewValue\\\":\\\"AssignedLicense, AssignedPlan, LicenseAssignmentDetail\\\"},{\\\"Name\\\":\\\"TargetId.UserType\\\",\\\"OldValue\\\":null,\\\"NewValue\\\":\\\"Member\\\"}]\",\"additionalTargets\":\"{\\\"AssignedSkuId\\\":[\\\"e0dfc8b9-9531-4ec8-94b4-9fec23b05fc8\\\",\\\"84a661c4-e949-4bd2-a560-ed7766fcaf2b\\\",\\\"4b9405b0-7788-4568-add1-99614e613b69\\\",\\\"cbdc14ab-d96c-4c30-b9f4-6ada7cdc1d46\\\"]}\",\"additionalDetails\":\"{\\\"User-Agent\\\":\\\"MCAPICommercialProductLicensing\\\"}\"}"},{"key":"c","value":"3"}]</t>
-  </si>
-  <si>
-    <t>3/1/2026, 5:24:48.523 AM</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"703e087d-3728-4730-a45d-131327b86066"},{"key":"seq","value":"2"},{"key":"b","value":"ba2d-059d74e89acf\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"3efbd4ed-8958-4824-8389-1321f8730af8\\\"},{\\\"SubscribedPlanId\\\":\\\"79a085f9-a0a5-47f8-87f4-aac406fd96e5\\\",\\\"ServiceInstance\\\":\\\"ccibotsprod/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"ded3d325-1bdc-453e-8432-5bac26d7a014\\\"},{\\\"SubscribedPlanId\\\":\\\"7aedce94-4e81-4a47-94fc-a18af8012419\\\",\\\"ServiceInstance\\\":\\\"SCO/PROD_AMSUD0101_01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8e9ff0ff-aa7a-4b20-83c1-2f636b600ac2\\\"},{\\\"SubscribedPlanId\\\":\\\"7c3a406a-7181-4717-a008-00e2b758651b\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"de377cbc-0019-4ec2-b77c-3f223947e102\\\"},{\\\"SubscribedPlanId\\\":\\\"7ed1f528-4e3a-4770-bbd1-fc1e8c5ed421\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"094e7854-93fc-4d55-b2c0-3ab5369ebdc1\\\"},{\\\"SubscribedPlanId\\\":\\\"7ff00ebf-2122-4a90-a21b-2dd8d91f47d0\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"afa73018-811e-46e9-988f-f75d2b1b8430\\\"},{\\\"SubscribedPlanId\\\":\\\"85ff92c3-df66-4ccc-ba0b-38683b60b371\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"33c4f319-9bdd-48d6-9c4d-410b750a4a5a\\\"},{\\\"SubscribedPlanId\\\":\\\"88ae6c56-fccc-497d-9e45-c0ea113b9406\\\",\\\"ServiceInstance\\\":\\\"PowerAppsService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"92f7a6f3-b89b-4bbd-8c30-809e6da5ad1c\\\"},{\\\"SubscribedPlanId\\\":\\\"956ea907-9a03-46cd-8699-95667e82355a\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c63d4d19-e8cb-460e-b37c-4d6c34603745\\\"},{\\\"SubscribedPlanId\\\":\\\"a09cb9c4-8e21-4801-8aa3-a841705b1497\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5bfe124c-bbdc-4494-8835-f1297d457d79\\\"},{\\\"SubscribedPlanId\\\":\\\"a22189d7-70fa-482b-9d57-ada39f5e0872\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"eec0eb4f-6444-4f95-aba0-50c24d67f998\\\"},{\\\"SubscribedPlanId\\\":\\\"a5d43ea2-3323-489d-a579-068f683b41f7\\\",\\\"ServiceInstance\\\":\\\"ccibotsprod/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0683001c-0492-4d59-9515-d9a6426b5813\\\"},{\\\"SubscribedPlanId\\\":\\\"a60c7542-c074-4479-af90-4af6caea7a57\\\",\\\"ServiceInstance\\\":\\\"ProjectProgramsAndPortfolios/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b21a6b06-1988-436e-a07b-51ec6d9f52ad\\\"},{\\\"SubscribedPlanId\\\":\\\"a83d2db3-81e2-45ee-bf0e-c1088b24bb96\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"e95bec33-7c88-4a70-8e19-b10bd9d0c014\\\"},{\\\"SubscribedPlanId\\\":\\\"b3ae2021-9f74-4a09-9845-42accad7b182\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bed136c6-b799-4462-824d-fc045d3a9d25\\\"},{\\\"SubscribedPlanId\\\":\\\"b7b9220c-a3f0-437e-b99a-0e925b312c86\\\",\\\"ServiceInstance\\\":\\\"YammerEnterprise/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"7547a3fe-08ee-4ccb-b430-5077c5041653\\\"},{\\\"SubscribedPlanId\\\":\\\"b7f56b27-f5ea-45fb-8884-1a5357c41c37\\\",\\\"ServiceInstance\\\":\\\"Microsoft.ProjectBabylon/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c948ea65-2053-4a5a-8a62-9eaaaf11b522\\\"},{\\\"SubscribedPlanId\\\":\\\"c4031b28-43f8-42d9-b1f4-06f5b955074c\\\",\\\"ServiceInstance\\\":\\\"Bing/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0d0c0d31-fae7-41f2-b909-eaf4d7f26dba\\\"},{\\\"SubscribedPlanId\\\":\\\"c73a8c4e-f6b6-4998-bf41-862fdea05abd\\\",\\\"ServiceInstance\\\":\\\"ProjectWorkManagement/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b737dad2-2f6c-4c65-90e3-ca563267e8b9\\\"},{\\\"SubscribedPlanId\\\":\\\"d1c57312-4814-4818-a991-38bb7429b211\\\",\\\"ServiceInstance\\\":\\\"TeamspaceAPI/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"57ff2da0-773e-42df-b2af-ffb7a2317929\\\"},{\\\"SubscribedPlanId\\\":\\\"dbae48d1-a0ef-497b-b857-608ffb8a0035\\\",\\\"ServiceInstance\\\":\\\"Windows/SDF\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8e229017-d77b-43d5-9305-903395523b99\\\"},{\\\"SubscribedPlanId\\\":\\\"dddc5824-34a0-4b85-b6b8-0fafe67a57b0\\\",\\\"ServiceInstance\\\":\\\"OfficeForms/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"159f4cd6-e380-449f-a816-af1a9ef76344\\\"},{\\\"SubscribedPlanId\\\":\\\"e039cc95-628d-4ade-80ce-f77a46135dde\\\",\\\"ServiceInstance\\\":\\\"MicrosoftStream/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"743dd19e-1ce3-4c62-a3ad-49ba8f63a2f6\\\"},{\\\"SubscribedPlanId\\\":\\\"e7733084-cf3d-4d56-9cfd-1cd9ea183052\\\",\\\"ServiceInstance\\\":\\\"Adallom/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"932ad362-64a8-4783-9106-97849a1a30b9\\\"},{\\\"SubscribedPlanId\\\":\\\"ea16e50b-9303-4b92-9e45-0c4c4f2482be\\\",\\\"ServiceInstance\\\":\\\"MicrosoftCommunicationsOnline/APAC-AU1-S1\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"42a3ec34-28ba-46b6-992f-db53a675ac5b\\\"},{\\\"SubscribedPlanId\\\":\\\"eaf152c0-4eeb-4f3c-8501-39ae7fe6989e\\\",\\\"ServiceInstance\\\":\\\"SCO/PROD_AMSUD0101_01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c1ec4a95-1f05-45b3-a911-aa3fa01094f5\\\"},{\\\"SubscribedPlanId\\\":\\\"eeed2477-7994-4b39-a03f-181c64c7f7fa\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bea4c11e-220a-4e6d-8eb8-8ea15d019f90\\\"},{\\\"SubscribedPlanId\\\":\\\"f16c6e89-93cc-4fd6-b474-59b2cea0231b\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a6520331-d7d4-4276-95f5-15c0933bc757\\\"},{\\\"SubscribedPlanId\\\":\\\"f6ef49c3-1a30-4a87-81bb-33eee7bba192\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"6c57d4b6-3b23-47a5-9bc9-69f17b4947b3\\\"}],\\\"NewValue\\\":[{\\\"SubscribedPlanId\\\":\\\"f6ef49c3-1a30-4a87-81bb-33eee7bba192\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"6c57d4b6-3b23-47a5-9bc9-69f17b4947b3\\\"},{\\\"SubscribedPlanId\\\":\\\"f16c6e89-93cc-4fd6-b474-59b2cea0231b\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a6520331-d7d4-4276-95f5-15c0933bc757\\\"},{\\\"SubscribedPlanId\\\":\\\"eeed2477-7994-4b39-a03f-181c64c7f7fa\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bea4c11e-220a-4e6d-8eb8-8ea15d019f90\\\"},{\\\"SubscribedPlanId\\\":\\\"eaf152c0-4eeb-4f3c-8501-39ae7fe6989e\\\",\\\"ServiceInstance\\\":\\\"SCO/PROD_AMSUD0101_01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c1ec4a95-1f05-45b3-a911-aa3fa01094f5\\\"},{\\\"SubscribedPlanId\\\":\\\"dbae48d1-a0ef-497b-b857-608ffb8a0035\\\",\\\"ServiceInstance\\\":\\\"Windows/SDF\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8e229017-d77b-43d5-9305-903395523b99\\\"},{\\\"SubscribedPlanId\\\":\\\"c4031b28-43f8-42d9-b1f4-06f5b955074c\\\",\\\"ServiceInstance\\\":\\\"Bing/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0d0c0d31-fae7-41f2-b909-eaf4d7f26dba\\\"},{\\\"SubscribedPlanId\\\":\\\"b7f56b27-f5ea-45fb-8884-1a5357c41c37\\\",\\\"ServiceInstance\\\":\\\"Microsoft.ProjectBabylon/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\""},{"key":"c","value":"5"}]</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"703e087d-3728-4730-a45d-131327b86066"},{"key":"seq","value":"3"},{"key":"b","value":"ServicePlanId\\\":\\\"c948ea65-2053-4a5a-8a62-9eaaaf11b522\\\"},{\\\"SubscribedPlanId\\\":\\\"a60c7542-c074-4479-af90-4af6caea7a57\\\",\\\"ServiceInstance\\\":\\\"ProjectProgramsAndPortfolios/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b21a6b06-1988-436e-a07b-51ec6d9f52ad\\\"},{\\\"SubscribedPlanId\\\":\\\"a09cb9c4-8e21-4801-8aa3-a841705b1497\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5bfe124c-bbdc-4494-8835-f1297d457d79\\\"},{\\\"SubscribedPlanId\\\":\\\"7ff00ebf-2122-4a90-a21b-2dd8d91f47d0\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"afa73018-811e-46e9-988f-f75d2b1b8430\\\"},{\\\"SubscribedPlanId\\\":\\\"7ed1f528-4e3a-4770-bbd1-fc1e8c5ed421\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"094e7854-93fc-4d55-b2c0-3ab5369ebdc1\\\"},{\\\"SubscribedPlanId\\\":\\\"7c3a406a-7181-4717-a008-00e2b758651b\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"de377cbc-0019-4ec2-b77c-3f223947e102\\\"},{\\\"SubscribedPlanId\\\":\\\"7aedce94-4e81-4a47-94fc-a18af8012419\\\",\\\"ServiceInstance\\\":\\\"SCO/PROD_AMSUD0101_01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8e9ff0ff-aa7a-4b20-83c1-2f636b600ac2\\\"},{\\\"SubscribedPlanId\\\":\\\"79a085f9-a0a5-47f8-87f4-aac406fd96e5\\\",\\\"ServiceInstance\\\":\\\"ccibotsprod/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"ded3d325-1bdc-453e-8432-5bac26d7a014\\\"},{\\\"SubscribedPlanId\\\":\\\"6bd8d315-6527-4b5e-af48-a682cf93421a\\\",\\\"ServiceInstance\\\":\\\"MicrosoftCommunicationsOnline/APAC-AU1-S1\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0feaeb32-d00e-4d66-bd5a-43b5b83db82c\\\"},{\\\"SubscribedPlanId\\\":\\\"694b4e1c-079c-4afe-9d08-f38537955130\\\",\\\"ServiceInstance\\\":\\\"OnlineService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"1fe6227d-3e01-46d0-9510-0acad4ff6e94\\\"},{\\\"SubscribedPlanId\\\":\\\"630b8d82-59e4-446a-9abe-48485d643257\\\",\\\"ServiceInstance\\\":\\\"WindowsDefenderATP/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bfc1bbd9-981b-4f71-9b82-17c35fd0e2a4\\\"},{\\\"SubscribedPlanId\\\":\\\"529909ed-7627-4843-bb53-3556b852c9d9\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.425751Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9aaf7827-d63c-4b61-89c3-182f06f82e5c\\\"},{\\\"SubscribedPlanId\\\":\\\"4352e4d1-8707-4b5f-bede-d27d1ba5ae13\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9bec7e34-c9fa-40b7-a9d1-bd6d1165c7ed\\\"},{\\\"SubscribedPlanId\\\":\\\"3fe538b9-ba8a-451d-a33d-531f60dc7176\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"28b0fa46-c39a-4188-89e2-58e979a6b014\\\"},{\\\"SubscribedPlanId\\\":\\\"36e41faa-1e78-4c8b-8453-6b3ca38ab4c1\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a1ace008-72f3-4ea0-8dac-33b3a23a2472\\\"},{\\\"SubscribedPlanId\\\":\\\"33797a9f-7ebf-4160-b3dd-01b418e7fad8\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"176a09a6-7ec5-4039-ac02-b2791c6ba793\\\"},{\\\"SubscribedPlanId\\\":\\\"29ff02e7-b9a1-4c7c-84a8-50aed2f7760d\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"199a5c09-e0ca-4e37-8f7c-b05d533e1ea2\\\"},{\\\"SubscribedPlanId\\\":\\\"22b5463b-d360-473f-80c2-be8e42afcc71\\\",\\\"ServiceInstance\\\":\\\"Chapter5FluidApp/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c4b8c31a-fb44-4c65-9837-a21f55fcabda\\\"},{\\\"SubscribedPlanId\\\":\\\"1e9fdb53-be7c-4185-8d79-17a4c14f96ea\\\",\\\"ServiceInstance\\\":\\\"WindowsUpdateforBusinessCloudExtensions/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"7bf960f6-2cd9-443a-8046-5dbff9558365\\\"},{\\\"SubscribedPlanId\\\":\\\"161014a9-b8bc-4869-85e0-38e0137851e1\\\",\\\"ServiceInstance\\\":\\\"MicrosoftKaizala/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"54fc630f-5a40-48ee-8965-af0503c1386e\\\"},{\\\"SubscribedPlanId\\\":\\\"108288ea-660d-4d4e-98ac-a651b4f33745\\\",\\\"ServiceInstance\\\":\\\"DynamicsNAV/OCN\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"39b5c996-467e-4e60-bd62-46066f572726\\\"},{\\\"SubscribedPlanId\\\":\\\"0ab4aba1-516c-4f2e-ab1d-4d251481d78b\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"276d6e8a-f056-4f70-b7e8-4fc27f79f809\\\"},{\\\"SubscribedPlanId\\\":\\\"0a80e2cd-b1e9-477d-829b-95dd228dd66a\\\",\\\"ServiceInstance\\\":\\\"LearningAppServiceInTeams/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b76fb638-6ba6-402a-b9f9-83d28acb3d86\\\"},{\\\"SubscribedPlanId\\\":\\\"02e3d1d6-4434-4d5c-88b7-a35a509cce87\\\",\\\"ServiceInstance\\\":\\\"YammerEnterprise/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a82fbf69-b4d7-49f4-83a6-915b2cf354f4\\\"},{\\\"SubscribedPlanId\\\":\\\"021ef71f-ddbf-4cfb-92fc-cc2c079d8025\\\",\\\"ServiceInstance\\\":\\\"MicrosoftPrint/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"795f6fe0-cc4d-4773-b050-5dde4dc704c9\\\"},{\\\"SubscribedPlanId\\\":\\\"020805e7-7d5f-4bb3-b898-a3b1259a976f\\\",\\\"ServiceInstance\\\":\\\"VivaSkills/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"13b6da2c-0d84-450e-9f69-a33e221387ca\\\"},{\\\"SubscribedPlanId\\\":\\\"ea16e50b-9303-4b92-9e45-0c4c4f2482be\\\",\\\"ServiceInstance\\\":\\\"MicrosoftCommunicationsOnline/APAC-AU1-S1\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"42a3ec34-28ba-46b6-992f-db53a675ac5b\\\"},{\\\"SubscribedPlanId\\\":\\\"e039cc95-628d-4ade-80ce-f77a46135dde\\\",\\\"ServiceInstance\\\":\\\"MicrosoftStream/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"743dd19e-1ce3-4c62-a3ad-49ba8f63a2f6\\\"},{\\\"SubscribedPlanId\\\":\\\"dddc5824-34a0-4b85-b6b8-0fafe67a57b0\\\",\\\"ServiceInstance\\\":\\\"OfficeForms/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"159f4cd6-e380-449f-a816-af1a9ef76344\\\"},{\\\"SubscribedPlanId\\\":\\\"d1c57312-4814-4818-a991-38bb7429b211\\\",\\\"ServiceInstance\\\":\\\"TeamspaceAPI/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"57ff2da0-773e-42df-b2af-ffb7a2317929\\\"},{\\\"SubscribedPlanId\\\":\\\"c73a8c4e-f6b6-4998-bf41-862fdea05abd\\\",\\\"ServiceInstance\\\":\\\"ProjectWorkManagement/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b737dad2-2f6c-4c65-90e3-ca563267e8b9\\\"},{\\\"SubscribedPlanId\\\":\\\"b7b9220c-a3f0-437e-b99a-0e925b312c86\\\",\\\"ServiceInstance\\\":\\\"YammerEnterprise/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"7547a3fe-08ee-4ccb-b430-5077c5041653\\\"},{\\\"SubscribedPlanId\\\":\\\"b3ae2021-9f74-4a09-9845-42accad7b182\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bed136c6-b799-4462-824d-fc045d3a9d25\\\"},{\\\"SubscribedPlanId\\\":\\\"a83d2db3-81e2-45ee-bf0e-c1088b24bb96\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"e95bec33-7c88-4a70-8e19-b10bd9d0c014\\\"},{\\\"SubscribedPlanId\\\":\\\"a5d43ea2-3323-489d-a579-068f683b41f7\\\",\\\"ServiceInstance\\\":\\\"ccibotsprod/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0683001c-0492-4d59-9515-d9a6426b5813\\\"},{\\\"SubscribedPlanId\\\":\\\"956ea907-9a03-46cd-8699-95667e82355a\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c63d4d19-e8cb-460e-b37c-4d6c34603745\\\"},{\\\"SubscribedPlanId\\\":\\\"88ae6c56-fccc"},{"key":"c","value":"5"}]</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"703e087d-3728-4730-a45d-131327b86066"},{"key":"seq","value":"1"},{"key":"b","value":"{\"targetUpdatedProperties\":\"[{\\\"Name\\\":\\\"AssignedLicense\\\",\\\"OldValue\\\":[\\\"[SkuName=EXCHANGESTANDARD, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=4b9405b0-7788-4568-add1-99614e613b69, DisabledPlans=[]]\\\",\\\"[SkuName=AAD_PREMIUM_P2, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=84a661c4-e949-4bd2-a560-ed7766fcaf2b, DisabledPlans=[]]\\\",\\\"[SkuName=SPB, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=cbdc14ab-d96c-4c30-b9f4-6ada7cdc1d46, DisabledPlans=[]]\\\",\\\"[SkuName=Microsoft_Teams_Exploratory_Dept, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=e0dfc8b9-9531-4ec8-94b4-9fec23b05fc8, DisabledPlans=[EXCHANGE_S_STANDARD]]\\\"],\\\"NewValue\\\":[\\\"[SkuName=Microsoft_Teams_Exploratory_Dept, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=e0dfc8b9-9531-4ec8-94b4-9fec23b05fc8, DisabledPlans=[EXCHANGE_S_STANDARD]]\\\",\\\"[SkuName=SPB, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=cbdc14ab-d96c-4c30-b9f4-6ada7cdc1d46, DisabledPlans=[]]\\\",\\\"[SkuName=AAD_PREMIUM_P2, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=84a661c4-e949-4bd2-a560-ed7766fcaf2b, DisabledPlans=[]]\\\",\\\"[SkuName=EXCHANGESTANDARD, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=4b9405b0-7788-4568-add1-99614e613b69, DisabledPlans=[]]\\\",\\\"[SkuName=PURVIEW_SUITE_FOR_BUSINESS_PREMIUM_NEW, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=4b60d63d-b535-4209-b2ed-91e5b0d355ea, DisabledPlans=[]]\\\"]},{\\\"Name\\\":\\\"AssignedPlan\\\",\\\"OldValue\\\":[{\\\"SubscribedPlanId\\\":\\\"020805e7-7d5f-4bb3-b898-a3b1259a976f\\\",\\\"ServiceInstance\\\":\\\"VivaSkills/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"13b6da2c-0d84-450e-9f69-a33e221387ca\\\"},{\\\"SubscribedPlanId\\\":\\\"021ef71f-ddbf-4cfb-92fc-cc2c079d8025\\\",\\\"ServiceInstance\\\":\\\"MicrosoftPrint/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"795f6fe0-cc4d-4773-b050-5dde4dc704c9\\\"},{\\\"SubscribedPlanId\\\":\\\"02e3d1d6-4434-4d5c-88b7-a35a509cce87\\\",\\\"ServiceInstance\\\":\\\"YammerEnterprise/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a82fbf69-b4d7-49f4-83a6-915b2cf354f4\\\"},{\\\"SubscribedPlanId\\\":\\\"0a80e2cd-b1e9-477d-829b-95dd228dd66a\\\",\\\"ServiceInstance\\\":\\\"LearningAppServiceInTeams/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b76fb638-6ba6-402a-b9f9-83d28acb3d86\\\"},{\\\"SubscribedPlanId\\\":\\\"0ab4aba1-516c-4f2e-ab1d-4d251481d78b\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"276d6e8a-f056-4f70-b7e8-4fc27f79f809\\\"},{\\\"SubscribedPlanId\\\":\\\"0dfd484c-cc3b-4cd7-be8e-e51c1b4bc0ea\\\",\\\"ServiceInstance\\\":\\\"Sway/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a23b959c-7ce8-4e57-9140-b90eb88a9e97\\\"},{\\\"SubscribedPlanId\\\":\\\"0e6e1ecc-f9bf-4414-9e6f-1828660fd975\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"40b010bb-0b69-4654-ac5e-ba161433f4b4\\\"},{\\\"SubscribedPlanId\\\":\\\"108288ea-660d-4d4e-98ac-a651b4f33745\\\",\\\"ServiceInstance\\\":\\\"DynamicsNAV/OCN\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"39b5c996-467e-4e60-bd62-46066f572726\\\"},{\\\"SubscribedPlanId\\\":\\\"11013c80-c192-4862-bbb5-7b86a741c83a\\\",\\\"ServiceInstance\\\":\\\"WhiteboardServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b8afc642-032e-4de5-8c0a-507a7bba7e5d\\\"},{\\\"SubscribedPlanId\\\":\\\"11b27917-6674-453b-9913-cba7aba6883a\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"dcf9d2f4-772e-4434-b757-77a453cfbc02\\\"},{\\\"SubscribedPlanId\\\":\\\"161014a9-b8bc-4869-85e0-38e0137851e1\\\",\\\"ServiceInstance\\\":\\\"MicrosoftKaizala/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"54fc630f-5a40-48ee-8965-af0503c1386e\\\"},{\\\"SubscribedPlanId\\\":\\\"177b15ab-51b1-47d1-b213-f0e968822a83\\\",\\\"ServiceInstance\\\":\\\"MultiFactorService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8a256a2b-b617-496d-b51b-e76466e88db0\\\"},{\\\"SubscribedPlanId\\\":\\\"1a6d321c-ebe3-4198-8527-0d14340c3009\\\",\\\"ServiceInstance\\\":\\\"ProcessSimple/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0f9b09cb-62d1-4ff4-9129-43f4996f83f4\\\"},{\\\"SubscribedPlanId\\\":\\\"1b044c1d-0c69-4b8d-8b93-03c2ef1fd3da\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c7699d2e-19aa-44de-8edf-1736da088ca1\\\"},{\\\"SubscribedPlanId\\\":\\\"1e9fdb53-be7c-4185-8d79-17a4c14f96ea\\\",\\\"ServiceInstance\\\":\\\"WindowsUpdateforBusinessCloudExtensions/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"7bf960f6-2cd9-443a-8046-5dbff9558365\\\"},{\\\"SubscribedPlanId\\\":\\\"2287b27a-b6ec-40e6-bb03-35170aa2c846\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"41781fb2-bc02-4b7c-bd55-b576c07bb09d\\\"},{\\\"SubscribedPlanId\\\":\\\"22b5463b-d360-473f-80c2-be8e42afcc71\\\",\\\"ServiceInstance\\\":\\\"Chapter5FluidApp/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c4b8c31a-fb44-4c65-9837-a21f55fcabda\\\"},{\\\"SubscribedPlanId\\\":\\\"29ff02e7-b9a1-4c7c-84a8-50aed2f7760d\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"199a5c09-e0ca-4e37-8f7c-b05d533e1ea2\\\"},{\\\"SubscribedPlanId\\\":\\\"33797a9f-7ebf-4160-b3dd-01b418e7fad8\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"176a09a6-7ec5-4039-ac02-b2791c6ba793\\\"},{\\\"SubscribedPlanId\\\":\\\"36e41faa-1e78-4c8b-8453-6b3ca38ab4c1\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a1ace008-72f3-4ea0-8dac-33b3a23a2472\\\"},{\\\"SubscribedPlanId\\\":\\\"3ef79a81-ae21-49b8-8fa7-dc1d795d9671\\\",\\\"ServiceInstance\\\":\\\"ProjectProgramsAndPortfolios/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a55dfd10-0864-46d9-a3cd-da5991a3e0e2\\\"},{\\\"SubscribedPlanId\\\":\\\"3fe538b9-ba8a-451d-a33d-531f60dc7176\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"28b0fa46-c39a-4188-89e2-58e979a6b014\\\"},{\\\"SubscribedPlanId\\\":\\\"4352e4d1-8707-4b5f-bede-d27d1ba5ae13\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9bec7e34-c9fa-40b7-a9d1-bd6d1165c7ed\\\"},{\\\"SubscribedPlanId\\\":\\\"449a3874-a6a4-498d-905d-662cfc611bea\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"f0ff6ac6-297d-49cd-be34-6dfef97f0c28\\\"},{\\\"SubscribedPlanId\\\":\\\"529909ed-7627-4843-bb53-3556b852c9d9\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9aaf7827-d63c-4b61-89c3-182f06f82e5c\\\"},{\\\"SubscribedPlanId\\\":\\\"53ac6e25-a8f6-44bf-b402-9f56b8eecfd9\\\",\\\"ServiceInstance\\\":\\\"To-Do/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5e62787c-c316-451f-b873-1d05acd4d12c\\\"},{\\\"SubscribedPlanId\\\":\\\"630b8d82-59e4-446a-9abe-48485d643257\\\",\\\"ServiceInstance\\\":\\\"WindowsDefenderATP/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bfc1bbd9-981b-4f71-9b82-17c35fd0e2a4\\\"},{\\\"SubscribedPlanId\\\":\\\"694b4e1c-079c-4afe-9d08-f38537955130\\\",\\\"ServiceInstance\\\":\\\"OnlineService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"1fe6227d-3e01-46d0-9510-0acad4ff6e94\\\"},{\\\"SubscribedPlanId\\\":\\\"6bd8d315-6527-4b5e-af48-a682cf93421a\\\",\\\"ServiceInstance\\\":\\\"MicrosoftCommunicationsOnline/APAC-AU1-S1\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0feaeb32-d00e-4d66-bd5a-43b5b83db82c\\\"},{\\\"SubscribedPlanId\\\":\\\"6f907b14-cb0b-4a3a-9bb9-4f951739e103\\\",\\\"ServiceInstance\\\":\\\"Deskless/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8c7d2df8-86f0-4902-b2ed-a0458298f3b3\\\"},{\\\"SubscribedPlanId\\\":\\\"71ac5b1a-e1dc-4ced-"},{"key":"c","value":"5"}]</t>
-  </si>
-  <si>
-    <t>3/1/2026, 5:24:48.524 AM</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"703e087d-3728-4730-a45d-131327b86066"},{"key":"seq","value":"4"},{"key":"b","value":"-497d-9e45-c0ea113b9406\\\",\\\"ServiceInstance\\\":\\\"PowerAppsService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"92f7a6f3-b89b-4bbd-8c30-809e6da5ad1c\\\"},{\\\"SubscribedPlanId\\\":\\\"85ff92c3-df66-4ccc-ba0b-38683b60b371\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"33c4f319-9bdd-48d6-9c4d-410b750a4a5a\\\"},{\\\"SubscribedPlanId\\\":\\\"71ac5b1a-e1dc-4ced-ba2d-059d74e89acf\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"3efbd4ed-8958-4824-8389-1321f8730af8\\\"},{\\\"SubscribedPlanId\\\":\\\"6f907b14-cb0b-4a3a-9bb9-4f951739e103\\\",\\\"ServiceInstance\\\":\\\"Deskless/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8c7d2df8-86f0-4902-b2ed-a0458298f3b3\\\"},{\\\"SubscribedPlanId\\\":\\\"53ac6e25-a8f6-44bf-b402-9f56b8eecfd9\\\",\\\"ServiceInstance\\\":\\\"To-Do/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5e62787c-c316-451f-b873-1d05acd4d12c\\\"},{\\\"SubscribedPlanId\\\":\\\"449a3874-a6a4-498d-905d-662cfc611bea\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"f0ff6ac6-297d-49cd-be34-6dfef97f0c28\\\"},{\\\"SubscribedPlanId\\\":\\\"3ef79a81-ae21-49b8-8fa7-dc1d795d9671\\\",\\\"ServiceInstance\\\":\\\"ProjectProgramsAndPortfolios/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a55dfd10-0864-46d9-a3cd-da5991a3e0e2\\\"},{\\\"SubscribedPlanId\\\":\\\"1b044c1d-0c69-4b8d-8b93-03c2ef1fd3da\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c7699d2e-19aa-44de-8edf-1736da088ca1\\\"},{\\\"SubscribedPlanId\\\":\\\"1a6d321c-ebe3-4198-8527-0d14340c3009\\\",\\\"ServiceInstance\\\":\\\"ProcessSimple/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0f9b09cb-62d1-4ff4-9129-43f4996f83f4\\\"},{\\\"SubscribedPlanId\\\":\\\"11b27917-6674-453b-9913-cba7aba6883a\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"dcf9d2f4-772e-4434-b757-77a453cfbc02\\\"},{\\\"SubscribedPlanId\\\":\\\"11013c80-c192-4862-bbb5-7b86a741c83a\\\",\\\"ServiceInstance\\\":\\\"WhiteboardServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b8afc642-032e-4de5-8c0a-507a7bba7e5d\\\"},{\\\"SubscribedPlanId\\\":\\\"0e6e1ecc-f9bf-4414-9e6f-1828660fd975\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"40b010bb-0b69-4654-ac5e-ba161433f4b4\\\"},{\\\"SubscribedPlanId\\\":\\\"0dfd484c-cc3b-4cd7-be8e-e51c1b4bc0ea\\\",\\\"ServiceInstance\\\":\\\"Sway/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a23b959c-7ce8-4e57-9140-b90eb88a9e97\\\"},{\\\"SubscribedPlanId\\\":\\\"e7733084-cf3d-4d56-9cfd-1cd9ea183052\\\",\\\"ServiceInstance\\\":\\\"Adallom/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"932ad362-64a8-4783-9106-97849a1a30b9\\\"},{\\\"SubscribedPlanId\\\":\\\"a22189d7-70fa-482b-9d57-ada39f5e0872\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"eec0eb4f-6444-4f95-aba0-50c24d67f998\\\"},{\\\"SubscribedPlanId\\\":\\\"2287b27a-b6ec-40e6-bb03-35170aa2c846\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"41781fb2-bc02-4b7c-bd55-b576c07bb09d\\\"},{\\\"SubscribedPlanId\\\":\\\"177b15ab-51b1-47d1-b213-f0e968822a83\\\",\\\"ServiceInstance\\\":\\\"MultiFactorService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8a256a2b-b617-496d-b51b-e76466e88db0\\\"},{\\\"SubscribedPlanId\\\":\\\"58567403-0357-4227-8e24-d24ac70caac2\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.425751Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"617b097b-4b93-4ede-83de-5f075bb5fb2f\\\"},{\\\"SubscribedPlanId\\\":\\\"963ac82d-37a8-4f4c-baa4-66b1534f8353\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.425751Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b1188c4c-1b36-4018-b48b-ee07604f6feb\\\"},{\\\"SubscribedPlanId\\\":\\\"32b1b5b1-66f5-440a-b9ab-761ae0de5c3d\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.425751Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"4de31727-a228-4ec3-a5bf-8e45b5ca48cc\\\"},{\\\"SubscribedPlanId\\\":\\\"9e5b8d09-b8e5-4f2c-93a0-fd7923ce9434\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.425751Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"65cc641f-cccd-4643-97e0-a17e3045e541\\\"},{\\\"SubscribedPlanId\\\":\\\"83ed6518-e5d3-4cf9-a57c-b3eb1231d38f\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.425751Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"d2d51368-76c9-4317-ada2-a12c004c432f\\\"},{\\\"SubscribedPlanId\\\":\\\"4d30549f-7bcb-4a9d-94e0-cfc57bf8ae10\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.425751Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9d0c4ee5-e4a1-4625-ab39-d82b619b1a34\\\"},{\\\"SubscribedPlanId\\\":\\\"5e83a7db-303f-48b4-9514-d8afa4ee812d\\\",\\\"ServiceInstance\\\":\\\"Office365InsiderRisk/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.425751Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"d587c7a3-bda9-4f99-8776-9bcf59c84f75\\\"},{\\\"SubscribedPlanId\\\":\\\"60517d0d-a18e-44b4-9967-dbbb00475411\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4267508Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"e26c2fcc-ab91-4a61-b35c-03cdc8dddf66\\\"},{\\\"SubscribedPlanId\\\":\\\"a507d475-c032-4d54-92a2-176f6b57256d\\\",\\\"ServiceInstance\\\":\\\"MicrosoftEndpointDLP/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4267508Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"64bfac92-2b17-4482-b5e5-a0304429de3e\\\"},{\\\"SubscribedPlanId\\\":\\\"f039ab05-e70d-49d9-884f-22b99b2b9464\\\",\\\"ServiceInstance\\\":\\\"Adallom/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4267508Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"2e2ddb96-6af9-4b1d-a3f0-d6ecfd22edb2\\\"},{\\\"SubscribedPlanId\\\":\\\"3d063696-1e64-4da3-bf5a-c9f9acad1a63\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4267508Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"6db1f1db-2b46-403f-be40-e39395f08dbb\\\"},{\\\"SubscribedPlanId\\\":\\\"42a28204-69e3-45a0-a05d-e3cab2f3a511\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4267508Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"6dc145d6-95dd-4191-b9c3-185575ee6f6b\\\"},{\\\"SubscribedPlanId\\\":\\\"9b6a0da3-ab6f-444c-9d2f-dd38db48e7c2\\\",\\\"ServiceInstance\\\":\\\"M365CommunicationCompliance/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4267508Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a413a9ff-720c-4822-98ef-2f37c2a21f4c\\\"},{\\\"SubscribedPlanId\\\":\\\"bb1ff8c5-ee94-4fb6-8303-cae3797020ad\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4267508Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"f6de4823-28fa-440b-b886-4783fa86ddba\\\"},{\\\"SubscribedPlanId\\\":\\\"6f498fb0-aae3-4b91-abaa-8aab59767e21\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4267508Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"2f442157-a11c-46b9-ae5b-6e39ff4e5849\\\"},{\\\"SubscribedPlanId\\\":\\\"03a75113-5b94-4083-9abc-38bf7ba38e84\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4267508Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5136a095-5cf0-4aff-bec3-e84448b38ea5\\\"},{\\\"SubscribedPlanId\\\":\\\"08dec763-2cbb-47b4-8862-ef7c18e61eec\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4267508Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"efb0351d-3b08-4503-993d-383af8de41e3\\\"},{\\\"SubscribedPlanId\\\":\\\"a2562c16-aca9-4316-a54b-3d8f61222c1e\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4267508Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c4801e8a-cb58-4c35-aca6-f2dcc106f287\\\"}"},{"key":"c","value":"5"}]</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"703e087d-3728-4730-a45d-131327b86066"},{"key":"seq","value":"5"},{"key":"b","value":",{\\\"SubscribedPlanId\\\":\\\"a48ddbe9-91e5-469c-ad84-9a44d5be8120\\\",\\\"ServiceInstance\\\":\\\"MIPExchangeSolutions/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4277509Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"cd31b152-6326-4d1b-ae1b-997b625182e6\\\"},{\\\"SubscribedPlanId\\\":\\\"77183285-9618-493a-aab7-221b307b5b22\\\",\\\"ServiceInstance\\\":\\\"CustomerLockbox/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4277509Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"3ec18638-bd4c-4d3b-8905-479ed636b83e\\\"},{\\\"SubscribedPlanId\\\":\\\"d2f707d4-5a1a-4448-85f0-2116fe2a3a39\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4277509Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9f431833-0334-42de-a7dc-70aa40db46db\\\"},{\\\"SubscribedPlanId\\\":\\\"60f24eff-dd31-4f08-a86f-53268db26a59\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4277509Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5689bec4-755d-4753-8b61-40975025187c\\\"}]},{\\\"Name\\\":\\\"LicenseAssignmentDetail\\\",\\\"OldValue\\\":[{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"4b9405b0-7788-4568-add1-99614e613b69\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:19:54.5991182Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"84a661c4-e949-4bd2-a560-ed7766fcaf2b\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:19:54.5991182Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"cbdc14ab-d96c-4c30-b9f4-6ada7cdc1d46\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:19:54.5991182Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"e0dfc8b9-9531-4ec8-94b4-9fec23b05fc8\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:19:54.5991182Z\\\",\\\"DisabledPlans\\\":[\\\"9aaf7827-d63c-4b61-89c3-182f06f82e5c\\\"],\\\"EncodingVersion\\\":2}],\\\"NewValue\\\":[{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"e0dfc8b9-9531-4ec8-94b4-9fec23b05fc8\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:24:48.403751Z\\\",\\\"DisabledPlans\\\":[\\\"9aaf7827-d63c-4b61-89c3-182f06f82e5c\\\"],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"cbdc14ab-d96c-4c30-b9f4-6ada7cdc1d46\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:24:48.4047537Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"84a661c4-e949-4bd2-a560-ed7766fcaf2b\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:24:48.4047537Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"4b9405b0-7788-4568-add1-99614e613b69\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:24:48.4047537Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"4b60d63d-b535-4209-b2ed-91e5b0d355ea\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:24:48.4047537Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2}]},{\\\"Name\\\":\\\"Included Updated Properties\\\",\\\"OldValue\\\":null,\\\"NewValue\\\":\\\"AssignedLicense, AssignedPlan, LicenseAssignmentDetail\\\"},{\\\"Name\\\":\\\"TargetId.UserType\\\",\\\"OldValue\\\":null,\\\"NewValue\\\":\\\"Member\\\"}]\",\"additionalTargets\":\"\",\"additionalDetails\":\"{\\\"UserType\\\":\\\"Member\\\",\\\"User-Agent\\\":\\\"MCAPICommercialProductLicensing\\\"}\"}"},{"key":"c","value":"5"}]</t>
-  </si>
-  <si>
-    <t>3/1/2026, 5:24:48.528 AM</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"1d93e232-9103-4dde-b79f-b88aa014100e"},{"key":"seq","value":"1"},{"key":"b","value":"{\"targetUpdatedProperties\":\"[{\\\"Name\\\":\\\"AssignedLicense\\\",\\\"OldValue\\\":[\\\"[SkuName=EXCHANGESTANDARD, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=4b9405b0-7788-4568-add1-99614e613b69, DisabledPlans=[]]\\\",\\\"[SkuName=AAD_PREMIUM_P2, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=84a661c4-e949-4bd2-a560-ed7766fcaf2b, DisabledPlans=[]]\\\",\\\"[SkuName=SPB, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=cbdc14ab-d96c-4c30-b9f4-6ada7cdc1d46, DisabledPlans=[]]\\\",\\\"[SkuName=Microsoft_Teams_Exploratory_Dept, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=e0dfc8b9-9531-4ec8-94b4-9fec23b05fc8, DisabledPlans=[EXCHANGE_S_STANDARD]]\\\"],\\\"NewValue\\\":[\\\"[SkuName=Microsoft_Teams_Exploratory_Dept, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=e0dfc8b9-9531-4ec8-94b4-9fec23b05fc8, DisabledPlans=[EXCHANGE_S_STANDARD]]\\\",\\\"[SkuName=SPB, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=cbdc14ab-d96c-4c30-b9f4-6ada7cdc1d46, DisabledPlans=[]]\\\",\\\"[SkuName=AAD_PREMIUM_P2, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=84a661c4-e949-4bd2-a560-ed7766fcaf2b, DisabledPlans=[]]\\\",\\\"[SkuName=EXCHANGESTANDARD, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=4b9405b0-7788-4568-add1-99614e613b69, DisabledPlans=[]]\\\",\\\"[SkuName=PURVIEW_SUITE_FOR_BUSINESS_PREMIUM_NEW, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=4b60d63d-b535-4209-b2ed-91e5b0d355ea, DisabledPlans=[]]\\\"]},{\\\"Name\\\":\\\"AssignedPlan\\\",\\\"OldValue\\\":[{\\\"SubscribedPlanId\\\":\\\"020805e7-7d5f-4bb3-b898-a3b1259a976f\\\",\\\"ServiceInstance\\\":\\\"VivaSkills/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"13b6da2c-0d84-450e-9f69-a33e221387ca\\\"},{\\\"SubscribedPlanId\\\":\\\"021ef71f-ddbf-4cfb-92fc-cc2c079d8025\\\",\\\"ServiceInstance\\\":\\\"MicrosoftPrint/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"795f6fe0-cc4d-4773-b050-5dde4dc704c9\\\"},{\\\"SubscribedPlanId\\\":\\\"02e3d1d6-4434-4d5c-88b7-a35a509cce87\\\",\\\"ServiceInstance\\\":\\\"YammerEnterprise/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a82fbf69-b4d7-49f4-83a6-915b2cf354f4\\\"},{\\\"SubscribedPlanId\\\":\\\"0a80e2cd-b1e9-477d-829b-95dd228dd66a\\\",\\\"ServiceInstance\\\":\\\"LearningAppServiceInTeams/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b76fb638-6ba6-402a-b9f9-83d28acb3d86\\\"},{\\\"SubscribedPlanId\\\":\\\"0ab4aba1-516c-4f2e-ab1d-4d251481d78b\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"276d6e8a-f056-4f70-b7e8-4fc27f79f809\\\"},{\\\"SubscribedPlanId\\\":\\\"0dfd484c-cc3b-4cd7-be8e-e51c1b4bc0ea\\\",\\\"ServiceInstance\\\":\\\"Sway/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a23b959c-7ce8-4e57-9140-b90eb88a9e97\\\"},{\\\"SubscribedPlanId\\\":\\\"0e6e1ecc-f9bf-4414-9e6f-1828660fd975\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"40b010bb-0b69-4654-ac5e-ba161433f4b4\\\"},{\\\"SubscribedPlanId\\\":\\\"108288ea-660d-4d4e-98ac-a651b4f33745\\\",\\\"ServiceInstance\\\":\\\"DynamicsNAV/OCN\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"39b5c996-467e-4e60-bd62-46066f572726\\\"},{\\\"SubscribedPlanId\\\":\\\"11013c80-c192-4862-bbb5-7b86a741c83a\\\",\\\"ServiceInstance\\\":\\\"WhiteboardServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b8afc642-032e-4de5-8c0a-507a7bba7e5d\\\"},{\\\"SubscribedPlanId\\\":\\\"11b27917-6674-453b-9913-cba7aba6883a\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"dcf9d2f4-772e-4434-b757-77a453cfbc02\\\"},{\\\"SubscribedPlanId\\\":\\\"161014a9-b8bc-4869-85e0-38e0137851e1\\\",\\\"ServiceInstance\\\":\\\"MicrosoftKaizala/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"54fc630f-5a40-48ee-8965-af0503c1386e\\\"},{\\\"SubscribedPlanId\\\":\\\"177b15ab-51b1-47d1-b213-f0e968822a83\\\",\\\"ServiceInstance\\\":\\\"MultiFactorService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8a256a2b-b617-496d-b51b-e76466e88db0\\\"},{\\\"SubscribedPlanId\\\":\\\"1a6d321c-ebe3-4198-8527-0d14340c3009\\\",\\\"ServiceInstance\\\":\\\"ProcessSimple/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0f9b09cb-62d1-4ff4-9129-43f4996f83f4\\\"},{\\\"SubscribedPlanId\\\":\\\"1b044c1d-0c69-4b8d-8b93-03c2ef1fd3da\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c7699d2e-19aa-44de-8edf-1736da088ca1\\\"},{\\\"SubscribedPlanId\\\":\\\"1e9fdb53-be7c-4185-8d79-17a4c14f96ea\\\",\\\"ServiceInstance\\\":\\\"WindowsUpdateforBusinessCloudExtensions/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"7bf960f6-2cd9-443a-8046-5dbff9558365\\\"},{\\\"SubscribedPlanId\\\":\\\"2287b27a-b6ec-40e6-bb03-35170aa2c846\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"41781fb2-bc02-4b7c-bd55-b576c07bb09d\\\"},{\\\"SubscribedPlanId\\\":\\\"22b5463b-d360-473f-80c2-be8e42afcc71\\\",\\\"ServiceInstance\\\":\\\"Chapter5FluidApp/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c4b8c31a-fb44-4c65-9837-a21f55fcabda\\\"},{\\\"SubscribedPlanId\\\":\\\"29ff02e7-b9a1-4c7c-84a8-50aed2f7760d\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"199a5c09-e0ca-4e37-8f7c-b05d533e1ea2\\\"},{\\\"SubscribedPlanId\\\":\\\"33797a9f-7ebf-4160-b3dd-01b418e7fad8\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"176a09a6-7ec5-4039-ac02-b2791c6ba793\\\"},{\\\"SubscribedPlanId\\\":\\\"36e41faa-1e78-4c8b-8453-6b3ca38ab4c1\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a1ace008-72f3-4ea0-8dac-33b3a23a2472\\\"},{\\\"SubscribedPlanId\\\":\\\"3ef79a81-ae21-49b8-8fa7-dc1d795d9671\\\",\\\"ServiceInstance\\\":\\\"ProjectProgramsAndPortfolios/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a55dfd10-0864-46d9-a3cd-da5991a3e0e2\\\"},{\\\"SubscribedPlanId\\\":\\\"3fe538b9-ba8a-451d-a33d-531f60dc7176\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"28b0fa46-c39a-4188-89e2-58e979a6b014\\\"},{\\\"SubscribedPlanId\\\":\\\"4352e4d1-8707-4b5f-bede-d27d1ba5ae13\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9bec7e34-c9fa-40b7-a9d1-bd6d1165c7ed\\\"},{\\\"SubscribedPlanId\\\":\\\"449a3874-a6a4-498d-905d-662cfc611bea\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"f0ff6ac6-297d-49cd-be34-6dfef97f0c28\\\"},{\\\"SubscribedPlanId\\\":\\\"529909ed-7627-4843-bb53-3556b852c9d9\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9aaf7827-d63c-4b61-89c3-182f06f82e5c\\\"},{\\\"SubscribedPlanId\\\":\\\"53ac6e25-a8f6-44bf-b402-9f56b8eecfd9\\\",\\\"ServiceInstance\\\":\\\"To-Do/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5e62787c-c316-451f-b873-1d05acd4d12c\\\"},{\\\"SubscribedPlanId\\\":\\\"630b8d82-59e4-446a-9abe-48485d643257\\\",\\\"ServiceInstance\\\":\\\"WindowsDefenderATP/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bfc1bbd9-981b-4f71-9b82-17c35fd0e2a4\\\"},{\\\"SubscribedPlanId\\\":\\\"694b4e1c-079c-4afe-9d08-f38537955130\\\",\\\"ServiceInstance\\\":\\\"OnlineService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"1fe6227d-3e01-46d0-9510-0acad4ff6e94\\\"},{\\\"SubscribedPlanId\\\":\\\"6bd8d315-6527-4b5e-af48-a682cf93421a\\\",\\\"ServiceInstance\\\":\\\"MicrosoftCommunicationsOnline/APAC-AU1-S1\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0feaeb32-d00e-4d66-bd5a-43b5b83db82c\\\"},{\\\"SubscribedPlanId\\\":\\\"6f907b14-cb0b-4a3a-9bb9-4f951739e103\\\",\\\"ServiceInstance\\\":\\\"Deskless/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8c7d2df8-86f0-4902-b2ed-a0458298f3b3\\\"},{\\\"SubscribedPlanId\\\":\\\"71ac5b1a-e1dc-4ced-"},{"key":"c","value":"5"}]</t>
-  </si>
-  <si>
-    <t>3/1/2026, 5:24:48.529 AM</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"1d93e232-9103-4dde-b79f-b88aa014100e"},{"key":"seq","value":"2"},{"key":"b","value":"ba2d-059d74e89acf\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"3efbd4ed-8958-4824-8389-1321f8730af8\\\"},{\\\"SubscribedPlanId\\\":\\\"79a085f9-a0a5-47f8-87f4-aac406fd96e5\\\",\\\"ServiceInstance\\\":\\\"ccibotsprod/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"ded3d325-1bdc-453e-8432-5bac26d7a014\\\"},{\\\"SubscribedPlanId\\\":\\\"7aedce94-4e81-4a47-94fc-a18af8012419\\\",\\\"ServiceInstance\\\":\\\"SCO/PROD_AMSUD0101_01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8e9ff0ff-aa7a-4b20-83c1-2f636b600ac2\\\"},{\\\"SubscribedPlanId\\\":\\\"7c3a406a-7181-4717-a008-00e2b758651b\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"de377cbc-0019-4ec2-b77c-3f223947e102\\\"},{\\\"SubscribedPlanId\\\":\\\"7ed1f528-4e3a-4770-bbd1-fc1e8c5ed421\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"094e7854-93fc-4d55-b2c0-3ab5369ebdc1\\\"},{\\\"SubscribedPlanId\\\":\\\"7ff00ebf-2122-4a90-a21b-2dd8d91f47d0\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"afa73018-811e-46e9-988f-f75d2b1b8430\\\"},{\\\"SubscribedPlanId\\\":\\\"85ff92c3-df66-4ccc-ba0b-38683b60b371\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"33c4f319-9bdd-48d6-9c4d-410b750a4a5a\\\"},{\\\"SubscribedPlanId\\\":\\\"88ae6c56-fccc-497d-9e45-c0ea113b9406\\\",\\\"ServiceInstance\\\":\\\"PowerAppsService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"92f7a6f3-b89b-4bbd-8c30-809e6da5ad1c\\\"},{\\\"SubscribedPlanId\\\":\\\"956ea907-9a03-46cd-8699-95667e82355a\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c63d4d19-e8cb-460e-b37c-4d6c34603745\\\"},{\\\"SubscribedPlanId\\\":\\\"a09cb9c4-8e21-4801-8aa3-a841705b1497\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5bfe124c-bbdc-4494-8835-f1297d457d79\\\"},{\\\"SubscribedPlanId\\\":\\\"a22189d7-70fa-482b-9d57-ada39f5e0872\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"eec0eb4f-6444-4f95-aba0-50c24d67f998\\\"},{\\\"SubscribedPlanId\\\":\\\"a5d43ea2-3323-489d-a579-068f683b41f7\\\",\\\"ServiceInstance\\\":\\\"ccibotsprod/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0683001c-0492-4d59-9515-d9a6426b5813\\\"},{\\\"SubscribedPlanId\\\":\\\"a60c7542-c074-4479-af90-4af6caea7a57\\\",\\\"ServiceInstance\\\":\\\"ProjectProgramsAndPortfolios/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b21a6b06-1988-436e-a07b-51ec6d9f52ad\\\"},{\\\"SubscribedPlanId\\\":\\\"a83d2db3-81e2-45ee-bf0e-c1088b24bb96\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"e95bec33-7c88-4a70-8e19-b10bd9d0c014\\\"},{\\\"SubscribedPlanId\\\":\\\"b3ae2021-9f74-4a09-9845-42accad7b182\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bed136c6-b799-4462-824d-fc045d3a9d25\\\"},{\\\"SubscribedPlanId\\\":\\\"b7b9220c-a3f0-437e-b99a-0e925b312c86\\\",\\\"ServiceInstance\\\":\\\"YammerEnterprise/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"7547a3fe-08ee-4ccb-b430-5077c5041653\\\"},{\\\"SubscribedPlanId\\\":\\\"b7f56b27-f5ea-45fb-8884-1a5357c41c37\\\",\\\"ServiceInstance\\\":\\\"Microsoft.ProjectBabylon/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c948ea65-2053-4a5a-8a62-9eaaaf11b522\\\"},{\\\"SubscribedPlanId\\\":\\\"c4031b28-43f8-42d9-b1f4-06f5b955074c\\\",\\\"ServiceInstance\\\":\\\"Bing/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0d0c0d31-fae7-41f2-b909-eaf4d7f26dba\\\"},{\\\"SubscribedPlanId\\\":\\\"c73a8c4e-f6b6-4998-bf41-862fdea05abd\\\",\\\"ServiceInstance\\\":\\\"ProjectWorkManagement/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b737dad2-2f6c-4c65-90e3-ca563267e8b9\\\"},{\\\"SubscribedPlanId\\\":\\\"d1c57312-4814-4818-a991-38bb7429b211\\\",\\\"ServiceInstance\\\":\\\"TeamspaceAPI/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"57ff2da0-773e-42df-b2af-ffb7a2317929\\\"},{\\\"SubscribedPlanId\\\":\\\"dbae48d1-a0ef-497b-b857-608ffb8a0035\\\",\\\"ServiceInstance\\\":\\\"Windows/SDF\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8e229017-d77b-43d5-9305-903395523b99\\\"},{\\\"SubscribedPlanId\\\":\\\"dddc5824-34a0-4b85-b6b8-0fafe67a57b0\\\",\\\"ServiceInstance\\\":\\\"OfficeForms/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"159f4cd6-e380-449f-a816-af1a9ef76344\\\"},{\\\"SubscribedPlanId\\\":\\\"e039cc95-628d-4ade-80ce-f77a46135dde\\\",\\\"ServiceInstance\\\":\\\"MicrosoftStream/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"743dd19e-1ce3-4c62-a3ad-49ba8f63a2f6\\\"},{\\\"SubscribedPlanId\\\":\\\"e7733084-cf3d-4d56-9cfd-1cd9ea183052\\\",\\\"ServiceInstance\\\":\\\"Adallom/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"932ad362-64a8-4783-9106-97849a1a30b9\\\"},{\\\"SubscribedPlanId\\\":\\\"ea16e50b-9303-4b92-9e45-0c4c4f2482be\\\",\\\"ServiceInstance\\\":\\\"MicrosoftCommunicationsOnline/APAC-AU1-S1\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"42a3ec34-28ba-46b6-992f-db53a675ac5b\\\"},{\\\"SubscribedPlanId\\\":\\\"eaf152c0-4eeb-4f3c-8501-39ae7fe6989e\\\",\\\"ServiceInstance\\\":\\\"SCO/PROD_AMSUD0101_01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c1ec4a95-1f05-45b3-a911-aa3fa01094f5\\\"},{\\\"SubscribedPlanId\\\":\\\"eeed2477-7994-4b39-a03f-181c64c7f7fa\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bea4c11e-220a-4e6d-8eb8-8ea15d019f90\\\"},{\\\"SubscribedPlanId\\\":\\\"f16c6e89-93cc-4fd6-b474-59b2cea0231b\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a6520331-d7d4-4276-95f5-15c0933bc757\\\"},{\\\"SubscribedPlanId\\\":\\\"f6ef49c3-1a30-4a87-81bb-33eee7bba192\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"6c57d4b6-3b23-47a5-9bc9-69f17b4947b3\\\"}],\\\"NewValue\\\":[{\\\"SubscribedPlanId\\\":\\\"f6ef49c3-1a30-4a87-81bb-33eee7bba192\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"6c57d4b6-3b23-47a5-9bc9-69f17b4947b3\\\"},{\\\"SubscribedPlanId\\\":\\\"f16c6e89-93cc-4fd6-b474-59b2cea0231b\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a6520331-d7d4-4276-95f5-15c0933bc757\\\"},{\\\"SubscribedPlanId\\\":\\\"eeed2477-7994-4b39-a03f-181c64c7f7fa\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bea4c11e-220a-4e6d-8eb8-8ea15d019f90\\\"},{\\\"SubscribedPlanId\\\":\\\"eaf152c0-4eeb-4f3c-8501-39ae7fe6989e\\\",\\\"ServiceInstance\\\":\\\"SCO/PROD_AMSUD0101_01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c1ec4a95-1f05-45b3-a911-aa3fa01094f5\\\"},{\\\"SubscribedPlanId\\\":\\\"dbae48d1-a0ef-497b-b857-608ffb8a0035\\\",\\\"ServiceInstance\\\":\\\"Windows/SDF\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8e229017-d77b-43d5-9305-903395523b99\\\"},{\\\"SubscribedPlanId\\\":\\\"c4031b28-43f8-42d9-b1f4-06f5b955074c\\\",\\\"ServiceInstance\\\":\\\"Bing/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0d0c0d31-fae7-41f2-b909-eaf4d7f26dba\\\"},{\\\"SubscribedPlanId\\\":\\\"b7f56b27-f5ea-45fb-8884-1a5357c41c37\\\",\\\"ServiceInstance\\\":\\\"Microsoft.ProjectBabylon/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\""},{"key":"c","value":"5"}]</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"1d93e232-9103-4dde-b79f-b88aa014100e"},{"key":"seq","value":"3"},{"key":"b","value":"ServicePlanId\\\":\\\"c948ea65-2053-4a5a-8a62-9eaaaf11b522\\\"},{\\\"SubscribedPlanId\\\":\\\"a60c7542-c074-4479-af90-4af6caea7a57\\\",\\\"ServiceInstance\\\":\\\"ProjectProgramsAndPortfolios/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b21a6b06-1988-436e-a07b-51ec6d9f52ad\\\"},{\\\"SubscribedPlanId\\\":\\\"a09cb9c4-8e21-4801-8aa3-a841705b1497\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5bfe124c-bbdc-4494-8835-f1297d457d79\\\"},{\\\"SubscribedPlanId\\\":\\\"7ff00ebf-2122-4a90-a21b-2dd8d91f47d0\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"afa73018-811e-46e9-988f-f75d2b1b8430\\\"},{\\\"SubscribedPlanId\\\":\\\"7ed1f528-4e3a-4770-bbd1-fc1e8c5ed421\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"094e7854-93fc-4d55-b2c0-3ab5369ebdc1\\\"},{\\\"SubscribedPlanId\\\":\\\"7c3a406a-7181-4717-a008-00e2b758651b\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"de377cbc-0019-4ec2-b77c-3f223947e102\\\"},{\\\"SubscribedPlanId\\\":\\\"7aedce94-4e81-4a47-94fc-a18af8012419\\\",\\\"ServiceInstance\\\":\\\"SCO/PROD_AMSUD0101_01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8e9ff0ff-aa7a-4b20-83c1-2f636b600ac2\\\"},{\\\"SubscribedPlanId\\\":\\\"79a085f9-a0a5-47f8-87f4-aac406fd96e5\\\",\\\"ServiceInstance\\\":\\\"ccibotsprod/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"ded3d325-1bdc-453e-8432-5bac26d7a014\\\"},{\\\"SubscribedPlanId\\\":\\\"6bd8d315-6527-4b5e-af48-a682cf93421a\\\",\\\"ServiceInstance\\\":\\\"MicrosoftCommunicationsOnline/APAC-AU1-S1\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0feaeb32-d00e-4d66-bd5a-43b5b83db82c\\\"},{\\\"SubscribedPlanId\\\":\\\"694b4e1c-079c-4afe-9d08-f38537955130\\\",\\\"ServiceInstance\\\":\\\"OnlineService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"1fe6227d-3e01-46d0-9510-0acad4ff6e94\\\"},{\\\"SubscribedPlanId\\\":\\\"630b8d82-59e4-446a-9abe-48485d643257\\\",\\\"ServiceInstance\\\":\\\"WindowsDefenderATP/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bfc1bbd9-981b-4f71-9b82-17c35fd0e2a4\\\"},{\\\"SubscribedPlanId\\\":\\\"529909ed-7627-4843-bb53-3556b852c9d9\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.425751Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9aaf7827-d63c-4b61-89c3-182f06f82e5c\\\"},{\\\"SubscribedPlanId\\\":\\\"4352e4d1-8707-4b5f-bede-d27d1ba5ae13\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9bec7e34-c9fa-40b7-a9d1-bd6d1165c7ed\\\"},{\\\"SubscribedPlanId\\\":\\\"3fe538b9-ba8a-451d-a33d-531f60dc7176\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"28b0fa46-c39a-4188-89e2-58e979a6b014\\\"},{\\\"SubscribedPlanId\\\":\\\"36e41faa-1e78-4c8b-8453-6b3ca38ab4c1\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a1ace008-72f3-4ea0-8dac-33b3a23a2472\\\"},{\\\"SubscribedPlanId\\\":\\\"33797a9f-7ebf-4160-b3dd-01b418e7fad8\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"176a09a6-7ec5-4039-ac02-b2791c6ba793\\\"},{\\\"SubscribedPlanId\\\":\\\"29ff02e7-b9a1-4c7c-84a8-50aed2f7760d\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"199a5c09-e0ca-4e37-8f7c-b05d533e1ea2\\\"},{\\\"SubscribedPlanId\\\":\\\"22b5463b-d360-473f-80c2-be8e42afcc71\\\",\\\"ServiceInstance\\\":\\\"Chapter5FluidApp/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c4b8c31a-fb44-4c65-9837-a21f55fcabda\\\"},{\\\"SubscribedPlanId\\\":\\\"1e9fdb53-be7c-4185-8d79-17a4c14f96ea\\\",\\\"ServiceInstance\\\":\\\"WindowsUpdateforBusinessCloudExtensions/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"7bf960f6-2cd9-443a-8046-5dbff9558365\\\"},{\\\"SubscribedPlanId\\\":\\\"161014a9-b8bc-4869-85e0-38e0137851e1\\\",\\\"ServiceInstance\\\":\\\"MicrosoftKaizala/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"54fc630f-5a40-48ee-8965-af0503c1386e\\\"},{\\\"SubscribedPlanId\\\":\\\"108288ea-660d-4d4e-98ac-a651b4f33745\\\",\\\"ServiceInstance\\\":\\\"DynamicsNAV/OCN\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"39b5c996-467e-4e60-bd62-46066f572726\\\"},{\\\"SubscribedPlanId\\\":\\\"0ab4aba1-516c-4f2e-ab1d-4d251481d78b\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"276d6e8a-f056-4f70-b7e8-4fc27f79f809\\\"},{\\\"SubscribedPlanId\\\":\\\"0a80e2cd-b1e9-477d-829b-95dd228dd66a\\\",\\\"ServiceInstance\\\":\\\"LearningAppServiceInTeams/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b76fb638-6ba6-402a-b9f9-83d28acb3d86\\\"},{\\\"SubscribedPlanId\\\":\\\"02e3d1d6-4434-4d5c-88b7-a35a509cce87\\\",\\\"ServiceInstance\\\":\\\"YammerEnterprise/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a82fbf69-b4d7-49f4-83a6-915b2cf354f4\\\"},{\\\"SubscribedPlanId\\\":\\\"021ef71f-ddbf-4cfb-92fc-cc2c079d8025\\\",\\\"ServiceInstance\\\":\\\"MicrosoftPrint/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"795f6fe0-cc4d-4773-b050-5dde4dc704c9\\\"},{\\\"SubscribedPlanId\\\":\\\"020805e7-7d5f-4bb3-b898-a3b1259a976f\\\",\\\"ServiceInstance\\\":\\\"VivaSkills/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"13b6da2c-0d84-450e-9f69-a33e221387ca\\\"},{\\\"SubscribedPlanId\\\":\\\"ea16e50b-9303-4b92-9e45-0c4c4f2482be\\\",\\\"ServiceInstance\\\":\\\"MicrosoftCommunicationsOnline/APAC-AU1-S1\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"42a3ec34-28ba-46b6-992f-db53a675ac5b\\\"},{\\\"SubscribedPlanId\\\":\\\"e039cc95-628d-4ade-80ce-f77a46135dde\\\",\\\"ServiceInstance\\\":\\\"MicrosoftStream/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"743dd19e-1ce3-4c62-a3ad-49ba8f63a2f6\\\"},{\\\"SubscribedPlanId\\\":\\\"dddc5824-34a0-4b85-b6b8-0fafe67a57b0\\\",\\\"ServiceInstance\\\":\\\"OfficeForms/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"159f4cd6-e380-449f-a816-af1a9ef76344\\\"},{\\\"SubscribedPlanId\\\":\\\"d1c57312-4814-4818-a991-38bb7429b211\\\",\\\"ServiceInstance\\\":\\\"TeamspaceAPI/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"57ff2da0-773e-42df-b2af-ffb7a2317929\\\"},{\\\"SubscribedPlanId\\\":\\\"c73a8c4e-f6b6-4998-bf41-862fdea05abd\\\",\\\"ServiceInstance\\\":\\\"ProjectWorkManagement/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b737dad2-2f6c-4c65-90e3-ca563267e8b9\\\"},{\\\"SubscribedPlanId\\\":\\\"b7b9220c-a3f0-437e-b99a-0e925b312c86\\\",\\\"ServiceInstance\\\":\\\"YammerEnterprise/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"7547a3fe-08ee-4ccb-b430-5077c5041653\\\"},{\\\"SubscribedPlanId\\\":\\\"b3ae2021-9f74-4a09-9845-42accad7b182\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bed136c6-b799-4462-824d-fc045d3a9d25\\\"},{\\\"SubscribedPlanId\\\":\\\"a83d2db3-81e2-45ee-bf0e-c1088b24bb96\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"e95bec33-7c88-4a70-8e19-b10bd9d0c014\\\"},{\\\"SubscribedPlanId\\\":\\\"a5d43ea2-3323-489d-a579-068f683b41f7\\\",\\\"ServiceInstance\\\":\\\"ccibotsprod/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0683001c-0492-4d59-9515-d9a6426b5813\\\"},{\\\"SubscribedPlanId\\\":\\\"956ea907-9a03-46cd-8699-95667e82355a\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c63d4d19-e8cb-460e-b37c-4d6c34603745\\\"},{\\\"SubscribedPlanId\\\":\\\"88ae6c56-fccc"},{"key":"c","value":"5"}]</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"1d93e232-9103-4dde-b79f-b88aa014100e"},{"key":"seq","value":"5"},{"key":"b","value":",{\\\"SubscribedPlanId\\\":\\\"a48ddbe9-91e5-469c-ad84-9a44d5be8120\\\",\\\"ServiceInstance\\\":\\\"MIPExchangeSolutions/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4277509Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"cd31b152-6326-4d1b-ae1b-997b625182e6\\\"},{\\\"SubscribedPlanId\\\":\\\"77183285-9618-493a-aab7-221b307b5b22\\\",\\\"ServiceInstance\\\":\\\"CustomerLockbox/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4277509Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"3ec18638-bd4c-4d3b-8905-479ed636b83e\\\"},{\\\"SubscribedPlanId\\\":\\\"d2f707d4-5a1a-4448-85f0-2116fe2a3a39\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4277509Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9f431833-0334-42de-a7dc-70aa40db46db\\\"},{\\\"SubscribedPlanId\\\":\\\"60f24eff-dd31-4f08-a86f-53268db26a59\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4277509Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5689bec4-755d-4753-8b61-40975025187c\\\"}]},{\\\"Name\\\":\\\"LicenseAssignmentDetail\\\",\\\"OldValue\\\":[{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"4b9405b0-7788-4568-add1-99614e613b69\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:19:54.5991182Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"84a661c4-e949-4bd2-a560-ed7766fcaf2b\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:19:54.5991182Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"cbdc14ab-d96c-4c30-b9f4-6ada7cdc1d46\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:19:54.5991182Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"e0dfc8b9-9531-4ec8-94b4-9fec23b05fc8\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:19:54.5991182Z\\\",\\\"DisabledPlans\\\":[\\\"9aaf7827-d63c-4b61-89c3-182f06f82e5c\\\"],\\\"EncodingVersion\\\":2}],\\\"NewValue\\\":[{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"e0dfc8b9-9531-4ec8-94b4-9fec23b05fc8\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:24:48.403751Z\\\",\\\"DisabledPlans\\\":[\\\"9aaf7827-d63c-4b61-89c3-182f06f82e5c\\\"],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"cbdc14ab-d96c-4c30-b9f4-6ada7cdc1d46\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:24:48.4047537Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"84a661c4-e949-4bd2-a560-ed7766fcaf2b\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:24:48.4047537Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"4b9405b0-7788-4568-add1-99614e613b69\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:24:48.4047537Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"4b60d63d-b535-4209-b2ed-91e5b0d355ea\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:24:48.4047537Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2}]},{\\\"Name\\\":\\\"Included Updated Properties\\\",\\\"OldValue\\\":null,\\\"NewValue\\\":\\\"AssignedLicense, AssignedPlan, LicenseAssignmentDetail\\\"},{\\\"Name\\\":\\\"TargetId.UserType\\\",\\\"OldValue\\\":null,\\\"NewValue\\\":\\\"Member\\\"}]\",\"additionalTargets\":\"{\\\"AssignedSkuId\\\":[\\\"e0dfc8b9-9531-4ec8-94b4-9fec23b05fc8\\\",\\\"cbdc14ab-d96c-4c30-b9f4-6ada7cdc1d46\\\",\\\"84a661c4-e949-4bd2-a560-ed7766fcaf2b\\\",\\\"4b9405b0-7788-4568-add1-99614e613b69\\\",\\\"4b60d63d-b535-4209-b2ed-91e5b0d355ea\\\"]}\",\"additionalDetails\":\"{\\\"User-Agent\\\":\\\"MCAPICommercialProductLicensing\\\"}\"}"},{"key":"c","value":"5"}]</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"1d93e232-9103-4dde-b79f-b88aa014100e"},{"key":"seq","value":"4"},{"key":"b","value":"-497d-9e45-c0ea113b9406\\\",\\\"ServiceInstance\\\":\\\"PowerAppsService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"92f7a6f3-b89b-4bbd-8c30-809e6da5ad1c\\\"},{\\\"SubscribedPlanId\\\":\\\"85ff92c3-df66-4ccc-ba0b-38683b60b371\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"33c4f319-9bdd-48d6-9c4d-410b750a4a5a\\\"},{\\\"SubscribedPlanId\\\":\\\"71ac5b1a-e1dc-4ced-ba2d-059d74e89acf\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"3efbd4ed-8958-4824-8389-1321f8730af8\\\"},{\\\"SubscribedPlanId\\\":\\\"6f907b14-cb0b-4a3a-9bb9-4f951739e103\\\",\\\"ServiceInstance\\\":\\\"Deskless/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8c7d2df8-86f0-4902-b2ed-a0458298f3b3\\\"},{\\\"SubscribedPlanId\\\":\\\"53ac6e25-a8f6-44bf-b402-9f56b8eecfd9\\\",\\\"ServiceInstance\\\":\\\"To-Do/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5e62787c-c316-451f-b873-1d05acd4d12c\\\"},{\\\"SubscribedPlanId\\\":\\\"449a3874-a6a4-498d-905d-662cfc611bea\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"f0ff6ac6-297d-49cd-be34-6dfef97f0c28\\\"},{\\\"SubscribedPlanId\\\":\\\"3ef79a81-ae21-49b8-8fa7-dc1d795d9671\\\",\\\"ServiceInstance\\\":\\\"ProjectProgramsAndPortfolios/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a55dfd10-0864-46d9-a3cd-da5991a3e0e2\\\"},{\\\"SubscribedPlanId\\\":\\\"1b044c1d-0c69-4b8d-8b93-03c2ef1fd3da\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c7699d2e-19aa-44de-8edf-1736da088ca1\\\"},{\\\"SubscribedPlanId\\\":\\\"1a6d321c-ebe3-4198-8527-0d14340c3009\\\",\\\"ServiceInstance\\\":\\\"ProcessSimple/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0f9b09cb-62d1-4ff4-9129-43f4996f83f4\\\"},{\\\"SubscribedPlanId\\\":\\\"11b27917-6674-453b-9913-cba7aba6883a\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"dcf9d2f4-772e-4434-b757-77a453cfbc02\\\"},{\\\"SubscribedPlanId\\\":\\\"11013c80-c192-4862-bbb5-7b86a741c83a\\\",\\\"ServiceInstance\\\":\\\"WhiteboardServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b8afc642-032e-4de5-8c0a-507a7bba7e5d\\\"},{\\\"SubscribedPlanId\\\":\\\"0e6e1ecc-f9bf-4414-9e6f-1828660fd975\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"40b010bb-0b69-4654-ac5e-ba161433f4b4\\\"},{\\\"SubscribedPlanId\\\":\\\"0dfd484c-cc3b-4cd7-be8e-e51c1b4bc0ea\\\",\\\"ServiceInstance\\\":\\\"Sway/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a23b959c-7ce8-4e57-9140-b90eb88a9e97\\\"},{\\\"SubscribedPlanId\\\":\\\"e7733084-cf3d-4d56-9cfd-1cd9ea183052\\\",\\\"ServiceInstance\\\":\\\"Adallom/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"932ad362-64a8-4783-9106-97849a1a30b9\\\"},{\\\"SubscribedPlanId\\\":\\\"a22189d7-70fa-482b-9d57-ada39f5e0872\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"eec0eb4f-6444-4f95-aba0-50c24d67f998\\\"},{\\\"SubscribedPlanId\\\":\\\"2287b27a-b6ec-40e6-bb03-35170aa2c846\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"41781fb2-bc02-4b7c-bd55-b576c07bb09d\\\"},{\\\"SubscribedPlanId\\\":\\\"177b15ab-51b1-47d1-b213-f0e968822a83\\\",\\\"ServiceInstance\\\":\\\"MultiFactorService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8a256a2b-b617-496d-b51b-e76466e88db0\\\"},{\\\"SubscribedPlanId\\\":\\\"58567403-0357-4227-8e24-d24ac70caac2\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.425751Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"617b097b-4b93-4ede-83de-5f075bb5fb2f\\\"},{\\\"SubscribedPlanId\\\":\\\"963ac82d-37a8-4f4c-baa4-66b1534f8353\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.425751Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b1188c4c-1b36-4018-b48b-ee07604f6feb\\\"},{\\\"SubscribedPlanId\\\":\\\"32b1b5b1-66f5-440a-b9ab-761ae0de5c3d\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.425751Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"4de31727-a228-4ec3-a5bf-8e45b5ca48cc\\\"},{\\\"SubscribedPlanId\\\":\\\"9e5b8d09-b8e5-4f2c-93a0-fd7923ce9434\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.425751Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"65cc641f-cccd-4643-97e0-a17e3045e541\\\"},{\\\"SubscribedPlanId\\\":\\\"83ed6518-e5d3-4cf9-a57c-b3eb1231d38f\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.425751Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"d2d51368-76c9-4317-ada2-a12c004c432f\\\"},{\\\"SubscribedPlanId\\\":\\\"4d30549f-7bcb-4a9d-94e0-cfc57bf8ae10\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.425751Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9d0c4ee5-e4a1-4625-ab39-d82b619b1a34\\\"},{\\\"SubscribedPlanId\\\":\\\"5e83a7db-303f-48b4-9514-d8afa4ee812d\\\",\\\"ServiceInstance\\\":\\\"Office365InsiderRisk/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.425751Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"d587c7a3-bda9-4f99-8776-9bcf59c84f75\\\"},{\\\"SubscribedPlanId\\\":\\\"60517d0d-a18e-44b4-9967-dbbb00475411\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4267508Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"e26c2fcc-ab91-4a61-b35c-03cdc8dddf66\\\"},{\\\"SubscribedPlanId\\\":\\\"a507d475-c032-4d54-92a2-176f6b57256d\\\",\\\"ServiceInstance\\\":\\\"MicrosoftEndpointDLP/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4267508Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"64bfac92-2b17-4482-b5e5-a0304429de3e\\\"},{\\\"SubscribedPlanId\\\":\\\"f039ab05-e70d-49d9-884f-22b99b2b9464\\\",\\\"ServiceInstance\\\":\\\"Adallom/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4267508Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"2e2ddb96-6af9-4b1d-a3f0-d6ecfd22edb2\\\"},{\\\"SubscribedPlanId\\\":\\\"3d063696-1e64-4da3-bf5a-c9f9acad1a63\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4267508Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"6db1f1db-2b46-403f-be40-e39395f08dbb\\\"},{\\\"SubscribedPlanId\\\":\\\"42a28204-69e3-45a0-a05d-e3cab2f3a511\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4267508Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"6dc145d6-95dd-4191-b9c3-185575ee6f6b\\\"},{\\\"SubscribedPlanId\\\":\\\"9b6a0da3-ab6f-444c-9d2f-dd38db48e7c2\\\",\\\"ServiceInstance\\\":\\\"M365CommunicationCompliance/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4267508Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a413a9ff-720c-4822-98ef-2f37c2a21f4c\\\"},{\\\"SubscribedPlanId\\\":\\\"bb1ff8c5-ee94-4fb6-8303-cae3797020ad\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4267508Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"f6de4823-28fa-440b-b886-4783fa86ddba\\\"},{\\\"SubscribedPlanId\\\":\\\"6f498fb0-aae3-4b91-abaa-8aab59767e21\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4267508Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"2f442157-a11c-46b9-ae5b-6e39ff4e5849\\\"},{\\\"SubscribedPlanId\\\":\\\"03a75113-5b94-4083-9abc-38bf7ba38e84\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4267508Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5136a095-5cf0-4aff-bec3-e84448b38ea5\\\"},{\\\"SubscribedPlanId\\\":\\\"08dec763-2cbb-47b4-8862-ef7c18e61eec\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4267508Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"efb0351d-3b08-4503-993d-383af8de41e3\\\"},{\\\"SubscribedPlanId\\\":\\\"a2562c16-aca9-4316-a54b-3d8f61222c1e\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48.4267508Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c4801e8a-cb58-4c35-aca6-f2dcc106f287\\\"}"},{"key":"c","value":"5"}]</t>
-  </si>
-  <si>
-    <t>3/5/2026, 9:54:25.339 AM</t>
-  </si>
-  <si>
-    <t>[{"id":"9ebb7bc1-ad39-486e-9bf5-056f352fed91","displayName":null,"type":"User","modifiedProperties":[{"displayName":"StrongAuthenticationPhoneAppDetail","oldValue":"[{\"DeviceName\":\"NO_DEVICE\",\"DeviceToken\":\"NO_DEVICE_TOKEN\",\"DeviceTag\":\"SoftwareTokenActivated\",\"PhoneAppVersion\":\"NO_PHONE_APP_VERSION\",\"OathTokenTimeDrift\":0,\"DeviceId\":\"00000000-0000-0000-0000-000000000000\",\"Id\":\"1378ded7-887e-417d-9f8c-0535c94eae5b\",\"TimeInterval\":0,\"AuthenticationType\":2,\"NotificationType\":1,\"LastAuthenticatedTimestamp\":\"2026-02-28T23:56:26.5933494Z\",\"AuthenticatorFlavor\":\"Authenticator\",\"HashFunction\":\"hmacsha1\",\"TenantDeviceId\":null,\"SecuredPartitionId\":20102,\"SecuredKeyId\":7}]","newValue":"[{\"DeviceName\":\"NO_DEVICE\",\"DeviceToken\":\"NO_DEVICE_TOKEN\",\"DeviceTag\":\"SoftwareTokenActivated\",\"PhoneAppVersion\":\"NO_PHONE_APP_VERSION\",\"OathTokenTimeDrift\":0,\"DeviceId\":\"00000000-0000-0000-0000-000000000000\",\"Id\":\"1378ded7-887e-417d-9f8c-0535c94eae5b\",\"TimeInterval\":0,\"AuthenticationType\":2,\"NotificationType\":1,\"LastAuthenticatedTimestamp\":\"2026-03-05T09:54:25.186239Z\",\"AuthenticatorFlavor\":\"Authenticator\",\"HashFunction\":\"hmacsha1\",\"TenantDeviceId\":null,\"SecuredPartitionId\":20102,\"SecuredKeyId\":7}]"},{"displayName":"Included Updated Properties","oldValue":null,"newValue":"\"StrongAuthenticationPhoneAppDetail\""},{"displayName":"TargetId.UserType","oldValue":null,"newValue":"\"Member\""},{"displayName":"ActorId.ServicePrincipalNames","oldValue":null,"newValue":"\"b5a60e17-278b-4c92-a4e2-b9262e66bb28\""},{"displayName":"SPN","oldValue":null,"newValue":"\"b5a60e17-278b-4c92-a4e2-b9262e66bb28\""}],"administrativeUnits":[],"agentType":"notAgentic","userPrincipalName":"donald.anderson@wdlabs.com.au"}]</t>
-  </si>
-  <si>
-    <t>3/6/2026, 3:19:34.986 PM</t>
-  </si>
-  <si>
     <t>[{"id":"9ebb7bc1-ad39-486e-9bf5-056f352fed91","displayName":null,"type":"User","userPrincipalName":"donald.anderson@wdlabs.com.au","modifiedProperties":[],"administrativeUnits":[],"agentType":"notAgentic"}]</t>
   </si>
   <si>
-    <t>[{"key":"id","value":"068fdb26-0bff-4257-a389-aba213b77135"},{"key":"seq","value":"2"},{"key":"b","value":"56b852c9d9\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9aaf7827-d63c-4b61-89c3-182f06f82e5c\\\"},{\\\"SubscribedPlanId\\\":\\\"53ac6e25-a8f6-44bf-b402-9f56b8eecfd9\\\",\\\"ServiceInstance\\\":\\\"To-Do/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5e62787c-c316-451f-b873-1d05acd4d12c\\\"},{\\\"SubscribedPlanId\\\":\\\"58567403-0357-4227-8e24-d24ac70caac2\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"617b097b-4b93-4ede-83de-5f075bb5fb2f\\\"},{\\\"SubscribedPlanId\\\":\\\"5e83a7db-303f-48b4-9514-d8afa4ee812d\\\",\\\"ServiceInstance\\\":\\\"Office365InsiderRisk/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"d587c7a3-bda9-4f99-8776-9bcf59c84f75\\\"},{\\\"SubscribedPlanId\\\":\\\"60517d0d-a18e-44b4-9967-dbbb00475411\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"e26c2fcc-ab91-4a61-b35c-03cdc8dddf66\\\"},{\\\"SubscribedPlanId\\\":\\\"60f24eff-dd31-4f08-a86f-53268db26a59\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5689bec4-755d-4753-8b61-40975025187c\\\"},{\\\"SubscribedPlanId\\\":\\\"630b8d82-59e4-446a-9abe-48485d643257\\\",\\\"ServiceInstance\\\":\\\"WindowsDefenderATP/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bfc1bbd9-981b-4f71-9b82-17c35fd0e2a4\\\"},{\\\"SubscribedPlanId\\\":\\\"694b4e1c-079c-4afe-9d08-f38537955130\\\",\\\"ServiceInstance\\\":\\\"OnlineService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"1fe6227d-3e01-46d0-9510-0acad4ff6e94\\\"},{\\\"SubscribedPlanId\\\":\\\"6bd8d315-6527-4b5e-af48-a682cf93421a\\\",\\\"ServiceInstance\\\":\\\"MicrosoftCommunicationsOnline/APAC-AU1-S1\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0feaeb32-d00e-4d66-bd5a-43b5b83db82c\\\"},{\\\"SubscribedPlanId\\\":\\\"6f498fb0-aae3-4b91-abaa-8aab59767e21\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"2f442157-a11c-46b9-ae5b-6e39ff4e5849\\\"},{\\\"SubscribedPlanId\\\":\\\"6f907b14-cb0b-4a3a-9bb9-4f951739e103\\\",\\\"ServiceInstance\\\":\\\"Deskless/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8c7d2df8-86f0-4902-b2ed-a0458298f3b3\\\"},{\\\"SubscribedPlanId\\\":\\\"71ac5b1a-e1dc-4ced-ba2d-059d74e89acf\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"3efbd4ed-8958-4824-8389-1321f8730af8\\\"},{\\\"SubscribedPlanId\\\":\\\"77183285-9618-493a-aab7-221b307b5b22\\\",\\\"ServiceInstance\\\":\\\"CustomerLockbox/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"3ec18638-bd4c-4d3b-8905-479ed636b83e\\\"},{\\\"SubscribedPlanId\\\":\\\"79a085f9-a0a5-47f8-87f4-aac406fd96e5\\\",\\\"ServiceInstance\\\":\\\"ccibotsprod/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"ded3d325-1bdc-453e-8432-5bac26d7a014\\\"},{\\\"SubscribedPlanId\\\":\\\"7aedce94-4e81-4a47-94fc-a18af8012419\\\",\\\"ServiceInstance\\\":\\\"SCO/PROD_AMSUD0101_01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8e9ff0ff-aa7a-4b20-83c1-2f636b600ac2\\\"},{\\\"SubscribedPlanId\\\":\\\"7c3a406a-7181-4717-a008-00e2b758651b\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"de377cbc-0019-4ec2-b77c-3f223947e102\\\"},{\\\"SubscribedPlanId\\\":\\\"7ed1f528-4e3a-4770-bbd1-fc1e8c5ed421\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"094e7854-93fc-4d55-b2c0-3ab5369ebdc1\\\"},{\\\"SubscribedPlanId\\\":\\\"7ff00ebf-2122-4a90-a21b-2dd8d91f47d0\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"afa73018-811e-46e9-988f-f75d2b1b8430\\\"},{\\\"SubscribedPlanId\\\":\\\"83ed6518-e5d3-4cf9-a57c-b3eb1231d38f\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"d2d51368-76c9-4317-ada2-a12c004c432f\\\"},{\\\"SubscribedPlanId\\\":\\\"85ff92c3-df66-4ccc-ba0b-38683b60b371\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"33c4f319-9bdd-48d6-9c4d-410b750a4a5a\\\"},{\\\"SubscribedPlanId\\\":\\\"88ae6c56-fccc-497d-9e45-c0ea113b9406\\\",\\\"ServiceInstance\\\":\\\"PowerAppsService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"92f7a6f3-b89b-4bbd-8c30-809e6da5ad1c\\\"},{\\\"SubscribedPlanId\\\":\\\"956ea907-9a03-46cd-8699-95667e82355a\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c63d4d19-e8cb-460e-b37c-4d6c34603745\\\"},{\\\"SubscribedPlanId\\\":\\\"963ac82d-37a8-4f4c-baa4-66b1534f8353\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b1188c4c-1b36-4018-b48b-ee07604f6feb\\\"},{\\\"SubscribedPlanId\\\":\\\"9b6a0da3-ab6f-444c-9d2f-dd38db48e7c2\\\",\\\"ServiceInstance\\\":\\\"M365CommunicationCompliance/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a413a9ff-720c-4822-98ef-2f37c2a21f4c\\\"},{\\\"SubscribedPlanId\\\":\\\"9e5b8d09-b8e5-4f2c-93a0-fd7923ce9434\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"65cc641f-cccd-4643-97e0-a17e3045e541\\\"},{\\\"SubscribedPlanId\\\":\\\"a09cb9c4-8e21-4801-8aa3-a841705b1497\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5bfe124c-bbdc-4494-8835-f1297d457d79\\\"},{\\\"SubscribedPlanId\\\":\\\"a22189d7-70fa-482b-9d57-ada39f5e0872\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"eec0eb4f-6444-4f95-aba0-50c24d67f998\\\"},{\\\"SubscribedPlanId\\\":\\\"a2562c16-aca9-4316-a54b-3d8f61222c1e\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c4801e8a-cb58-4c35-aca6-f2dcc106f287\\\"},{\\\"SubscribedPlanId\\\":\\\"a48ddbe9-91e5-469c-ad84-9a44d5be8120\\\",\\\"ServiceInstance\\\":\\\"MIPExchangeSolutions/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"cd31b152-6326-4d1b-ae1b-997b625182e6\\\"},{\\\"SubscribedPlanId\\\":\\\"a507d475-c032-4d54-92a2-176f6b57256d\\\",\\\"ServiceInstance\\\":\\\"MicrosoftEndpointDLP/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"64bfac92-2b17-4482-b5e5-a0304429de3e\\\"},{\\\"SubscribedPlanId\\\":\\\"a5d43ea2-3323-489d-a579-068f683b41f7\\\",\\\"ServiceInstance\\\":\\\"ccibotsprod/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0683001c-0492-4d59-9515-d9a6426b5813\\\"},{\\\"SubscribedPlanId\\\":\\\"a60c7542-c074-4479-af90-4af6caea7a57\\\",\\\"ServiceInstance\\\":\\\"ProjectProgramsAndPortfolios/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b21a6b06-1988-436e-a07b-51ec6d9f52ad\\\"},{\\\"SubscribedPlanId\\\":\\\"a83d2db3-81e2-45ee-bf0e-c1088b24bb96\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"e95bec33-7c88-4a70-8e19-b10bd9d0c014\\\"},{\\\"SubscribedPlanId\\\":\\\"b3ae2021-9f74-4a09-9845-42accad7b182\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bed136c6-b799-4462-824d-fc045d3a9d25\\\"},{\\\"SubscribedPlanId\\\":\\\"b7b9220c-a3f0-437e-b99a-0e925b312c86\\\",\\\"ServiceInstance\\\":\\\"YammerEnterprise/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"7547a3fe-08ee-4ccb-b430-5077c5041653\\\"},{\\\"SubscribedPlanId\\\":\\\"b7f56b27-f5ea-45fb-8884-1a5357c41c37\\\",\\\"ServiceInstance\\\":\\\"Microsoft.ProjectBabylon/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTim"},{"key":"c","value":"6"}]</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"068fdb26-0bff-4257-a389-aba213b77135"},{"key":"seq","value":"1"},{"key":"b","value":"{\"targetUpdatedProperties\":\"[{\\\"Name\\\":\\\"AssignedLicense\\\",\\\"OldValue\\\":[\\\"[SkuName=PURVIEW_SUITE_FOR_BUSINESS_PREMIUM_NEW, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=4b60d63d-b535-4209-b2ed-91e5b0d355ea, DisabledPlans=[]]\\\",\\\"[SkuName=EXCHANGESTANDARD, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=4b9405b0-7788-4568-add1-99614e613b69, DisabledPlans=[]]\\\",\\\"[SkuName=AAD_PREMIUM_P2, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=84a661c4-e949-4bd2-a560-ed7766fcaf2b, DisabledPlans=[]]\\\",\\\"[SkuName=SPB, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=cbdc14ab-d96c-4c30-b9f4-6ada7cdc1d46, DisabledPlans=[]]\\\",\\\"[SkuName=Microsoft_Teams_Exploratory_Dept, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=e0dfc8b9-9531-4ec8-94b4-9fec23b05fc8, DisabledPlans=[EXCHANGE_S_STANDARD]]\\\"],\\\"NewValue\\\":[\\\"[SkuName=SPB, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=cbdc14ab-d96c-4c30-b9f4-6ada7cdc1d46, DisabledPlans=[]]\\\",\\\"[SkuName=AAD_PREMIUM_P2, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=84a661c4-e949-4bd2-a560-ed7766fcaf2b, DisabledPlans=[]]\\\",\\\"[SkuName=EXCHANGESTANDARD, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=4b9405b0-7788-4568-add1-99614e613b69, DisabledPlans=[]]\\\",\\\"[SkuName=PURVIEW_SUITE_FOR_BUSINESS_PREMIUM_NEW, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=4b60d63d-b535-4209-b2ed-91e5b0d355ea, DisabledPlans=[]]\\\"]},{\\\"Name\\\":\\\"AssignedPlan\\\",\\\"OldValue\\\":[{\\\"SubscribedPlanId\\\":\\\"020805e7-7d5f-4bb3-b898-a3b1259a976f\\\",\\\"ServiceInstance\\\":\\\"VivaSkills/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"13b6da2c-0d84-450e-9f69-a33e221387ca\\\"},{\\\"SubscribedPlanId\\\":\\\"021ef71f-ddbf-4cfb-92fc-cc2c079d8025\\\",\\\"ServiceInstance\\\":\\\"MicrosoftPrint/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"795f6fe0-cc4d-4773-b050-5dde4dc704c9\\\"},{\\\"SubscribedPlanId\\\":\\\"02e3d1d6-4434-4d5c-88b7-a35a509cce87\\\",\\\"ServiceInstance\\\":\\\"YammerEnterprise/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a82fbf69-b4d7-49f4-83a6-915b2cf354f4\\\"},{\\\"SubscribedPlanId\\\":\\\"03a75113-5b94-4083-9abc-38bf7ba38e84\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5136a095-5cf0-4aff-bec3-e84448b38ea5\\\"},{\\\"SubscribedPlanId\\\":\\\"08dec763-2cbb-47b4-8862-ef7c18e61eec\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"efb0351d-3b08-4503-993d-383af8de41e3\\\"},{\\\"SubscribedPlanId\\\":\\\"0a80e2cd-b1e9-477d-829b-95dd228dd66a\\\",\\\"ServiceInstance\\\":\\\"LearningAppServiceInTeams/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b76fb638-6ba6-402a-b9f9-83d28acb3d86\\\"},{\\\"SubscribedPlanId\\\":\\\"0ab4aba1-516c-4f2e-ab1d-4d251481d78b\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"276d6e8a-f056-4f70-b7e8-4fc27f79f809\\\"},{\\\"SubscribedPlanId\\\":\\\"0dfd484c-cc3b-4cd7-be8e-e51c1b4bc0ea\\\",\\\"ServiceInstance\\\":\\\"Sway/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a23b959c-7ce8-4e57-9140-b90eb88a9e97\\\"},{\\\"SubscribedPlanId\\\":\\\"0e6e1ecc-f9bf-4414-9e6f-1828660fd975\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"40b010bb-0b69-4654-ac5e-ba161433f4b4\\\"},{\\\"SubscribedPlanId\\\":\\\"108288ea-660d-4d4e-98ac-a651b4f33745\\\",\\\"ServiceInstance\\\":\\\"DynamicsNAV/OCN\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"39b5c996-467e-4e60-bd62-46066f572726\\\"},{\\\"SubscribedPlanId\\\":\\\"11013c80-c192-4862-bbb5-7b86a741c83a\\\",\\\"ServiceInstance\\\":\\\"WhiteboardServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b8afc642-032e-4de5-8c0a-507a7bba7e5d\\\"},{\\\"SubscribedPlanId\\\":\\\"11b27917-6674-453b-9913-cba7aba6883a\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"dcf9d2f4-772e-4434-b757-77a453cfbc02\\\"},{\\\"SubscribedPlanId\\\":\\\"161014a9-b8bc-4869-85e0-38e0137851e1\\\",\\\"ServiceInstance\\\":\\\"MicrosoftKaizala/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"54fc630f-5a40-48ee-8965-af0503c1386e\\\"},{\\\"SubscribedPlanId\\\":\\\"177b15ab-51b1-47d1-b213-f0e968822a83\\\",\\\"ServiceInstance\\\":\\\"MultiFactorService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8a256a2b-b617-496d-b51b-e76466e88db0\\\"},{\\\"SubscribedPlanId\\\":\\\"1a6d321c-ebe3-4198-8527-0d14340c3009\\\",\\\"ServiceInstance\\\":\\\"ProcessSimple/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0f9b09cb-62d1-4ff4-9129-43f4996f83f4\\\"},{\\\"SubscribedPlanId\\\":\\\"1b044c1d-0c69-4b8d-8b93-03c2ef1fd3da\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c7699d2e-19aa-44de-8edf-1736da088ca1\\\"},{\\\"SubscribedPlanId\\\":\\\"1e9fdb53-be7c-4185-8d79-17a4c14f96ea\\\",\\\"ServiceInstance\\\":\\\"WindowsUpdateforBusinessCloudExtensions/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"7bf960f6-2cd9-443a-8046-5dbff9558365\\\"},{\\\"SubscribedPlanId\\\":\\\"2287b27a-b6ec-40e6-bb03-35170aa2c846\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"41781fb2-bc02-4b7c-bd55-b576c07bb09d\\\"},{\\\"SubscribedPlanId\\\":\\\"22b5463b-d360-473f-80c2-be8e42afcc71\\\",\\\"ServiceInstance\\\":\\\"Chapter5FluidApp/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c4b8c31a-fb44-4c65-9837-a21f55fcabda\\\"},{\\\"SubscribedPlanId\\\":\\\"29ff02e7-b9a1-4c7c-84a8-50aed2f7760d\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"199a5c09-e0ca-4e37-8f7c-b05d533e1ea2\\\"},{\\\"SubscribedPlanId\\\":\\\"32b1b5b1-66f5-440a-b9ab-761ae0de5c3d\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"4de31727-a228-4ec3-a5bf-8e45b5ca48cc\\\"},{\\\"SubscribedPlanId\\\":\\\"33797a9f-7ebf-4160-b3dd-01b418e7fad8\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"176a09a6-7ec5-4039-ac02-b2791c6ba793\\\"},{\\\"SubscribedPlanId\\\":\\\"36e41faa-1e78-4c8b-8453-6b3ca38ab4c1\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a1ace008-72f3-4ea0-8dac-33b3a23a2472\\\"},{\\\"SubscribedPlanId\\\":\\\"3d063696-1e64-4da3-bf5a-c9f9acad1a63\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"6db1f1db-2b46-403f-be40-e39395f08dbb\\\"},{\\\"SubscribedPlanId\\\":\\\"3ef79a81-ae21-49b8-8fa7-dc1d795d9671\\\",\\\"ServiceInstance\\\":\\\"ProjectProgramsAndPortfolios/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a55dfd10-0864-46d9-a3cd-da5991a3e0e2\\\"},{\\\"SubscribedPlanId\\\":\\\"3fe538b9-ba8a-451d-a33d-531f60dc7176\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"28b0fa46-c39a-4188-89e2-58e979a6b014\\\"},{\\\"SubscribedPlanId\\\":\\\"42a28204-69e3-45a0-a05d-e3cab2f3a511\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"6dc145d6-95dd-4191-b9c3-185575ee6f6b\\\"},{\\\"SubscribedPlanId\\\":\\\"4352e4d1-8707-4b5f-bede-d27d1ba5ae13\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9bec7e34-c9fa-40b7-a9d1-bd6d1165c7ed\\\"},{\\\"SubscribedPlanId\\\":\\\"449a3874-a6a4-498d-905d-662cfc611bea\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"f0ff6ac6-297d-49cd-be34-6dfef97f0c28\\\"},{\\\"SubscribedPlanId\\\":\\\"4d30549f-7bcb-4a9d-94e0-cfc57bf8ae10\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9d0c4ee5-e4a1-4625-ab39-d82b619b1a34\\\"},{\\\"SubscribedPlanId\\\":\\\"529909ed-7627-4843-bb53-35"},{"key":"c","value":"6"}]</t>
-  </si>
-  <si>
-    <t>3/6/2026, 3:19:34.987 PM</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"068fdb26-0bff-4257-a389-aba213b77135"},{"key":"seq","value":"3"},{"key":"b","value":"estamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c948ea65-2053-4a5a-8a62-9eaaaf11b522\\\"},{\\\"SubscribedPlanId\\\":\\\"bb1ff8c5-ee94-4fb6-8303-cae3797020ad\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"f6de4823-28fa-440b-b886-4783fa86ddba\\\"},{\\\"SubscribedPlanId\\\":\\\"c4031b28-43f8-42d9-b1f4-06f5b955074c\\\",\\\"ServiceInstance\\\":\\\"Bing/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0d0c0d31-fae7-41f2-b909-eaf4d7f26dba\\\"},{\\\"SubscribedPlanId\\\":\\\"c73a8c4e-f6b6-4998-bf41-862fdea05abd\\\",\\\"ServiceInstance\\\":\\\"ProjectWorkManagement/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b737dad2-2f6c-4c65-90e3-ca563267e8b9\\\"},{\\\"SubscribedPlanId\\\":\\\"d1c57312-4814-4818-a991-38bb7429b211\\\",\\\"ServiceInstance\\\":\\\"TeamspaceAPI/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"57ff2da0-773e-42df-b2af-ffb7a2317929\\\"},{\\\"SubscribedPlanId\\\":\\\"d2f707d4-5a1a-4448-85f0-2116fe2a3a39\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9f431833-0334-42de-a7dc-70aa40db46db\\\"},{\\\"SubscribedPlanId\\\":\\\"dbae48d1-a0ef-497b-b857-608ffb8a0035\\\",\\\"ServiceInstance\\\":\\\"Windows/SDF\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8e229017-d77b-43d5-9305-903395523b99\\\"},{\\\"SubscribedPlanId\\\":\\\"dddc5824-34a0-4b85-b6b8-0fafe67a57b0\\\",\\\"ServiceInstance\\\":\\\"OfficeForms/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"159f4cd6-e380-449f-a816-af1a9ef76344\\\"},{\\\"SubscribedPlanId\\\":\\\"e039cc95-628d-4ade-80ce-f77a46135dde\\\",\\\"ServiceInstance\\\":\\\"MicrosoftStream/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"743dd19e-1ce3-4c62-a3ad-49ba8f63a2f6\\\"},{\\\"SubscribedPlanId\\\":\\\"e7733084-cf3d-4d56-9cfd-1cd9ea183052\\\",\\\"ServiceInstance\\\":\\\"Adallom/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"932ad362-64a8-4783-9106-97849a1a30b9\\\"},{\\\"SubscribedPlanId\\\":\\\"ea16e50b-9303-4b92-9e45-0c4c4f2482be\\\",\\\"ServiceInstance\\\":\\\"MicrosoftCommunicationsOnline/APAC-AU1-S1\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"42a3ec34-28ba-46b6-992f-db53a675ac5b\\\"},{\\\"SubscribedPlanId\\\":\\\"eaf152c0-4eeb-4f3c-8501-39ae7fe6989e\\\",\\\"ServiceInstance\\\":\\\"SCO/PROD_AMSUD0101_01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c1ec4a95-1f05-45b3-a911-aa3fa01094f5\\\"},{\\\"SubscribedPlanId\\\":\\\"eeed2477-7994-4b39-a03f-181c64c7f7fa\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bea4c11e-220a-4e6d-8eb8-8ea15d019f90\\\"},{\\\"SubscribedPlanId\\\":\\\"f039ab05-e70d-49d9-884f-22b99b2b9464\\\",\\\"ServiceInstance\\\":\\\"Adallom/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"2e2ddb96-6af9-4b1d-a3f0-d6ecfd22edb2\\\"},{\\\"SubscribedPlanId\\\":\\\"f16c6e89-93cc-4fd6-b474-59b2cea0231b\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a6520331-d7d4-4276-95f5-15c0933bc757\\\"},{\\\"SubscribedPlanId\\\":\\\"f6ef49c3-1a30-4a87-81bb-33eee7bba192\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"6c57d4b6-3b23-47a5-9bc9-69f17b4947b3\\\"}],\\\"NewValue\\\":[{\\\"SubscribedPlanId\\\":\\\"f039ab05-e70d-49d9-884f-22b99b2b9464\\\",\\\"ServiceInstance\\\":\\\"Adallom/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"2e2ddb96-6af9-4b1d-a3f0-d6ecfd22edb2\\\"},{\\\"SubscribedPlanId\\\":\\\"d2f707d4-5a1a-4448-85f0-2116fe2a3a39\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9f431833-0334-42de-a7dc-70aa40db46db\\\"},{\\\"SubscribedPlanId\\\":\\\"bb1ff8c5-ee94-4fb6-8303-cae3797020ad\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"f6de4823-28fa-440b-b886-4783fa86ddba\\\"},{\\\"SubscribedPlanId\\\":\\\"a507d475-c032-4d54-92a2-176f6b57256d\\\",\\\"ServiceInstance\\\":\\\"MicrosoftEndpointDLP/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"64bfac92-2b17-4482-b5e5-a0304429de3e\\\"},{\\\"SubscribedPlanId\\\":\\\"a48ddbe9-91e5-469c-ad84-9a44d5be8120\\\",\\\"ServiceInstance\\\":\\\"MIPExchangeSolutions/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"cd31b152-6326-4d1b-ae1b-997b625182e6\\\"},{\\\"SubscribedPlanId\\\":\\\"a2562c16-aca9-4316-a54b-3d8f61222c1e\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c4801e8a-cb58-4c35-aca6-f2dcc106f287\\\"},{\\\"SubscribedPlanId\\\":\\\"9e5b8d09-b8e5-4f2c-93a0-fd7923ce9434\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"65cc641f-cccd-4643-97e0-a17e3045e541\\\"},{\\\"SubscribedPlanId\\\":\\\"9b6a0da3-ab6f-444c-9d2f-dd38db48e7c2\\\",\\\"ServiceInstance\\\":\\\"M365CommunicationCompliance/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a413a9ff-720c-4822-98ef-2f37c2a21f4c\\\"},{\\\"SubscribedPlanId\\\":\\\"963ac82d-37a8-4f4c-baa4-66b1534f8353\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b1188c4c-1b36-4018-b48b-ee07604f6feb\\\"},{\\\"SubscribedPlanId\\\":\\\"83ed6518-e5d3-4cf9-a57c-b3eb1231d38f\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"d2d51368-76c9-4317-ada2-a12c004c432f\\\"},{\\\"SubscribedPlanId\\\":\\\"77183285-9618-493a-aab7-221b307b5b22\\\",\\\"ServiceInstance\\\":\\\"CustomerLockbox/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"3ec18638-bd4c-4d3b-8905-479ed636b83e\\\"},{\\\"SubscribedPlanId\\\":\\\"6f498fb0-aae3-4b91-abaa-8aab59767e21\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"2f442157-a11c-46b9-ae5b-6e39ff4e5849\\\"},{\\\"SubscribedPlanId\\\":\\\"60f24eff-dd31-4f08-a86f-53268db26a59\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5689bec4-755d-4753-8b61-40975025187c\\\"},{\\\"SubscribedPlanId\\\":\\\"60517d0d-a18e-44b4-9967-dbbb00475411\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"e26c2fcc-ab91-4a61-b35c-03cdc8dddf66\\\"},{\\\"SubscribedPlanId\\\":\\\"5e83a7db-303f-48b4-9514-d8afa4ee812d\\\",\\\"ServiceInstance\\\":\\\"Office365InsiderRisk/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"d587c7a3-bda9-4f99-8776-9bcf59c84f75\\\"},{\\\"SubscribedPlanId\\\":\\\"58567403-0357-4227-8e24-d24ac70caac2\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"617b097b-4b93-4ede-83de-5f075bb5fb2f\\\"},{\\\"SubscribedPlanId\\\":\\\"529909ed-7627-4843-bb53-3556b852c9d9\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9270494Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9aaf7827-d63c-4b61-89c3-182f06f82e5c\\\"},{\\\"SubscribedPlanId\\\":\\\"4d30549f-7bcb-4a9d-94e0-cfc57bf8ae10\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9d0c4ee5-e4a1-4625-ab39-d82b619b1a34\\\"},{\\\"SubscribedPlanId\\\":\\\"42a28204-69e3-45a0-a05d-e3cab2f3a511\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"6dc145d6-95dd-4191-b9c3-185575ee6f6b\\\"},{\\\"SubscribedPlanId\\\":\\\"3d063696-1e64-4da3-bf5a-c9f9acad1a63\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"6db1f1db-2b46-403f-be40-e39395f08dbb\\\"},{\\\"SubscribedPla"},{"key":"c","value":"6"}]</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"068fdb26-0bff-4257-a389-aba213b77135"},{"key":"seq","value":"5"},{"key":"b","value":"yStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9260535Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"743dd19e-1ce3-4c62-a3ad-49ba8f63a2f6\\\"},{\\\"SubscribedPlanId\\\":\\\"dddc5824-34a0-4b85-b6b8-0fafe67a57b0\\\",\\\"ServiceInstance\\\":\\\"OfficeForms/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9260535Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"159f4cd6-e380-449f-a816-af1a9ef76344\\\"},{\\\"SubscribedPlanId\\\":\\\"d1c57312-4814-4818-a991-38bb7429b211\\\",\\\"ServiceInstance\\\":\\\"TeamspaceAPI/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9260535Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"57ff2da0-773e-42df-b2af-ffb7a2317929\\\"},{\\\"SubscribedPlanId\\\":\\\"c73a8c4e-f6b6-4998-bf41-862fdea05abd\\\",\\\"ServiceInstance\\\":\\\"ProjectWorkManagement/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9270494Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b737dad2-2f6c-4c65-90e3-ca563267e8b9\\\"},{\\\"SubscribedPlanId\\\":\\\"b7b9220c-a3f0-437e-b99a-0e925b312c86\\\",\\\"ServiceInstance\\\":\\\"YammerEnterprise/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9260535Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"7547a3fe-08ee-4ccb-b430-5077c5041653\\\"},{\\\"SubscribedPlanId\\\":\\\"b3ae2021-9f74-4a09-9845-42accad7b182\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":3,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9240496Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bed136c6-b799-4462-824d-fc045d3a9d25\\\"},{\\\"SubscribedPlanId\\\":\\\"a83d2db3-81e2-45ee-bf0e-c1088b24bb96\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9260535Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"e95bec33-7c88-4a70-8e19-b10bd9d0c014\\\"},{\\\"SubscribedPlanId\\\":\\\"a5d43ea2-3323-489d-a579-068f683b41f7\\\",\\\"ServiceInstance\\\":\\\"ccibotsprod/NA001\\\",\\\"CapabilityStatus\\\":3,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9220495Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0683001c-0492-4d59-9515-d9a6426b5813\\\"},{\\\"SubscribedPlanId\\\":\\\"956ea907-9a03-46cd-8699-95667e82355a\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":3,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9230493Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c63d4d19-e8cb-460e-b37c-4d6c34603745\\\"},{\\\"SubscribedPlanId\\\":\\\"88ae6c56-fccc-497d-9e45-c0ea113b9406\\\",\\\"ServiceInstance\\\":\\\"PowerAppsService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9270494Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"92f7a6f3-b89b-4bbd-8c30-809e6da5ad1c\\\"},{\\\"SubscribedPlanId\\\":\\\"85ff92c3-df66-4ccc-ba0b-38683b60b371\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9250496Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"33c4f319-9bdd-48d6-9c4d-410b750a4a5a\\\"},{\\\"SubscribedPlanId\\\":\\\"71ac5b1a-e1dc-4ced-ba2d-059d74e89acf\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9240496Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"3efbd4ed-8958-4824-8389-1321f8730af8\\\"},{\\\"SubscribedPlanId\\\":\\\"6f907b14-cb0b-4a3a-9bb9-4f951739e103\\\",\\\"ServiceInstance\\\":\\\"Deskless/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9250496Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8c7d2df8-86f0-4902-b2ed-a0458298f3b3\\\"},{\\\"SubscribedPlanId\\\":\\\"53ac6e25-a8f6-44bf-b402-9f56b8eecfd9\\\",\\\"ServiceInstance\\\":\\\"To-Do/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9250496Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5e62787c-c316-451f-b873-1d05acd4d12c\\\"},{\\\"SubscribedPlanId\\\":\\\"449a3874-a6a4-498d-905d-662cfc611bea\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9240496Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"f0ff6ac6-297d-49cd-be34-6dfef97f0c28\\\"},{\\\"SubscribedPlanId\\\":\\\"3ef79a81-ae21-49b8-8fa7-dc1d795d9671\\\",\\\"ServiceInstance\\\":\\\"ProjectProgramsAndPortfolios/NA001\\\",\\\"CapabilityStatus\\\":3,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9210495Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a55dfd10-0864-46d9-a3cd-da5991a3e0e2\\\"},{\\\"SubscribedPlanId\\\":\\\"1b044c1d-0c69-4b8d-8b93-03c2ef1fd3da\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9260535Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c7699d2e-19aa-44de-8edf-1736da088ca1\\\"},{\\\"SubscribedPlanId\\\":\\\"1a6d321c-ebe3-4198-8527-0d14340c3009\\\",\\\"ServiceInstance\\\":\\\"ProcessSimple/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9270494Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0f9b09cb-62d1-4ff4-9129-43f4996f83f4\\\"},{\\\"SubscribedPlanId\\\":\\\"11b27917-6674-453b-9913-cba7aba6883a\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9240496Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"dcf9d2f4-772e-4434-b757-77a453cfbc02\\\"},{\\\"SubscribedPlanId\\\":\\\"11013c80-c192-4862-bbb5-7b86a741c83a\\\",\\\"ServiceInstance\\\":\\\"WhiteboardServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9250496Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b8afc642-032e-4de5-8c0a-507a7bba7e5d\\\"},{\\\"SubscribedPlanId\\\":\\\"0e6e1ecc-f9bf-4414-9e6f-1828660fd975\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":3,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9210495Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"40b010bb-0b69-4654-ac5e-ba161433f4b4\\\"},{\\\"SubscribedPlanId\\\":\\\"0dfd484c-cc3b-4cd7-be8e-e51c1b4bc0ea\\\",\\\"ServiceInstance\\\":\\\"Sway/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9260535Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a23b959c-7ce8-4e57-9140-b90eb88a9e97\\\"},{\\\"SubscribedPlanId\\\":\\\"e7733084-cf3d-4d56-9cfd-1cd9ea183052\\\",\\\"ServiceInstance\\\":\\\"Adallom/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"932ad362-64a8-4783-9106-97849a1a30b9\\\"},{\\\"SubscribedPlanId\\\":\\\"a22189d7-70fa-482b-9d57-ada39f5e0872\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"eec0eb4f-6444-4f95-aba0-50c24d67f998\\\"},{\\\"SubscribedPlanId\\\":\\\"2287b27a-b6ec-40e6-bb03-35170aa2c846\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"41781fb2-bc02-4b7c-bd55-b576c07bb09d\\\"},{\\\"SubscribedPlanId\\\":\\\"177b15ab-51b1-47d1-b213-f0e968822a83\\\",\\\"ServiceInstance\\\":\\\"MultiFactorService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8a256a2b-b617-496d-b51b-e76466e88db0\\\"}]},{\\\"Name\\\":\\\"LicenseAssignmentDetail\\\",\\\"OldValue\\\":[{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"4b60d63d-b535-4209-b2ed-91e5b0d355ea\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:24:48.4047537Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"4b9405b0-7788-4568-add1-99614e613b69\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:24:48.4047537Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"84a661c4-e949-4bd2-a560-ed7766fcaf2b\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:24:48.4047537Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"cbdc14ab-d96c-4c30-b9f4-6ada7cdc1d46\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:24:48.4047537Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"e0dfc8b9-9531-4ec8-94b4-9fec23b05fc8\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:24:48.403751Z\\\",\\\"DisabledPlans\\\":[\\\"9aaf7827-d63c-4b61-89c3-182f06f82e5c\\\"],\\\"EncodingVersion\\\":2}],\\\"NewValue\\\":[{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"cbdc14ab-d96c-4c30-b9f4-6ada7cdc1d46\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-06T15:19:34.9040498Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"84a661c4-e949-4bd2-a560-ed7766fcaf2b\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-06T15:19:34.9040498Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"4b9405b0-7788-4568-add1-99614e613b69\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-06T15:19:34.9040498Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\","},{"key":"c","value":"6"}]</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"068fdb26-0bff-4257-a389-aba213b77135"},{"key":"seq","value":"4"},{"key":"b","value":"nId\\\":\\\"32b1b5b1-66f5-440a-b9ab-761ae0de5c3d\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"4de31727-a228-4ec3-a5bf-8e45b5ca48cc\\\"},{\\\"SubscribedPlanId\\\":\\\"08dec763-2cbb-47b4-8862-ef7c18e61eec\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"efb0351d-3b08-4503-993d-383af8de41e3\\\"},{\\\"SubscribedPlanId\\\":\\\"03a75113-5b94-4083-9abc-38bf7ba38e84\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5136a095-5cf0-4aff-bec3-e84448b38ea5\\\"},{\\\"SubscribedPlanId\\\":\\\"f6ef49c3-1a30-4a87-81bb-33eee7bba192\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"6c57d4b6-3b23-47a5-9bc9-69f17b4947b3\\\"},{\\\"SubscribedPlanId\\\":\\\"f16c6e89-93cc-4fd6-b474-59b2cea0231b\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a6520331-d7d4-4276-95f5-15c0933bc757\\\"},{\\\"SubscribedPlanId\\\":\\\"eeed2477-7994-4b39-a03f-181c64c7f7fa\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bea4c11e-220a-4e6d-8eb8-8ea15d019f90\\\"},{\\\"SubscribedPlanId\\\":\\\"eaf152c0-4eeb-4f3c-8501-39ae7fe6989e\\\",\\\"ServiceInstance\\\":\\\"SCO/PROD_AMSUD0101_01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c1ec4a95-1f05-45b3-a911-aa3fa01094f5\\\"},{\\\"SubscribedPlanId\\\":\\\"dbae48d1-a0ef-497b-b857-608ffb8a0035\\\",\\\"ServiceInstance\\\":\\\"Windows/SDF\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8e229017-d77b-43d5-9305-903395523b99\\\"},{\\\"SubscribedPlanId\\\":\\\"c4031b28-43f8-42d9-b1f4-06f5b955074c\\\",\\\"ServiceInstance\\\":\\\"Bing/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0d0c0d31-fae7-41f2-b909-eaf4d7f26dba\\\"},{\\\"SubscribedPlanId\\\":\\\"b7f56b27-f5ea-45fb-8884-1a5357c41c37\\\",\\\"ServiceInstance\\\":\\\"Microsoft.ProjectBabylon/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c948ea65-2053-4a5a-8a62-9eaaaf11b522\\\"},{\\\"SubscribedPlanId\\\":\\\"a60c7542-c074-4479-af90-4af6caea7a57\\\",\\\"ServiceInstance\\\":\\\"ProjectProgramsAndPortfolios/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b21a6b06-1988-436e-a07b-51ec6d9f52ad\\\"},{\\\"SubscribedPlanId\\\":\\\"a09cb9c4-8e21-4801-8aa3-a841705b1497\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5bfe124c-bbdc-4494-8835-f1297d457d79\\\"},{\\\"SubscribedPlanId\\\":\\\"7ff00ebf-2122-4a90-a21b-2dd8d91f47d0\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"afa73018-811e-46e9-988f-f75d2b1b8430\\\"},{\\\"SubscribedPlanId\\\":\\\"7ed1f528-4e3a-4770-bbd1-fc1e8c5ed421\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"094e7854-93fc-4d55-b2c0-3ab5369ebdc1\\\"},{\\\"SubscribedPlanId\\\":\\\"7c3a406a-7181-4717-a008-00e2b758651b\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"de377cbc-0019-4ec2-b77c-3f223947e102\\\"},{\\\"SubscribedPlanId\\\":\\\"7aedce94-4e81-4a47-94fc-a18af8012419\\\",\\\"ServiceInstance\\\":\\\"SCO/PROD_AMSUD0101_01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8e9ff0ff-aa7a-4b20-83c1-2f636b600ac2\\\"},{\\\"SubscribedPlanId\\\":\\\"79a085f9-a0a5-47f8-87f4-aac406fd96e5\\\",\\\"ServiceInstance\\\":\\\"ccibotsprod/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"ded3d325-1bdc-453e-8432-5bac26d7a014\\\"},{\\\"SubscribedPlanId\\\":\\\"6bd8d315-6527-4b5e-af48-a682cf93421a\\\",\\\"ServiceInstance\\\":\\\"MicrosoftCommunicationsOnline/APAC-AU1-S1\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0feaeb32-d00e-4d66-bd5a-43b5b83db82c\\\"},{\\\"SubscribedPlanId\\\":\\\"694b4e1c-079c-4afe-9d08-f38537955130\\\",\\\"ServiceInstance\\\":\\\"OnlineService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"1fe6227d-3e01-46d0-9510-0acad4ff6e94\\\"},{\\\"SubscribedPlanId\\\":\\\"630b8d82-59e4-446a-9abe-48485d643257\\\",\\\"ServiceInstance\\\":\\\"WindowsDefenderATP/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bfc1bbd9-981b-4f71-9b82-17c35fd0e2a4\\\"},{\\\"SubscribedPlanId\\\":\\\"4352e4d1-8707-4b5f-bede-d27d1ba5ae13\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9bec7e34-c9fa-40b7-a9d1-bd6d1165c7ed\\\"},{\\\"SubscribedPlanId\\\":\\\"3fe538b9-ba8a-451d-a33d-531f60dc7176\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"28b0fa46-c39a-4188-89e2-58e979a6b014\\\"},{\\\"SubscribedPlanId\\\":\\\"36e41faa-1e78-4c8b-8453-6b3ca38ab4c1\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a1ace008-72f3-4ea0-8dac-33b3a23a2472\\\"},{\\\"SubscribedPlanId\\\":\\\"33797a9f-7ebf-4160-b3dd-01b418e7fad8\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"176a09a6-7ec5-4039-ac02-b2791c6ba793\\\"},{\\\"SubscribedPlanId\\\":\\\"29ff02e7-b9a1-4c7c-84a8-50aed2f7760d\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"199a5c09-e0ca-4e37-8f7c-b05d533e1ea2\\\"},{\\\"SubscribedPlanId\\\":\\\"22b5463b-d360-473f-80c2-be8e42afcc71\\\",\\\"ServiceInstance\\\":\\\"Chapter5FluidApp/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c4b8c31a-fb44-4c65-9837-a21f55fcabda\\\"},{\\\"SubscribedPlanId\\\":\\\"1e9fdb53-be7c-4185-8d79-17a4c14f96ea\\\",\\\"ServiceInstance\\\":\\\"WindowsUpdateforBusinessCloudExtensions/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"7bf960f6-2cd9-443a-8046-5dbff9558365\\\"},{\\\"SubscribedPlanId\\\":\\\"161014a9-b8bc-4869-85e0-38e0137851e1\\\",\\\"ServiceInstance\\\":\\\"MicrosoftKaizala/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"54fc630f-5a40-48ee-8965-af0503c1386e\\\"},{\\\"SubscribedPlanId\\\":\\\"108288ea-660d-4d4e-98ac-a651b4f33745\\\",\\\"ServiceInstance\\\":\\\"DynamicsNAV/OCN\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"39b5c996-467e-4e60-bd62-46066f572726\\\"},{\\\"SubscribedPlanId\\\":\\\"0ab4aba1-516c-4f2e-ab1d-4d251481d78b\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"276d6e8a-f056-4f70-b7e8-4fc27f79f809\\\"},{\\\"SubscribedPlanId\\\":\\\"0a80e2cd-b1e9-477d-829b-95dd228dd66a\\\",\\\"ServiceInstance\\\":\\\"LearningAppServiceInTeams/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b76fb638-6ba6-402a-b9f9-83d28acb3d86\\\"},{\\\"SubscribedPlanId\\\":\\\"02e3d1d6-4434-4d5c-88b7-a35a509cce87\\\",\\\"ServiceInstance\\\":\\\"YammerEnterprise/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a82fbf69-b4d7-49f4-83a6-915b2cf354f4\\\"},{\\\"SubscribedPlanId\\\":\\\"021ef71f-ddbf-4cfb-92fc-cc2c079d8025\\\",\\\"ServiceInstance\\\":\\\"MicrosoftPrint/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"795f6fe0-cc4d-4773-b050-5dde4dc704c9\\\"},{\\\"SubscribedPlanId\\\":\\\"020805e7-7d5f-4bb3-b898-a3b1259a976f\\\",\\\"ServiceInstance\\\":\\\"VivaSkills/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"13b6da2c-0d84-450e-9f69-a33e221387ca\\\"},{\\\"SubscribedPlanId\\\":\\\"ea16e50b-9303-4b92-9e45-0c4c4f2482be\\\",\\\"ServiceInstance\\\":\\\"MicrosoftCommunicationsOnline/APAC-AU1-S1\\\",\\\"CapabilityStatus\\\":3,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9230493Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"42a3ec34-28ba-46b6-992f-db53a675ac5b\\\"},{\\\"SubscribedPlanId\\\":\\\"e039cc95-628d-4ade-80ce-f77a46135dde\\\",\\\"ServiceInstance\\\":\\\"MicrosoftStream/NA001\\\",\\\"Capabilit"},{"key":"c","value":"6"}]</t>
-  </si>
-  <si>
-    <t>3/6/2026, 3:19:34.988 PM</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"068fdb26-0bff-4257-a389-aba213b77135"},{"key":"seq","value":"6"},{"key":"b","value":"\\\"SkuId\\\":\\\"4b60d63d-b535-4209-b2ed-91e5b0d355ea\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-06T15:19:34.9040498Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2}]},{\\\"Name\\\":\\\"Included Updated Properties\\\",\\\"OldValue\\\":null,\\\"NewValue\\\":\\\"AssignedLicense, AssignedPlan, LicenseAssignmentDetail\\\"},{\\\"Name\\\":\\\"TargetId.UserType\\\",\\\"OldValue\\\":null,\\\"NewValue\\\":\\\"Member\\\"},{\\\"Name\\\":\\\"ActorId.ServicePrincipalNames\\\",\\\"OldValue\\\":null,\\\"NewValue\\\":\\\"aeb86249-8ea3-49e2-900b-54cc8e308f85\\\"},{\\\"Name\\\":\\\"SPN\\\",\\\"OldValue\\\":null,\\\"NewValue\\\":\\\"aeb86249-8ea3-49e2-900b-54cc8e308f85\\\"}]\",\"additionalTargets\":\"\",\"additionalDetails\":\"{\\\"UserType\\\":\\\"Member\\\"}\"}"},{"key":"c","value":"6"}]</t>
-  </si>
-  <si>
-    <t>3/6/2026, 3:19:34.993 PM</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"e36c876c-0cbb-486b-a997-c6110e6b01de"},{"key":"seq","value":"1"},{"key":"b","value":"{\"targetUpdatedProperties\":\"[{\\\"Name\\\":\\\"AssignedLicense\\\",\\\"OldValue\\\":[\\\"[SkuName=PURVIEW_SUITE_FOR_BUSINESS_PREMIUM_NEW, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=4b60d63d-b535-4209-b2ed-91e5b0d355ea, DisabledPlans=[]]\\\",\\\"[SkuName=EXCHANGESTANDARD, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=4b9405b0-7788-4568-add1-99614e613b69, DisabledPlans=[]]\\\",\\\"[SkuName=AAD_PREMIUM_P2, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=84a661c4-e949-4bd2-a560-ed7766fcaf2b, DisabledPlans=[]]\\\",\\\"[SkuName=SPB, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=cbdc14ab-d96c-4c30-b9f4-6ada7cdc1d46, DisabledPlans=[]]\\\",\\\"[SkuName=Microsoft_Teams_Exploratory_Dept, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=e0dfc8b9-9531-4ec8-94b4-9fec23b05fc8, DisabledPlans=[EXCHANGE_S_STANDARD]]\\\"],\\\"NewValue\\\":[\\\"[SkuName=SPB, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=cbdc14ab-d96c-4c30-b9f4-6ada7cdc1d46, DisabledPlans=[]]\\\",\\\"[SkuName=AAD_PREMIUM_P2, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=84a661c4-e949-4bd2-a560-ed7766fcaf2b, DisabledPlans=[]]\\\",\\\"[SkuName=EXCHANGESTANDARD, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=4b9405b0-7788-4568-add1-99614e613b69, DisabledPlans=[]]\\\",\\\"[SkuName=PURVIEW_SUITE_FOR_BUSINESS_PREMIUM_NEW, AccountId=567ea528-4e82-40fa-914e-38c05fd69677, SkuId=4b60d63d-b535-4209-b2ed-91e5b0d355ea, DisabledPlans=[]]\\\"]},{\\\"Name\\\":\\\"AssignedPlan\\\",\\\"OldValue\\\":[{\\\"SubscribedPlanId\\\":\\\"020805e7-7d5f-4bb3-b898-a3b1259a976f\\\",\\\"ServiceInstance\\\":\\\"VivaSkills/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"13b6da2c-0d84-450e-9f69-a33e221387ca\\\"},{\\\"SubscribedPlanId\\\":\\\"021ef71f-ddbf-4cfb-92fc-cc2c079d8025\\\",\\\"ServiceInstance\\\":\\\"MicrosoftPrint/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"795f6fe0-cc4d-4773-b050-5dde4dc704c9\\\"},{\\\"SubscribedPlanId\\\":\\\"02e3d1d6-4434-4d5c-88b7-a35a509cce87\\\",\\\"ServiceInstance\\\":\\\"YammerEnterprise/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a82fbf69-b4d7-49f4-83a6-915b2cf354f4\\\"},{\\\"SubscribedPlanId\\\":\\\"03a75113-5b94-4083-9abc-38bf7ba38e84\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5136a095-5cf0-4aff-bec3-e84448b38ea5\\\"},{\\\"SubscribedPlanId\\\":\\\"08dec763-2cbb-47b4-8862-ef7c18e61eec\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"efb0351d-3b08-4503-993d-383af8de41e3\\\"},{\\\"SubscribedPlanId\\\":\\\"0a80e2cd-b1e9-477d-829b-95dd228dd66a\\\",\\\"ServiceInstance\\\":\\\"LearningAppServiceInTeams/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b76fb638-6ba6-402a-b9f9-83d28acb3d86\\\"},{\\\"SubscribedPlanId\\\":\\\"0ab4aba1-516c-4f2e-ab1d-4d251481d78b\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"276d6e8a-f056-4f70-b7e8-4fc27f79f809\\\"},{\\\"SubscribedPlanId\\\":\\\"0dfd484c-cc3b-4cd7-be8e-e51c1b4bc0ea\\\",\\\"ServiceInstance\\\":\\\"Sway/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a23b959c-7ce8-4e57-9140-b90eb88a9e97\\\"},{\\\"SubscribedPlanId\\\":\\\"0e6e1ecc-f9bf-4414-9e6f-1828660fd975\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"40b010bb-0b69-4654-ac5e-ba161433f4b4\\\"},{\\\"SubscribedPlanId\\\":\\\"108288ea-660d-4d4e-98ac-a651b4f33745\\\",\\\"ServiceInstance\\\":\\\"DynamicsNAV/OCN\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"39b5c996-467e-4e60-bd62-46066f572726\\\"},{\\\"SubscribedPlanId\\\":\\\"11013c80-c192-4862-bbb5-7b86a741c83a\\\",\\\"ServiceInstance\\\":\\\"WhiteboardServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b8afc642-032e-4de5-8c0a-507a7bba7e5d\\\"},{\\\"SubscribedPlanId\\\":\\\"11b27917-6674-453b-9913-cba7aba6883a\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"dcf9d2f4-772e-4434-b757-77a453cfbc02\\\"},{\\\"SubscribedPlanId\\\":\\\"161014a9-b8bc-4869-85e0-38e0137851e1\\\",\\\"ServiceInstance\\\":\\\"MicrosoftKaizala/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"54fc630f-5a40-48ee-8965-af0503c1386e\\\"},{\\\"SubscribedPlanId\\\":\\\"177b15ab-51b1-47d1-b213-f0e968822a83\\\",\\\"ServiceInstance\\\":\\\"MultiFactorService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8a256a2b-b617-496d-b51b-e76466e88db0\\\"},{\\\"SubscribedPlanId\\\":\\\"1a6d321c-ebe3-4198-8527-0d14340c3009\\\",\\\"ServiceInstance\\\":\\\"ProcessSimple/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0f9b09cb-62d1-4ff4-9129-43f4996f83f4\\\"},{\\\"SubscribedPlanId\\\":\\\"1b044c1d-0c69-4b8d-8b93-03c2ef1fd3da\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c7699d2e-19aa-44de-8edf-1736da088ca1\\\"},{\\\"SubscribedPlanId\\\":\\\"1e9fdb53-be7c-4185-8d79-17a4c14f96ea\\\",\\\"ServiceInstance\\\":\\\"WindowsUpdateforBusinessCloudExtensions/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"7bf960f6-2cd9-443a-8046-5dbff9558365\\\"},{\\\"SubscribedPlanId\\\":\\\"2287b27a-b6ec-40e6-bb03-35170aa2c846\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"41781fb2-bc02-4b7c-bd55-b576c07bb09d\\\"},{\\\"SubscribedPlanId\\\":\\\"22b5463b-d360-473f-80c2-be8e42afcc71\\\",\\\"ServiceInstance\\\":\\\"Chapter5FluidApp/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c4b8c31a-fb44-4c65-9837-a21f55fcabda\\\"},{\\\"SubscribedPlanId\\\":\\\"29ff02e7-b9a1-4c7c-84a8-50aed2f7760d\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"199a5c09-e0ca-4e37-8f7c-b05d533e1ea2\\\"},{\\\"SubscribedPlanId\\\":\\\"32b1b5b1-66f5-440a-b9ab-761ae0de5c3d\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"4de31727-a228-4ec3-a5bf-8e45b5ca48cc\\\"},{\\\"SubscribedPlanId\\\":\\\"33797a9f-7ebf-4160-b3dd-01b418e7fad8\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"176a09a6-7ec5-4039-ac02-b2791c6ba793\\\"},{\\\"SubscribedPlanId\\\":\\\"36e41faa-1e78-4c8b-8453-6b3ca38ab4c1\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a1ace008-72f3-4ea0-8dac-33b3a23a2472\\\"},{\\\"SubscribedPlanId\\\":\\\"3d063696-1e64-4da3-bf5a-c9f9acad1a63\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"6db1f1db-2b46-403f-be40-e39395f08dbb\\\"},{\\\"SubscribedPlanId\\\":\\\"3ef79a81-ae21-49b8-8fa7-dc1d795d9671\\\",\\\"ServiceInstance\\\":\\\"ProjectProgramsAndPortfolios/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a55dfd10-0864-46d9-a3cd-da5991a3e0e2\\\"},{\\\"SubscribedPlanId\\\":\\\"3fe538b9-ba8a-451d-a33d-531f60dc7176\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"28b0fa46-c39a-4188-89e2-58e979a6b014\\\"},{\\\"SubscribedPlanId\\\":\\\"42a28204-69e3-45a0-a05d-e3cab2f3a511\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"6dc145d6-95dd-4191-b9c3-185575ee6f6b\\\"},{\\\"SubscribedPlanId\\\":\\\"4352e4d1-8707-4b5f-bede-d27d1ba5ae13\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9bec7e34-c9fa-40b7-a9d1-bd6d1165c7ed\\\"},{\\\"SubscribedPlanId\\\":\\\"449a3874-a6a4-498d-905d-662cfc611bea\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"f0ff6ac6-297d-49cd-be34-6dfef97f0c28\\\"},{\\\"SubscribedPlanId\\\":\\\"4d30549f-7bcb-4a9d-94e0-cfc57bf8ae10\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9d0c4ee5-e4a1-4625-ab39-d82b619b1a34\\\"},{\\\"SubscribedPlanId\\\":\\\"529909ed-7627-4843-bb53-35"},{"key":"c","value":"6"}]</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"e36c876c-0cbb-486b-a997-c6110e6b01de"},{"key":"seq","value":"2"},{"key":"b","value":"56b852c9d9\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9aaf7827-d63c-4b61-89c3-182f06f82e5c\\\"},{\\\"SubscribedPlanId\\\":\\\"53ac6e25-a8f6-44bf-b402-9f56b8eecfd9\\\",\\\"ServiceInstance\\\":\\\"To-Do/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5e62787c-c316-451f-b873-1d05acd4d12c\\\"},{\\\"SubscribedPlanId\\\":\\\"58567403-0357-4227-8e24-d24ac70caac2\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"617b097b-4b93-4ede-83de-5f075bb5fb2f\\\"},{\\\"SubscribedPlanId\\\":\\\"5e83a7db-303f-48b4-9514-d8afa4ee812d\\\",\\\"ServiceInstance\\\":\\\"Office365InsiderRisk/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"d587c7a3-bda9-4f99-8776-9bcf59c84f75\\\"},{\\\"SubscribedPlanId\\\":\\\"60517d0d-a18e-44b4-9967-dbbb00475411\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"e26c2fcc-ab91-4a61-b35c-03cdc8dddf66\\\"},{\\\"SubscribedPlanId\\\":\\\"60f24eff-dd31-4f08-a86f-53268db26a59\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5689bec4-755d-4753-8b61-40975025187c\\\"},{\\\"SubscribedPlanId\\\":\\\"630b8d82-59e4-446a-9abe-48485d643257\\\",\\\"ServiceInstance\\\":\\\"WindowsDefenderATP/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bfc1bbd9-981b-4f71-9b82-17c35fd0e2a4\\\"},{\\\"SubscribedPlanId\\\":\\\"694b4e1c-079c-4afe-9d08-f38537955130\\\",\\\"ServiceInstance\\\":\\\"OnlineService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"1fe6227d-3e01-46d0-9510-0acad4ff6e94\\\"},{\\\"SubscribedPlanId\\\":\\\"6bd8d315-6527-4b5e-af48-a682cf93421a\\\",\\\"ServiceInstance\\\":\\\"MicrosoftCommunicationsOnline/APAC-AU1-S1\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0feaeb32-d00e-4d66-bd5a-43b5b83db82c\\\"},{\\\"SubscribedPlanId\\\":\\\"6f498fb0-aae3-4b91-abaa-8aab59767e21\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"2f442157-a11c-46b9-ae5b-6e39ff4e5849\\\"},{\\\"SubscribedPlanId\\\":\\\"6f907b14-cb0b-4a3a-9bb9-4f951739e103\\\",\\\"ServiceInstance\\\":\\\"Deskless/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8c7d2df8-86f0-4902-b2ed-a0458298f3b3\\\"},{\\\"SubscribedPlanId\\\":\\\"71ac5b1a-e1dc-4ced-ba2d-059d74e89acf\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"3efbd4ed-8958-4824-8389-1321f8730af8\\\"},{\\\"SubscribedPlanId\\\":\\\"77183285-9618-493a-aab7-221b307b5b22\\\",\\\"ServiceInstance\\\":\\\"CustomerLockbox/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"3ec18638-bd4c-4d3b-8905-479ed636b83e\\\"},{\\\"SubscribedPlanId\\\":\\\"79a085f9-a0a5-47f8-87f4-aac406fd96e5\\\",\\\"ServiceInstance\\\":\\\"ccibotsprod/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"ded3d325-1bdc-453e-8432-5bac26d7a014\\\"},{\\\"SubscribedPlanId\\\":\\\"7aedce94-4e81-4a47-94fc-a18af8012419\\\",\\\"ServiceInstance\\\":\\\"SCO/PROD_AMSUD0101_01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8e9ff0ff-aa7a-4b20-83c1-2f636b600ac2\\\"},{\\\"SubscribedPlanId\\\":\\\"7c3a406a-7181-4717-a008-00e2b758651b\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"de377cbc-0019-4ec2-b77c-3f223947e102\\\"},{\\\"SubscribedPlanId\\\":\\\"7ed1f528-4e3a-4770-bbd1-fc1e8c5ed421\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"094e7854-93fc-4d55-b2c0-3ab5369ebdc1\\\"},{\\\"SubscribedPlanId\\\":\\\"7ff00ebf-2122-4a90-a21b-2dd8d91f47d0\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"afa73018-811e-46e9-988f-f75d2b1b8430\\\"},{\\\"SubscribedPlanId\\\":\\\"83ed6518-e5d3-4cf9-a57c-b3eb1231d38f\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"d2d51368-76c9-4317-ada2-a12c004c432f\\\"},{\\\"SubscribedPlanId\\\":\\\"85ff92c3-df66-4ccc-ba0b-38683b60b371\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"33c4f319-9bdd-48d6-9c4d-410b750a4a5a\\\"},{\\\"SubscribedPlanId\\\":\\\"88ae6c56-fccc-497d-9e45-c0ea113b9406\\\",\\\"ServiceInstance\\\":\\\"PowerAppsService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"92f7a6f3-b89b-4bbd-8c30-809e6da5ad1c\\\"},{\\\"SubscribedPlanId\\\":\\\"956ea907-9a03-46cd-8699-95667e82355a\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c63d4d19-e8cb-460e-b37c-4d6c34603745\\\"},{\\\"SubscribedPlanId\\\":\\\"963ac82d-37a8-4f4c-baa4-66b1534f8353\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b1188c4c-1b36-4018-b48b-ee07604f6feb\\\"},{\\\"SubscribedPlanId\\\":\\\"9b6a0da3-ab6f-444c-9d2f-dd38db48e7c2\\\",\\\"ServiceInstance\\\":\\\"M365CommunicationCompliance/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a413a9ff-720c-4822-98ef-2f37c2a21f4c\\\"},{\\\"SubscribedPlanId\\\":\\\"9e5b8d09-b8e5-4f2c-93a0-fd7923ce9434\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"65cc641f-cccd-4643-97e0-a17e3045e541\\\"},{\\\"SubscribedPlanId\\\":\\\"a09cb9c4-8e21-4801-8aa3-a841705b1497\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5bfe124c-bbdc-4494-8835-f1297d457d79\\\"},{\\\"SubscribedPlanId\\\":\\\"a22189d7-70fa-482b-9d57-ada39f5e0872\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"eec0eb4f-6444-4f95-aba0-50c24d67f998\\\"},{\\\"SubscribedPlanId\\\":\\\"a2562c16-aca9-4316-a54b-3d8f61222c1e\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c4801e8a-cb58-4c35-aca6-f2dcc106f287\\\"},{\\\"SubscribedPlanId\\\":\\\"a48ddbe9-91e5-469c-ad84-9a44d5be8120\\\",\\\"ServiceInstance\\\":\\\"MIPExchangeSolutions/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"cd31b152-6326-4d1b-ae1b-997b625182e6\\\"},{\\\"SubscribedPlanId\\\":\\\"a507d475-c032-4d54-92a2-176f6b57256d\\\",\\\"ServiceInstance\\\":\\\"MicrosoftEndpointDLP/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"64bfac92-2b17-4482-b5e5-a0304429de3e\\\"},{\\\"SubscribedPlanId\\\":\\\"a5d43ea2-3323-489d-a579-068f683b41f7\\\",\\\"ServiceInstance\\\":\\\"ccibotsprod/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0683001c-0492-4d59-9515-d9a6426b5813\\\"},{\\\"SubscribedPlanId\\\":\\\"a60c7542-c074-4479-af90-4af6caea7a57\\\",\\\"ServiceInstance\\\":\\\"ProjectProgramsAndPortfolios/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b21a6b06-1988-436e-a07b-51ec6d9f52ad\\\"},{\\\"SubscribedPlanId\\\":\\\"a83d2db3-81e2-45ee-bf0e-c1088b24bb96\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"e95bec33-7c88-4a70-8e19-b10bd9d0c014\\\"},{\\\"SubscribedPlanId\\\":\\\"b3ae2021-9f74-4a09-9845-42accad7b182\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bed136c6-b799-4462-824d-fc045d3a9d25\\\"},{\\\"SubscribedPlanId\\\":\\\"b7b9220c-a3f0-437e-b99a-0e925b312c86\\\",\\\"ServiceInstance\\\":\\\"YammerEnterprise/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"7547a3fe-08ee-4ccb-b430-5077c5041653\\\"},{\\\"SubscribedPlanId\\\":\\\"b7f56b27-f5ea-45fb-8884-1a5357c41c37\\\",\\\"ServiceInstance\\\":\\\"Microsoft.ProjectBabylon/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTim"},{"key":"c","value":"6"}]</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"e36c876c-0cbb-486b-a997-c6110e6b01de"},{"key":"seq","value":"3"},{"key":"b","value":"estamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c948ea65-2053-4a5a-8a62-9eaaaf11b522\\\"},{\\\"SubscribedPlanId\\\":\\\"bb1ff8c5-ee94-4fb6-8303-cae3797020ad\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"f6de4823-28fa-440b-b886-4783fa86ddba\\\"},{\\\"SubscribedPlanId\\\":\\\"c4031b28-43f8-42d9-b1f4-06f5b955074c\\\",\\\"ServiceInstance\\\":\\\"Bing/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0d0c0d31-fae7-41f2-b909-eaf4d7f26dba\\\"},{\\\"SubscribedPlanId\\\":\\\"c73a8c4e-f6b6-4998-bf41-862fdea05abd\\\",\\\"ServiceInstance\\\":\\\"ProjectWorkManagement/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b737dad2-2f6c-4c65-90e3-ca563267e8b9\\\"},{\\\"SubscribedPlanId\\\":\\\"d1c57312-4814-4818-a991-38bb7429b211\\\",\\\"ServiceInstance\\\":\\\"TeamspaceAPI/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"57ff2da0-773e-42df-b2af-ffb7a2317929\\\"},{\\\"SubscribedPlanId\\\":\\\"d2f707d4-5a1a-4448-85f0-2116fe2a3a39\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9f431833-0334-42de-a7dc-70aa40db46db\\\"},{\\\"SubscribedPlanId\\\":\\\"dbae48d1-a0ef-497b-b857-608ffb8a0035\\\",\\\"ServiceInstance\\\":\\\"Windows/SDF\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8e229017-d77b-43d5-9305-903395523b99\\\"},{\\\"SubscribedPlanId\\\":\\\"dddc5824-34a0-4b85-b6b8-0fafe67a57b0\\\",\\\"ServiceInstance\\\":\\\"OfficeForms/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"159f4cd6-e380-449f-a816-af1a9ef76344\\\"},{\\\"SubscribedPlanId\\\":\\\"e039cc95-628d-4ade-80ce-f77a46135dde\\\",\\\"ServiceInstance\\\":\\\"MicrosoftStream/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"743dd19e-1ce3-4c62-a3ad-49ba8f63a2f6\\\"},{\\\"SubscribedPlanId\\\":\\\"e7733084-cf3d-4d56-9cfd-1cd9ea183052\\\",\\\"ServiceInstance\\\":\\\"Adallom/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"932ad362-64a8-4783-9106-97849a1a30b9\\\"},{\\\"SubscribedPlanId\\\":\\\"ea16e50b-9303-4b92-9e45-0c4c4f2482be\\\",\\\"ServiceInstance\\\":\\\"MicrosoftCommunicationsOnline/APAC-AU1-S1\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-02T19:56:29Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"42a3ec34-28ba-46b6-992f-db53a675ac5b\\\"},{\\\"SubscribedPlanId\\\":\\\"eaf152c0-4eeb-4f3c-8501-39ae7fe6989e\\\",\\\"ServiceInstance\\\":\\\"SCO/PROD_AMSUD0101_01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c1ec4a95-1f05-45b3-a911-aa3fa01094f5\\\"},{\\\"SubscribedPlanId\\\":\\\"eeed2477-7994-4b39-a03f-181c64c7f7fa\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bea4c11e-220a-4e6d-8eb8-8ea15d019f90\\\"},{\\\"SubscribedPlanId\\\":\\\"f039ab05-e70d-49d9-884f-22b99b2b9464\\\",\\\"ServiceInstance\\\":\\\"Adallom/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"2e2ddb96-6af9-4b1d-a3f0-d6ecfd22edb2\\\"},{\\\"SubscribedPlanId\\\":\\\"f16c6e89-93cc-4fd6-b474-59b2cea0231b\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a6520331-d7d4-4276-95f5-15c0933bc757\\\"},{\\\"SubscribedPlanId\\\":\\\"f6ef49c3-1a30-4a87-81bb-33eee7bba192\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"6c57d4b6-3b23-47a5-9bc9-69f17b4947b3\\\"}],\\\"NewValue\\\":[{\\\"SubscribedPlanId\\\":\\\"f039ab05-e70d-49d9-884f-22b99b2b9464\\\",\\\"ServiceInstance\\\":\\\"Adallom/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"2e2ddb96-6af9-4b1d-a3f0-d6ecfd22edb2\\\"},{\\\"SubscribedPlanId\\\":\\\"d2f707d4-5a1a-4448-85f0-2116fe2a3a39\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9f431833-0334-42de-a7dc-70aa40db46db\\\"},{\\\"SubscribedPlanId\\\":\\\"bb1ff8c5-ee94-4fb6-8303-cae3797020ad\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"f6de4823-28fa-440b-b886-4783fa86ddba\\\"},{\\\"SubscribedPlanId\\\":\\\"a507d475-c032-4d54-92a2-176f6b57256d\\\",\\\"ServiceInstance\\\":\\\"MicrosoftEndpointDLP/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"64bfac92-2b17-4482-b5e5-a0304429de3e\\\"},{\\\"SubscribedPlanId\\\":\\\"a48ddbe9-91e5-469c-ad84-9a44d5be8120\\\",\\\"ServiceInstance\\\":\\\"MIPExchangeSolutions/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"cd31b152-6326-4d1b-ae1b-997b625182e6\\\"},{\\\"SubscribedPlanId\\\":\\\"a2562c16-aca9-4316-a54b-3d8f61222c1e\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c4801e8a-cb58-4c35-aca6-f2dcc106f287\\\"},{\\\"SubscribedPlanId\\\":\\\"9e5b8d09-b8e5-4f2c-93a0-fd7923ce9434\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"65cc641f-cccd-4643-97e0-a17e3045e541\\\"},{\\\"SubscribedPlanId\\\":\\\"9b6a0da3-ab6f-444c-9d2f-dd38db48e7c2\\\",\\\"ServiceInstance\\\":\\\"M365CommunicationCompliance/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a413a9ff-720c-4822-98ef-2f37c2a21f4c\\\"},{\\\"SubscribedPlanId\\\":\\\"963ac82d-37a8-4f4c-baa4-66b1534f8353\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b1188c4c-1b36-4018-b48b-ee07604f6feb\\\"},{\\\"SubscribedPlanId\\\":\\\"83ed6518-e5d3-4cf9-a57c-b3eb1231d38f\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"d2d51368-76c9-4317-ada2-a12c004c432f\\\"},{\\\"SubscribedPlanId\\\":\\\"77183285-9618-493a-aab7-221b307b5b22\\\",\\\"ServiceInstance\\\":\\\"CustomerLockbox/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"3ec18638-bd4c-4d3b-8905-479ed636b83e\\\"},{\\\"SubscribedPlanId\\\":\\\"6f498fb0-aae3-4b91-abaa-8aab59767e21\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"2f442157-a11c-46b9-ae5b-6e39ff4e5849\\\"},{\\\"SubscribedPlanId\\\":\\\"60f24eff-dd31-4f08-a86f-53268db26a59\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5689bec4-755d-4753-8b61-40975025187c\\\"},{\\\"SubscribedPlanId\\\":\\\"60517d0d-a18e-44b4-9967-dbbb00475411\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"e26c2fcc-ab91-4a61-b35c-03cdc8dddf66\\\"},{\\\"SubscribedPlanId\\\":\\\"5e83a7db-303f-48b4-9514-d8afa4ee812d\\\",\\\"ServiceInstance\\\":\\\"Office365InsiderRisk/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"d587c7a3-bda9-4f99-8776-9bcf59c84f75\\\"},{\\\"SubscribedPlanId\\\":\\\"58567403-0357-4227-8e24-d24ac70caac2\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"617b097b-4b93-4ede-83de-5f075bb5fb2f\\\"},{\\\"SubscribedPlanId\\\":\\\"529909ed-7627-4843-bb53-3556b852c9d9\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9270494Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9aaf7827-d63c-4b61-89c3-182f06f82e5c\\\"},{\\\"SubscribedPlanId\\\":\\\"4d30549f-7bcb-4a9d-94e0-cfc57bf8ae10\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9d0c4ee5-e4a1-4625-ab39-d82b619b1a34\\\"},{\\\"SubscribedPlanId\\\":\\\"42a28204-69e3-45a0-a05d-e3cab2f3a511\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"6dc145d6-95dd-4191-b9c3-185575ee6f6b\\\"},{\\\"SubscribedPlanId\\\":\\\"3d063696-1e64-4da3-bf5a-c9f9acad1a63\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"6db1f1db-2b46-403f-be40-e39395f08dbb\\\"},{\\\"SubscribedPla"},{"key":"c","value":"6"}]</t>
-  </si>
-  <si>
-    <t>3/6/2026, 3:19:34.994 PM</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"e36c876c-0cbb-486b-a997-c6110e6b01de"},{"key":"seq","value":"4"},{"key":"b","value":"nId\\\":\\\"32b1b5b1-66f5-440a-b9ab-761ae0de5c3d\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"4de31727-a228-4ec3-a5bf-8e45b5ca48cc\\\"},{\\\"SubscribedPlanId\\\":\\\"08dec763-2cbb-47b4-8862-ef7c18e61eec\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"efb0351d-3b08-4503-993d-383af8de41e3\\\"},{\\\"SubscribedPlanId\\\":\\\"03a75113-5b94-4083-9abc-38bf7ba38e84\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:24:48Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5136a095-5cf0-4aff-bec3-e84448b38ea5\\\"},{\\\"SubscribedPlanId\\\":\\\"f6ef49c3-1a30-4a87-81bb-33eee7bba192\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"6c57d4b6-3b23-47a5-9bc9-69f17b4947b3\\\"},{\\\"SubscribedPlanId\\\":\\\"f16c6e89-93cc-4fd6-b474-59b2cea0231b\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a6520331-d7d4-4276-95f5-15c0933bc757\\\"},{\\\"SubscribedPlanId\\\":\\\"eeed2477-7994-4b39-a03f-181c64c7f7fa\\\",\\\"ServiceInstance\\\":\\\"RMSOnline/AP\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bea4c11e-220a-4e6d-8eb8-8ea15d019f90\\\"},{\\\"SubscribedPlanId\\\":\\\"eaf152c0-4eeb-4f3c-8501-39ae7fe6989e\\\",\\\"ServiceInstance\\\":\\\"SCO/PROD_AMSUD0101_01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c1ec4a95-1f05-45b3-a911-aa3fa01094f5\\\"},{\\\"SubscribedPlanId\\\":\\\"dbae48d1-a0ef-497b-b857-608ffb8a0035\\\",\\\"ServiceInstance\\\":\\\"Windows/SDF\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8e229017-d77b-43d5-9305-903395523b99\\\"},{\\\"SubscribedPlanId\\\":\\\"c4031b28-43f8-42d9-b1f4-06f5b955074c\\\",\\\"ServiceInstance\\\":\\\"Bing/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0d0c0d31-fae7-41f2-b909-eaf4d7f26dba\\\"},{\\\"SubscribedPlanId\\\":\\\"b7f56b27-f5ea-45fb-8884-1a5357c41c37\\\",\\\"ServiceInstance\\\":\\\"Microsoft.ProjectBabylon/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c948ea65-2053-4a5a-8a62-9eaaaf11b522\\\"},{\\\"SubscribedPlanId\\\":\\\"a60c7542-c074-4479-af90-4af6caea7a57\\\",\\\"ServiceInstance\\\":\\\"ProjectProgramsAndPortfolios/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b21a6b06-1988-436e-a07b-51ec6d9f52ad\\\"},{\\\"SubscribedPlanId\\\":\\\"a09cb9c4-8e21-4801-8aa3-a841705b1497\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5bfe124c-bbdc-4494-8835-f1297d457d79\\\"},{\\\"SubscribedPlanId\\\":\\\"7ff00ebf-2122-4a90-a21b-2dd8d91f47d0\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"afa73018-811e-46e9-988f-f75d2b1b8430\\\"},{\\\"SubscribedPlanId\\\":\\\"7ed1f528-4e3a-4770-bbd1-fc1e8c5ed421\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"094e7854-93fc-4d55-b2c0-3ab5369ebdc1\\\"},{\\\"SubscribedPlanId\\\":\\\"7c3a406a-7181-4717-a008-00e2b758651b\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"de377cbc-0019-4ec2-b77c-3f223947e102\\\"},{\\\"SubscribedPlanId\\\":\\\"7aedce94-4e81-4a47-94fc-a18af8012419\\\",\\\"ServiceInstance\\\":\\\"SCO/PROD_AMSUD0101_01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8e9ff0ff-aa7a-4b20-83c1-2f636b600ac2\\\"},{\\\"SubscribedPlanId\\\":\\\"79a085f9-a0a5-47f8-87f4-aac406fd96e5\\\",\\\"ServiceInstance\\\":\\\"ccibotsprod/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"ded3d325-1bdc-453e-8432-5bac26d7a014\\\"},{\\\"SubscribedPlanId\\\":\\\"6bd8d315-6527-4b5e-af48-a682cf93421a\\\",\\\"ServiceInstance\\\":\\\"MicrosoftCommunicationsOnline/APAC-AU1-S1\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0feaeb32-d00e-4d66-bd5a-43b5b83db82c\\\"},{\\\"SubscribedPlanId\\\":\\\"694b4e1c-079c-4afe-9d08-f38537955130\\\",\\\"ServiceInstance\\\":\\\"OnlineService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"1fe6227d-3e01-46d0-9510-0acad4ff6e94\\\"},{\\\"SubscribedPlanId\\\":\\\"630b8d82-59e4-446a-9abe-48485d643257\\\",\\\"ServiceInstance\\\":\\\"WindowsDefenderATP/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bfc1bbd9-981b-4f71-9b82-17c35fd0e2a4\\\"},{\\\"SubscribedPlanId\\\":\\\"4352e4d1-8707-4b5f-bede-d27d1ba5ae13\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"9bec7e34-c9fa-40b7-a9d1-bd6d1165c7ed\\\"},{\\\"SubscribedPlanId\\\":\\\"3fe538b9-ba8a-451d-a33d-531f60dc7176\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"28b0fa46-c39a-4188-89e2-58e979a6b014\\\"},{\\\"SubscribedPlanId\\\":\\\"36e41faa-1e78-4c8b-8453-6b3ca38ab4c1\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a1ace008-72f3-4ea0-8dac-33b3a23a2472\\\"},{\\\"SubscribedPlanId\\\":\\\"33797a9f-7ebf-4160-b3dd-01b418e7fad8\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"176a09a6-7ec5-4039-ac02-b2791c6ba793\\\"},{\\\"SubscribedPlanId\\\":\\\"29ff02e7-b9a1-4c7c-84a8-50aed2f7760d\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"199a5c09-e0ca-4e37-8f7c-b05d533e1ea2\\\"},{\\\"SubscribedPlanId\\\":\\\"22b5463b-d360-473f-80c2-be8e42afcc71\\\",\\\"ServiceInstance\\\":\\\"Chapter5FluidApp/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c4b8c31a-fb44-4c65-9837-a21f55fcabda\\\"},{\\\"SubscribedPlanId\\\":\\\"1e9fdb53-be7c-4185-8d79-17a4c14f96ea\\\",\\\"ServiceInstance\\\":\\\"WindowsUpdateforBusinessCloudExtensions/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"7bf960f6-2cd9-443a-8046-5dbff9558365\\\"},{\\\"SubscribedPlanId\\\":\\\"161014a9-b8bc-4869-85e0-38e0137851e1\\\",\\\"ServiceInstance\\\":\\\"MicrosoftKaizala/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"54fc630f-5a40-48ee-8965-af0503c1386e\\\"},{\\\"SubscribedPlanId\\\":\\\"108288ea-660d-4d4e-98ac-a651b4f33745\\\",\\\"ServiceInstance\\\":\\\"DynamicsNAV/OCN\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"39b5c996-467e-4e60-bd62-46066f572726\\\"},{\\\"SubscribedPlanId\\\":\\\"0ab4aba1-516c-4f2e-ab1d-4d251481d78b\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"276d6e8a-f056-4f70-b7e8-4fc27f79f809\\\"},{\\\"SubscribedPlanId\\\":\\\"0a80e2cd-b1e9-477d-829b-95dd228dd66a\\\",\\\"ServiceInstance\\\":\\\"LearningAppServiceInTeams/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b76fb638-6ba6-402a-b9f9-83d28acb3d86\\\"},{\\\"SubscribedPlanId\\\":\\\"02e3d1d6-4434-4d5c-88b7-a35a509cce87\\\",\\\"ServiceInstance\\\":\\\"YammerEnterprise/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a82fbf69-b4d7-49f4-83a6-915b2cf354f4\\\"},{\\\"SubscribedPlanId\\\":\\\"021ef71f-ddbf-4cfb-92fc-cc2c079d8025\\\",\\\"ServiceInstance\\\":\\\"MicrosoftPrint/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"795f6fe0-cc4d-4773-b050-5dde4dc704c9\\\"},{\\\"SubscribedPlanId\\\":\\\"020805e7-7d5f-4bb3-b898-a3b1259a976f\\\",\\\"ServiceInstance\\\":\\\"VivaSkills/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-01T05:19:54Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"13b6da2c-0d84-450e-9f69-a33e221387ca\\\"},{\\\"SubscribedPlanId\\\":\\\"ea16e50b-9303-4b92-9e45-0c4c4f2482be\\\",\\\"ServiceInstance\\\":\\\"MicrosoftCommunicationsOnline/APAC-AU1-S1\\\",\\\"CapabilityStatus\\\":3,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9230493Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"42a3ec34-28ba-46b6-992f-db53a675ac5b\\\"},{\\\"SubscribedPlanId\\\":\\\"e039cc95-628d-4ade-80ce-f77a46135dde\\\",\\\"ServiceInstance\\\":\\\"MicrosoftStream/NA001\\\",\\\"Capabilit"},{"key":"c","value":"6"}]</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"e36c876c-0cbb-486b-a997-c6110e6b01de"},{"key":"seq","value":"6"},{"key":"b","value":"\\\"SkuId\\\":\\\"4b60d63d-b535-4209-b2ed-91e5b0d355ea\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-06T15:19:34.9040498Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2}]},{\\\"Name\\\":\\\"Included Updated Properties\\\",\\\"OldValue\\\":null,\\\"NewValue\\\":\\\"AssignedLicense, AssignedPlan, LicenseAssignmentDetail\\\"},{\\\"Name\\\":\\\"TargetId.UserType\\\",\\\"OldValue\\\":null,\\\"NewValue\\\":\\\"Member\\\"},{\\\"Name\\\":\\\"ActorId.ServicePrincipalNames\\\",\\\"OldValue\\\":null,\\\"NewValue\\\":\\\"aeb86249-8ea3-49e2-900b-54cc8e308f85\\\"},{\\\"Name\\\":\\\"SPN\\\",\\\"OldValue\\\":null,\\\"NewValue\\\":\\\"aeb86249-8ea3-49e2-900b-54cc8e308f85\\\"}]\",\"additionalTargets\":\"{\\\"AssignedSkuId\\\":[\\\"cbdc14ab-d96c-4c30-b9f4-6ada7cdc1d46\\\",\\\"84a661c4-e949-4bd2-a560-ed7766fcaf2b\\\",\\\"4b9405b0-7788-4568-add1-99614e613b69\\\",\\\"4b60d63d-b535-4209-b2ed-91e5b0d355ea\\\"]}\",\"additionalDetails\":\"{}\"}"},{"key":"c","value":"6"}]</t>
-  </si>
-  <si>
-    <t>[{"key":"id","value":"e36c876c-0cbb-486b-a997-c6110e6b01de"},{"key":"seq","value":"5"},{"key":"b","value":"yStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9260535Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"743dd19e-1ce3-4c62-a3ad-49ba8f63a2f6\\\"},{\\\"SubscribedPlanId\\\":\\\"dddc5824-34a0-4b85-b6b8-0fafe67a57b0\\\",\\\"ServiceInstance\\\":\\\"OfficeForms/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9260535Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"159f4cd6-e380-449f-a816-af1a9ef76344\\\"},{\\\"SubscribedPlanId\\\":\\\"d1c57312-4814-4818-a991-38bb7429b211\\\",\\\"ServiceInstance\\\":\\\"TeamspaceAPI/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9260535Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"57ff2da0-773e-42df-b2af-ffb7a2317929\\\"},{\\\"SubscribedPlanId\\\":\\\"c73a8c4e-f6b6-4998-bf41-862fdea05abd\\\",\\\"ServiceInstance\\\":\\\"ProjectWorkManagement/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9270494Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b737dad2-2f6c-4c65-90e3-ca563267e8b9\\\"},{\\\"SubscribedPlanId\\\":\\\"b7b9220c-a3f0-437e-b99a-0e925b312c86\\\",\\\"ServiceInstance\\\":\\\"YammerEnterprise/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9260535Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"7547a3fe-08ee-4ccb-b430-5077c5041653\\\"},{\\\"SubscribedPlanId\\\":\\\"b3ae2021-9f74-4a09-9845-42accad7b182\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":3,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9240496Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"bed136c6-b799-4462-824d-fc045d3a9d25\\\"},{\\\"SubscribedPlanId\\\":\\\"a83d2db3-81e2-45ee-bf0e-c1088b24bb96\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9260535Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"e95bec33-7c88-4a70-8e19-b10bd9d0c014\\\"},{\\\"SubscribedPlanId\\\":\\\"a5d43ea2-3323-489d-a579-068f683b41f7\\\",\\\"ServiceInstance\\\":\\\"ccibotsprod/NA001\\\",\\\"CapabilityStatus\\\":3,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9220495Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0683001c-0492-4d59-9515-d9a6426b5813\\\"},{\\\"SubscribedPlanId\\\":\\\"956ea907-9a03-46cd-8699-95667e82355a\\\",\\\"ServiceInstance\\\":\\\"MicrosoftOffice/NorthAmerica9\\\",\\\"CapabilityStatus\\\":3,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9230493Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c63d4d19-e8cb-460e-b37c-4d6c34603745\\\"},{\\\"SubscribedPlanId\\\":\\\"88ae6c56-fccc-497d-9e45-c0ea113b9406\\\",\\\"ServiceInstance\\\":\\\"PowerAppsService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9270494Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"92f7a6f3-b89b-4bbd-8c30-809e6da5ad1c\\\"},{\\\"SubscribedPlanId\\\":\\\"85ff92c3-df66-4ccc-ba0b-38683b60b371\\\",\\\"ServiceInstance\\\":\\\"exchange/ausp300-002-01\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9250496Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"33c4f319-9bdd-48d6-9c4d-410b750a4a5a\\\"},{\\\"SubscribedPlanId\\\":\\\"71ac5b1a-e1dc-4ced-ba2d-059d74e89acf\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9240496Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"3efbd4ed-8958-4824-8389-1321f8730af8\\\"},{\\\"SubscribedPlanId\\\":\\\"6f907b14-cb0b-4a3a-9bb9-4f951739e103\\\",\\\"ServiceInstance\\\":\\\"Deskless/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9250496Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8c7d2df8-86f0-4902-b2ed-a0458298f3b3\\\"},{\\\"SubscribedPlanId\\\":\\\"53ac6e25-a8f6-44bf-b402-9f56b8eecfd9\\\",\\\"ServiceInstance\\\":\\\"To-Do/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9250496Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"5e62787c-c316-451f-b873-1d05acd4d12c\\\"},{\\\"SubscribedPlanId\\\":\\\"449a3874-a6a4-498d-905d-662cfc611bea\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9240496Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"f0ff6ac6-297d-49cd-be34-6dfef97f0c28\\\"},{\\\"SubscribedPlanId\\\":\\\"3ef79a81-ae21-49b8-8fa7-dc1d795d9671\\\",\\\"ServiceInstance\\\":\\\"ProjectProgramsAndPortfolios/NA001\\\",\\\"CapabilityStatus\\\":3,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9210495Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a55dfd10-0864-46d9-a3cd-da5991a3e0e2\\\"},{\\\"SubscribedPlanId\\\":\\\"1b044c1d-0c69-4b8d-8b93-03c2ef1fd3da\\\",\\\"ServiceInstance\\\":\\\"SharePoint/AUS-106-0013\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9260535Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"c7699d2e-19aa-44de-8edf-1736da088ca1\\\"},{\\\"SubscribedPlanId\\\":\\\"1a6d321c-ebe3-4198-8527-0d14340c3009\\\",\\\"ServiceInstance\\\":\\\"ProcessSimple/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9270494Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"0f9b09cb-62d1-4ff4-9129-43f4996f83f4\\\"},{\\\"SubscribedPlanId\\\":\\\"11b27917-6674-453b-9913-cba7aba6883a\\\",\\\"ServiceInstance\\\":\\\"MixedRealityCollaborationServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9240496Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"dcf9d2f4-772e-4434-b757-77a453cfbc02\\\"},{\\\"SubscribedPlanId\\\":\\\"11013c80-c192-4862-bbb5-7b86a741c83a\\\",\\\"ServiceInstance\\\":\\\"WhiteboardServices/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9250496Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"b8afc642-032e-4de5-8c0a-507a7bba7e5d\\\"},{\\\"SubscribedPlanId\\\":\\\"0e6e1ecc-f9bf-4414-9e6f-1828660fd975\\\",\\\"ServiceInstance\\\":\\\"CRM/OCE01\\\",\\\"CapabilityStatus\\\":3,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9210495Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"40b010bb-0b69-4654-ac5e-ba161433f4b4\\\"},{\\\"SubscribedPlanId\\\":\\\"0dfd484c-cc3b-4cd7-be8e-e51c1b4bc0ea\\\",\\\"ServiceInstance\\\":\\\"Sway/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-03-06T15:19:34.9260535Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"a23b959c-7ce8-4e57-9140-b90eb88a9e97\\\"},{\\\"SubscribedPlanId\\\":\\\"e7733084-cf3d-4d56-9cfd-1cd9ea183052\\\",\\\"ServiceInstance\\\":\\\"Adallom/*\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"932ad362-64a8-4783-9106-97849a1a30b9\\\"},{\\\"SubscribedPlanId\\\":\\\"a22189d7-70fa-482b-9d57-ada39f5e0872\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"eec0eb4f-6444-4f95-aba0-50c24d67f998\\\"},{\\\"SubscribedPlanId\\\":\\\"2287b27a-b6ec-40e6-bb03-35170aa2c846\\\",\\\"ServiceInstance\\\":\\\"AADPremiumService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"41781fb2-bc02-4b7c-bd55-b576c07bb09d\\\"},{\\\"SubscribedPlanId\\\":\\\"177b15ab-51b1-47d1-b213-f0e968822a83\\\",\\\"ServiceInstance\\\":\\\"MultiFactorService/NA001\\\",\\\"CapabilityStatus\\\":0,\\\"AssignedTimestamp\\\":\\\"2026-02-01T21:52:35Z\\\",\\\"InitialState\\\":null,\\\"Capability\\\":null,\\\"ServicePlanId\\\":\\\"8a256a2b-b617-496d-b51b-e76466e88db0\\\"}]},{\\\"Name\\\":\\\"LicenseAssignmentDetail\\\",\\\"OldValue\\\":[{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"4b60d63d-b535-4209-b2ed-91e5b0d355ea\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:24:48.4047537Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"4b9405b0-7788-4568-add1-99614e613b69\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:24:48.4047537Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"84a661c4-e949-4bd2-a560-ed7766fcaf2b\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:24:48.4047537Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"cbdc14ab-d96c-4c30-b9f4-6ada7cdc1d46\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:24:48.4047537Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"e0dfc8b9-9531-4ec8-94b4-9fec23b05fc8\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-01T05:24:48.403751Z\\\",\\\"DisabledPlans\\\":[\\\"9aaf7827-d63c-4b61-89c3-182f06f82e5c\\\"],\\\"EncodingVersion\\\":2}],\\\"NewValue\\\":[{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"cbdc14ab-d96c-4c30-b9f4-6ada7cdc1d46\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-06T15:19:34.9040498Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"84a661c4-e949-4bd2-a560-ed7766fcaf2b\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-06T15:19:34.9040498Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\",\\\"SkuId\\\":\\\"4b9405b0-7788-4568-add1-99614e613b69\\\",\\\"Error\\\":0,\\\"StatusUpdateTimestamp\\\":\\\"2026-03-06T15:19:34.9040498Z\\\",\\\"DisabledPlans\\\":[],\\\"EncodingVersion\\\":2},{\\\"ReferenceObjectId\\\":\\\"9ebb7bc1-ad39-486e-9bf5-056f352fed91\\\",\\\"Status\\\":0,\\\"AccountId\\\":\\\"567ea528-4e82-40fa-914e-38c05fd69677\\\","},{"key":"c","value":"6"}]</t>
-  </si>
-  <si>
-    <t>3/7/2026, 12:25:42.360 AM</t>
-  </si>
-  <si>
-    <t>[{"id":"9ebb7bc1-ad39-486e-9bf5-056f352fed91","displayName":null,"type":"User","userPrincipalName":"donald.anderson@wdlabs.com.au","modifiedProperties":[{"displayName":"StrongAuthenticationPhoneAppDetail","oldValue":"[{\"DeviceName\":\"NO_DEVICE\",\"DeviceToken\":\"NO_DEVICE_TOKEN\",\"DeviceTag\":\"SoftwareTokenActivated\",\"PhoneAppVersion\":\"NO_PHONE_APP_VERSION\",\"OathTokenTimeDrift\":0,\"DeviceId\":\"00000000-0000-0000-0000-000000000000\",\"Id\":\"1378ded7-887e-417d-9f8c-0535c94eae5b\",\"TimeInterval\":0,\"AuthenticationType\":2,\"NotificationType\":1,\"LastAuthenticatedTimestamp\":\"2026-03-05T09:54:25.186239Z\",\"AuthenticatorFlavor\":\"Authenticator\",\"HashFunction\":\"hmacsha1\",\"TenantDeviceId\":null,\"SecuredPartitionId\":20102,\"SecuredKeyId\":7}]","newValue":"[{\"DeviceName\":\"NO_DEVICE\",\"DeviceToken\":\"NO_DEVICE_TOKEN\",\"DeviceTag\":\"SoftwareTokenActivated\",\"PhoneAppVersion\":\"NO_PHONE_APP_VERSION\",\"OathTokenTimeDrift\":0,\"DeviceId\":\"00000000-0000-0000-0000-000000000000\",\"Id\":\"1378ded7-887e-417d-9f8c-0535c94eae5b\",\"TimeInterval\":0,\"AuthenticationType\":2,\"NotificationType\":1,\"LastAuthenticatedTimestamp\":\"2026-03-07T00:25:42.2541002Z\",\"AuthenticatorFlavor\":\"Authenticator\",\"HashFunction\":\"hmacsha1\",\"TenantDeviceId\":null,\"SecuredPartitionId\":20102,\"SecuredKeyId\":7}]"},{"displayName":"Included Updated Properties","oldValue":null,"newValue":"\"StrongAuthenticationPhoneAppDetail\""},{"displayName":"TargetId.UserType","oldValue":null,"newValue":"\"Member\""},{"displayName":"ActorId.ServicePrincipalNames","oldValue":null,"newValue":"\"b5a60e17-278b-4c92-a4e2-b9262e66bb28\""},{"displayName":"SPN","oldValue":null,"newValue":"\"b5a60e17-278b-4c92-a4e2-b9262e66bb28\""}],"administrativeUnits":[],"agentType":"notAgentic"}]</t>
-  </si>
-  <si>
-    <t>3/7/2026, 2:27:32.070 AM</t>
-  </si>
-  <si>
-    <t>[{"id":"9ebb7bc1-ad39-486e-9bf5-056f352fed91","displayName":null,"type":"User","userPrincipalName":"donald.anderson@wdlabs.com.au","modifiedProperties":[{"displayName":"StrongAuthenticationPhoneAppDetail","oldValue":"[{\"DeviceName\":\"NO_DEVICE\",\"DeviceToken\":\"NO_DEVICE_TOKEN\",\"DeviceTag\":\"SoftwareTokenActivated\",\"PhoneAppVersion\":\"NO_PHONE_APP_VERSION\",\"OathTokenTimeDrift\":0,\"DeviceId\":\"00000000-0000-0000-0000-000000000000\",\"Id\":\"1378ded7-887e-417d-9f8c-0535c94eae5b\",\"TimeInterval\":0,\"AuthenticationType\":2,\"NotificationType\":1,\"LastAuthenticatedTimestamp\":\"2026-03-07T00:25:42.2541002Z\",\"AuthenticatorFlavor\":\"Authenticator\",\"HashFunction\":\"hmacsha1\",\"TenantDeviceId\":null,\"SecuredPartitionId\":20102,\"SecuredKeyId\":7}]","newValue":"[{\"DeviceName\":\"NO_DEVICE\",\"DeviceToken\":\"NO_DEVICE_TOKEN\",\"DeviceTag\":\"SoftwareTokenActivated\",\"PhoneAppVersion\":\"NO_PHONE_APP_VERSION\",\"OathTokenTimeDrift\":-1,\"DeviceId\":\"00000000-0000-0000-0000-000000000000\",\"Id\":\"1378ded7-887e-417d-9f8c-0535c94eae5b\",\"TimeInterval\":0,\"AuthenticationType\":2,\"NotificationType\":1,\"LastAuthenticatedTimestamp\":\"2026-03-07T00:25:42.2541002Z\",\"AuthenticatorFlavor\":\"Authenticator\",\"HashFunction\":\"hmacsha1\",\"TenantDeviceId\":null,\"SecuredPartitionId\":20102,\"SecuredKeyId\":7}]"},{"displayName":"Included Updated Properties","oldValue":null,"newValue":"\"StrongAuthenticationPhoneAppDetail\""},{"displayName":"TargetId.UserType","oldValue":null,"newValue":"\"Member\""},{"displayName":"ActorId.ServicePrincipalNames","oldValue":null,"newValue":"\"b5a60e17-278b-4c92-a4e2-b9262e66bb28\""},{"displayName":"SPN","oldValue":null,"newValue":"\"b5a60e17-278b-4c92-a4e2-b9262e66bb28\""}],"administrativeUnits":[],"agentType":"notAgentic"}]</t>
-  </si>
-  <si>
-    <t>3/7/2026, 2:31:18.375 AM</t>
-  </si>
-  <si>
-    <t>[{"id":"9ebb7bc1-ad39-486e-9bf5-056f352fed91","displayName":null,"type":"User","userPrincipalName":"donald.anderson@wdlabs.com.au","modifiedProperties":[{"displayName":"StrongAuthenticationPhoneAppDetail","oldValue":"[{\"DeviceName\":\"NO_DEVICE\",\"DeviceToken\":\"NO_DEVICE_TOKEN\",\"DeviceTag\":\"SoftwareTokenActivated\",\"PhoneAppVersion\":\"NO_PHONE_APP_VERSION\",\"OathTokenTimeDrift\":-1,\"DeviceId\":\"00000000-0000-0000-0000-000000000000\",\"Id\":\"1378ded7-887e-417d-9f8c-0535c94eae5b\",\"TimeInterval\":0,\"AuthenticationType\":2,\"NotificationType\":1,\"LastAuthenticatedTimestamp\":\"2026-03-07T00:25:42.2541002Z\",\"AuthenticatorFlavor\":\"Authenticator\",\"HashFunction\":\"hmacsha1\",\"TenantDeviceId\":null,\"SecuredPartitionId\":20102,\"SecuredKeyId\":7}]","newValue":"[{\"DeviceName\":\"NO_DEVICE\",\"DeviceToken\":\"NO_DEVICE_TOKEN\",\"DeviceTag\":\"SoftwareTokenActivated\",\"PhoneAppVersion\":\"NO_PHONE_APP_VERSION\",\"OathTokenTimeDrift\":0,\"DeviceId\":\"00000000-0000-0000-0000-000000000000\",\"Id\":\"1378ded7-887e-417d-9f8c-0535c94eae5b\",\"TimeInterval\":0,\"AuthenticationType\":2,\"NotificationType\":1,\"LastAuthenticatedTimestamp\":\"2026-03-07T00:25:42.2541002Z\",\"AuthenticatorFlavor\":\"Authenticator\",\"HashFunction\":\"hmacsha1\",\"TenantDeviceId\":null,\"SecuredPartitionId\":20102,\"SecuredKeyId\":7}]"},{"displayName":"Included Updated Properties","oldValue":null,"newValue":"\"StrongAuthenticationPhoneAppDetail\""},{"displayName":"TargetId.UserType","oldValue":null,"newValue":"\"Member\""}],"administrativeUnits":[],"agentType":"notAgentic"}]</t>
-  </si>
-  <si>
-    <t>3/10/2026, 9:29:17.771 AM</t>
-  </si>
-  <si>
-    <t>[{"id":"9ebb7bc1-ad39-486e-9bf5-056f352fed91","displayName":null,"type":"User","userPrincipalName":"donald.anderson@wdlabs.com.au","modifiedProperties":[{"displayName":"StrongAuthenticationPhoneAppDetail","oldValue":"[{\"DeviceName\":\"NO_DEVICE\",\"DeviceToken\":\"NO_DEVICE_TOKEN\",\"DeviceTag\":\"SoftwareTokenActivated\",\"PhoneAppVersion\":\"NO_PHONE_APP_VERSION\",\"OathTokenTimeDrift\":0,\"DeviceId\":\"00000000-0000-0000-0000-000000000000\",\"Id\":\"1378ded7-887e-417d-9f8c-0535c94eae5b\",\"TimeInterval\":0,\"AuthenticationType\":2,\"NotificationType\":1,\"LastAuthenticatedTimestamp\":\"2026-03-07T00:25:42.2541002Z\",\"AuthenticatorFlavor\":\"Authenticator\",\"HashFunction\":\"hmacsha1\",\"TenantDeviceId\":null,\"SecuredPartitionId\":20102,\"SecuredKeyId\":7}]","newValue":"[{\"DeviceName\":\"NO_DEVICE\",\"DeviceToken\":\"NO_DEVICE_TOKEN\",\"DeviceTag\":\"SoftwareTokenActivated\",\"PhoneAppVersion\":\"NO_PHONE_APP_VERSION\",\"OathTokenTimeDrift\":0,\"DeviceId\":\"00000000-0000-0000-0000-000000000000\",\"Id\":\"1378ded7-887e-417d-9f8c-0535c94eae5b\",\"TimeInterval\":0,\"AuthenticationType\":2,\"NotificationType\":1,\"LastAuthenticatedTimestamp\":\"2026-03-10T09:29:17.6564412Z\",\"AuthenticatorFlavor\":\"Authenticator\",\"HashFunction\":\"hmacsha1\",\"TenantDeviceId\":null,\"SecuredPartitionId\":20102,\"SecuredKeyId\":7}]"},{"displayName":"Included Updated Properties","oldValue":null,"newValue":"\"StrongAuthenticationPhoneAppDetail\""},{"displayName":"TargetId.UserType","oldValue":null,"newValue":"\"Member\""}],"administrativeUnits":[],"agentType":"notAgentic"}]</t>
-  </si>
-  <si>
     <t>ipAddress</t>
   </si>
   <si>
@@ -2179,9 +2011,6 @@
     <t>Remediation Actions below</t>
   </si>
   <si>
-    <t>Threat Actor Activity</t>
-  </si>
-  <si>
     <t>3/15/2026, 3:07:37.343 PM</t>
   </si>
   <si>
@@ -2288,13 +2117,21 @@
   </si>
   <si>
     <t>Naomi reported suspicious email to Head Office Admin.</t>
+  </si>
+  <si>
+    <t>AuditLogs
+| where TargetResources has "donald"
+| where Category in ("UserManagement", "AuthenticationMethod")
+   or OperationName has_any ("password", "MFA", "authentication method", "strong authentication", "security info")
+| project TimeGenerated, OperationName, InitiatedBy, TargetResources, Result, AdditionalDetails
+| order by TimeGenerated asc</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2484,6 +2321,12 @@
     </font>
     <font>
       <u/>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -2868,7 +2711,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2886,7 +2729,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="19" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="22" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -2917,6 +2759,12 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3482,162 +3330,162 @@
   <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.140625" style="14" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.140625" style="13" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="39.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="148.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="106.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
+        <v>629</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>601</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>602</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="19" t="s">
+        <v>630</v>
+      </c>
+      <c r="B2" t="s">
+        <v>605</v>
+      </c>
+      <c r="C2" t="s">
+        <v>692</v>
+      </c>
+      <c r="D2" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="19"/>
+      <c r="B3" t="s">
+        <v>606</v>
+      </c>
+      <c r="C3" t="s">
+        <v>684</v>
+      </c>
+      <c r="D3" t="s">
+        <v>626</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="14" t="s">
+        <v>631</v>
+      </c>
+      <c r="B4" t="s">
+        <v>607</v>
+      </c>
+      <c r="C4" t="s">
         <v>685</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>657</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>658</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>659</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+      <c r="D4" t="s">
+        <v>625</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="20" t="s">
+        <v>632</v>
+      </c>
+      <c r="B5" t="s">
+        <v>683</v>
+      </c>
+      <c r="C5" t="s">
         <v>686</v>
       </c>
-      <c r="B2" t="s">
-        <v>661</v>
-      </c>
-      <c r="C2" t="s">
-        <v>749</v>
-      </c>
-      <c r="D2" t="s">
-        <v>683</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="20"/>
-      <c r="B3" t="s">
-        <v>662</v>
-      </c>
-      <c r="C3" t="s">
-        <v>741</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="D5" t="s">
         <v>682</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="20"/>
+      <c r="B6" t="s">
+        <v>608</v>
+      </c>
+      <c r="C6" t="s">
         <v>687</v>
       </c>
-      <c r="B4" t="s">
-        <v>663</v>
-      </c>
-      <c r="C4" t="s">
-        <v>742</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="D6" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="20"/>
+      <c r="B7" t="s">
+        <v>609</v>
+      </c>
+      <c r="C7" t="s">
+        <v>688</v>
+      </c>
+      <c r="D7" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="20"/>
+      <c r="B8" t="s">
+        <v>619</v>
+      </c>
+      <c r="C8" t="s">
+        <v>689</v>
+      </c>
+      <c r="D8" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="20"/>
+      <c r="B9" t="s">
+        <v>620</v>
+      </c>
+      <c r="C9" t="s">
+        <v>690</v>
+      </c>
+      <c r="D9" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="20"/>
+      <c r="B10" t="s">
+        <v>620</v>
+      </c>
+      <c r="C10" t="s">
+        <v>691</v>
+      </c>
+      <c r="D10" t="s">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="17"/>
+      <c r="B11" s="18" t="s">
+        <v>678</v>
+      </c>
+      <c r="C11" t="s">
+        <v>694</v>
+      </c>
+      <c r="D11" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="16" t="s">
+        <v>679</v>
+      </c>
+      <c r="B12" s="9"/>
+      <c r="C12" s="15" t="s">
+        <v>693</v>
+      </c>
+      <c r="D12" s="15" t="s">
         <v>681</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="21" t="s">
-        <v>688</v>
-      </c>
-      <c r="B5" t="s">
-        <v>740</v>
-      </c>
-      <c r="C5" t="s">
-        <v>743</v>
-      </c>
-      <c r="D5" t="s">
-        <v>739</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="21"/>
-      <c r="B6" t="s">
-        <v>664</v>
-      </c>
-      <c r="C6" t="s">
-        <v>744</v>
-      </c>
-      <c r="D6" t="s">
-        <v>680</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="21"/>
-      <c r="B7" t="s">
-        <v>665</v>
-      </c>
-      <c r="C7" t="s">
-        <v>745</v>
-      </c>
-      <c r="D7" t="s">
-        <v>679</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="21"/>
-      <c r="B8" t="s">
-        <v>675</v>
-      </c>
-      <c r="C8" t="s">
-        <v>746</v>
-      </c>
-      <c r="D8" t="s">
-        <v>678</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="21"/>
-      <c r="B9" t="s">
-        <v>676</v>
-      </c>
-      <c r="C9" t="s">
-        <v>747</v>
-      </c>
-      <c r="D9" t="s">
-        <v>677</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="21"/>
-      <c r="B10" t="s">
-        <v>676</v>
-      </c>
-      <c r="C10" t="s">
-        <v>748</v>
-      </c>
-      <c r="D10" t="s">
-        <v>684</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="18"/>
-      <c r="B11" s="19" t="s">
-        <v>735</v>
-      </c>
-      <c r="C11" t="s">
-        <v>751</v>
-      </c>
-      <c r="D11" t="s">
-        <v>737</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="17" t="s">
-        <v>736</v>
-      </c>
-      <c r="B12" s="9"/>
-      <c r="C12" s="16" t="s">
-        <v>750</v>
-      </c>
-      <c r="D12" s="16" t="s">
-        <v>738</v>
       </c>
     </row>
   </sheetData>
@@ -4201,31 +4049,31 @@
         <v>135</v>
       </c>
       <c r="EG1" s="3" t="s">
-        <v>666</v>
+        <v>610</v>
       </c>
       <c r="EH1" s="3" t="s">
-        <v>667</v>
+        <v>611</v>
       </c>
       <c r="EI1" s="3" t="s">
-        <v>668</v>
+        <v>612</v>
       </c>
       <c r="EJ1" s="3" t="s">
-        <v>669</v>
+        <v>613</v>
       </c>
       <c r="EK1" s="3" t="s">
-        <v>670</v>
+        <v>614</v>
       </c>
       <c r="EL1" s="3" t="s">
-        <v>671</v>
+        <v>615</v>
       </c>
       <c r="EM1" s="3" t="s">
-        <v>672</v>
+        <v>616</v>
       </c>
       <c r="EN1" s="3" t="s">
-        <v>673</v>
+        <v>617</v>
       </c>
       <c r="EO1" s="3" t="s">
-        <v>674</v>
+        <v>618</v>
       </c>
     </row>
     <row r="2" spans="1:145" ht="75" x14ac:dyDescent="0.25">
@@ -12723,187 +12571,187 @@
     </row>
     <row r="84" spans="1:136" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="8"/>
-      <c r="B84" s="22" t="s">
+      <c r="B84" s="21" t="s">
         <v>518</v>
       </c>
-      <c r="C84" s="22"/>
-      <c r="D84" s="22"/>
-      <c r="E84" s="22"/>
-      <c r="F84" s="22"/>
-      <c r="G84" s="22"/>
-      <c r="H84" s="22"/>
-      <c r="I84" s="22"/>
-      <c r="J84" s="22"/>
-      <c r="K84" s="22"/>
-      <c r="L84" s="22"/>
-      <c r="M84" s="22"/>
-      <c r="N84" s="22"/>
-      <c r="O84" s="22"/>
-      <c r="P84" s="22"/>
-      <c r="Q84" s="22"/>
-      <c r="R84" s="22"/>
+      <c r="C84" s="21"/>
+      <c r="D84" s="21"/>
+      <c r="E84" s="21"/>
+      <c r="F84" s="21"/>
+      <c r="G84" s="21"/>
+      <c r="H84" s="21"/>
+      <c r="I84" s="21"/>
+      <c r="J84" s="21"/>
+      <c r="K84" s="21"/>
+      <c r="L84" s="21"/>
+      <c r="M84" s="21"/>
+      <c r="N84" s="21"/>
+      <c r="O84" s="21"/>
+      <c r="P84" s="21"/>
+      <c r="Q84" s="21"/>
+      <c r="R84" s="21"/>
     </row>
     <row r="85" spans="1:136" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="9"/>
-      <c r="B85" s="23" t="s">
+      <c r="B85" s="22" t="s">
         <v>519</v>
       </c>
-      <c r="C85" s="23"/>
-      <c r="D85" s="23"/>
-      <c r="E85" s="23"/>
-      <c r="F85" s="23"/>
-      <c r="G85" s="23"/>
-      <c r="H85" s="23"/>
-      <c r="I85" s="23"/>
-      <c r="J85" s="23"/>
-      <c r="K85" s="23"/>
-      <c r="L85" s="23"/>
-      <c r="M85" s="23"/>
-      <c r="N85" s="23"/>
-      <c r="O85" s="23"/>
-      <c r="P85" s="23"/>
-      <c r="Q85" s="23"/>
-      <c r="R85" s="23"/>
+      <c r="C85" s="22"/>
+      <c r="D85" s="22"/>
+      <c r="E85" s="22"/>
+      <c r="F85" s="22"/>
+      <c r="G85" s="22"/>
+      <c r="H85" s="22"/>
+      <c r="I85" s="22"/>
+      <c r="J85" s="22"/>
+      <c r="K85" s="22"/>
+      <c r="L85" s="22"/>
+      <c r="M85" s="22"/>
+      <c r="N85" s="22"/>
+      <c r="O85" s="22"/>
+      <c r="P85" s="22"/>
+      <c r="Q85" s="22"/>
+      <c r="R85" s="22"/>
     </row>
     <row r="86" spans="1:136" x14ac:dyDescent="0.25">
       <c r="A86" s="9"/>
-      <c r="B86" s="23"/>
-      <c r="C86" s="23"/>
-      <c r="D86" s="23"/>
-      <c r="E86" s="23"/>
-      <c r="F86" s="23"/>
-      <c r="G86" s="23"/>
-      <c r="H86" s="23"/>
-      <c r="I86" s="23"/>
-      <c r="J86" s="23"/>
-      <c r="K86" s="23"/>
-      <c r="L86" s="23"/>
-      <c r="M86" s="23"/>
-      <c r="N86" s="23"/>
-      <c r="O86" s="23"/>
-      <c r="P86" s="23"/>
-      <c r="Q86" s="23"/>
-      <c r="R86" s="23"/>
+      <c r="B86" s="22"/>
+      <c r="C86" s="22"/>
+      <c r="D86" s="22"/>
+      <c r="E86" s="22"/>
+      <c r="F86" s="22"/>
+      <c r="G86" s="22"/>
+      <c r="H86" s="22"/>
+      <c r="I86" s="22"/>
+      <c r="J86" s="22"/>
+      <c r="K86" s="22"/>
+      <c r="L86" s="22"/>
+      <c r="M86" s="22"/>
+      <c r="N86" s="22"/>
+      <c r="O86" s="22"/>
+      <c r="P86" s="22"/>
+      <c r="Q86" s="22"/>
+      <c r="R86" s="22"/>
     </row>
     <row r="87" spans="1:136" x14ac:dyDescent="0.25">
       <c r="A87" s="9"/>
-      <c r="B87" s="23"/>
-      <c r="C87" s="23"/>
-      <c r="D87" s="23"/>
-      <c r="E87" s="23"/>
-      <c r="F87" s="23"/>
-      <c r="G87" s="23"/>
-      <c r="H87" s="23"/>
-      <c r="I87" s="23"/>
-      <c r="J87" s="23"/>
-      <c r="K87" s="23"/>
-      <c r="L87" s="23"/>
-      <c r="M87" s="23"/>
-      <c r="N87" s="23"/>
-      <c r="O87" s="23"/>
-      <c r="P87" s="23"/>
-      <c r="Q87" s="23"/>
-      <c r="R87" s="23"/>
+      <c r="B87" s="22"/>
+      <c r="C87" s="22"/>
+      <c r="D87" s="22"/>
+      <c r="E87" s="22"/>
+      <c r="F87" s="22"/>
+      <c r="G87" s="22"/>
+      <c r="H87" s="22"/>
+      <c r="I87" s="22"/>
+      <c r="J87" s="22"/>
+      <c r="K87" s="22"/>
+      <c r="L87" s="22"/>
+      <c r="M87" s="22"/>
+      <c r="N87" s="22"/>
+      <c r="O87" s="22"/>
+      <c r="P87" s="22"/>
+      <c r="Q87" s="22"/>
+      <c r="R87" s="22"/>
     </row>
     <row r="88" spans="1:136" x14ac:dyDescent="0.25">
       <c r="A88" s="9"/>
-      <c r="B88" s="23"/>
-      <c r="C88" s="23"/>
-      <c r="D88" s="23"/>
-      <c r="E88" s="23"/>
-      <c r="F88" s="23"/>
-      <c r="G88" s="23"/>
-      <c r="H88" s="23"/>
-      <c r="I88" s="23"/>
-      <c r="J88" s="23"/>
-      <c r="K88" s="23"/>
-      <c r="L88" s="23"/>
-      <c r="M88" s="23"/>
-      <c r="N88" s="23"/>
-      <c r="O88" s="23"/>
-      <c r="P88" s="23"/>
-      <c r="Q88" s="23"/>
-      <c r="R88" s="23"/>
+      <c r="B88" s="22"/>
+      <c r="C88" s="22"/>
+      <c r="D88" s="22"/>
+      <c r="E88" s="22"/>
+      <c r="F88" s="22"/>
+      <c r="G88" s="22"/>
+      <c r="H88" s="22"/>
+      <c r="I88" s="22"/>
+      <c r="J88" s="22"/>
+      <c r="K88" s="22"/>
+      <c r="L88" s="22"/>
+      <c r="M88" s="22"/>
+      <c r="N88" s="22"/>
+      <c r="O88" s="22"/>
+      <c r="P88" s="22"/>
+      <c r="Q88" s="22"/>
+      <c r="R88" s="22"/>
     </row>
     <row r="89" spans="1:136" x14ac:dyDescent="0.25">
       <c r="A89" s="9"/>
-      <c r="B89" s="23"/>
-      <c r="C89" s="23"/>
-      <c r="D89" s="23"/>
-      <c r="E89" s="23"/>
-      <c r="F89" s="23"/>
-      <c r="G89" s="23"/>
-      <c r="H89" s="23"/>
-      <c r="I89" s="23"/>
-      <c r="J89" s="23"/>
-      <c r="K89" s="23"/>
-      <c r="L89" s="23"/>
-      <c r="M89" s="23"/>
-      <c r="N89" s="23"/>
-      <c r="O89" s="23"/>
-      <c r="P89" s="23"/>
-      <c r="Q89" s="23"/>
-      <c r="R89" s="23"/>
+      <c r="B89" s="22"/>
+      <c r="C89" s="22"/>
+      <c r="D89" s="22"/>
+      <c r="E89" s="22"/>
+      <c r="F89" s="22"/>
+      <c r="G89" s="22"/>
+      <c r="H89" s="22"/>
+      <c r="I89" s="22"/>
+      <c r="J89" s="22"/>
+      <c r="K89" s="22"/>
+      <c r="L89" s="22"/>
+      <c r="M89" s="22"/>
+      <c r="N89" s="22"/>
+      <c r="O89" s="22"/>
+      <c r="P89" s="22"/>
+      <c r="Q89" s="22"/>
+      <c r="R89" s="22"/>
     </row>
     <row r="90" spans="1:136" x14ac:dyDescent="0.25">
       <c r="A90" s="9"/>
-      <c r="B90" s="23"/>
-      <c r="C90" s="23"/>
-      <c r="D90" s="23"/>
-      <c r="E90" s="23"/>
-      <c r="F90" s="23"/>
-      <c r="G90" s="23"/>
-      <c r="H90" s="23"/>
-      <c r="I90" s="23"/>
-      <c r="J90" s="23"/>
-      <c r="K90" s="23"/>
-      <c r="L90" s="23"/>
-      <c r="M90" s="23"/>
-      <c r="N90" s="23"/>
-      <c r="O90" s="23"/>
-      <c r="P90" s="23"/>
-      <c r="Q90" s="23"/>
-      <c r="R90" s="23"/>
+      <c r="B90" s="22"/>
+      <c r="C90" s="22"/>
+      <c r="D90" s="22"/>
+      <c r="E90" s="22"/>
+      <c r="F90" s="22"/>
+      <c r="G90" s="22"/>
+      <c r="H90" s="22"/>
+      <c r="I90" s="22"/>
+      <c r="J90" s="22"/>
+      <c r="K90" s="22"/>
+      <c r="L90" s="22"/>
+      <c r="M90" s="22"/>
+      <c r="N90" s="22"/>
+      <c r="O90" s="22"/>
+      <c r="P90" s="22"/>
+      <c r="Q90" s="22"/>
+      <c r="R90" s="22"/>
     </row>
     <row r="91" spans="1:136" x14ac:dyDescent="0.25">
       <c r="A91" s="9"/>
-      <c r="B91" s="23"/>
-      <c r="C91" s="23"/>
-      <c r="D91" s="23"/>
-      <c r="E91" s="23"/>
-      <c r="F91" s="23"/>
-      <c r="G91" s="23"/>
-      <c r="H91" s="23"/>
-      <c r="I91" s="23"/>
-      <c r="J91" s="23"/>
-      <c r="K91" s="23"/>
-      <c r="L91" s="23"/>
-      <c r="M91" s="23"/>
-      <c r="N91" s="23"/>
-      <c r="O91" s="23"/>
-      <c r="P91" s="23"/>
-      <c r="Q91" s="23"/>
-      <c r="R91" s="23"/>
+      <c r="B91" s="22"/>
+      <c r="C91" s="22"/>
+      <c r="D91" s="22"/>
+      <c r="E91" s="22"/>
+      <c r="F91" s="22"/>
+      <c r="G91" s="22"/>
+      <c r="H91" s="22"/>
+      <c r="I91" s="22"/>
+      <c r="J91" s="22"/>
+      <c r="K91" s="22"/>
+      <c r="L91" s="22"/>
+      <c r="M91" s="22"/>
+      <c r="N91" s="22"/>
+      <c r="O91" s="22"/>
+      <c r="P91" s="22"/>
+      <c r="Q91" s="22"/>
+      <c r="R91" s="22"/>
     </row>
     <row r="92" spans="1:136" x14ac:dyDescent="0.25">
       <c r="A92" s="9"/>
-      <c r="B92" s="23"/>
-      <c r="C92" s="23"/>
-      <c r="D92" s="23"/>
-      <c r="E92" s="23"/>
-      <c r="F92" s="23"/>
-      <c r="G92" s="23"/>
-      <c r="H92" s="23"/>
-      <c r="I92" s="23"/>
-      <c r="J92" s="23"/>
-      <c r="K92" s="23"/>
-      <c r="L92" s="23"/>
-      <c r="M92" s="23"/>
-      <c r="N92" s="23"/>
-      <c r="O92" s="23"/>
-      <c r="P92" s="23"/>
-      <c r="Q92" s="23"/>
-      <c r="R92" s="23"/>
+      <c r="B92" s="22"/>
+      <c r="C92" s="22"/>
+      <c r="D92" s="22"/>
+      <c r="E92" s="22"/>
+      <c r="F92" s="22"/>
+      <c r="G92" s="22"/>
+      <c r="H92" s="22"/>
+      <c r="I92" s="22"/>
+      <c r="J92" s="22"/>
+      <c r="K92" s="22"/>
+      <c r="L92" s="22"/>
+      <c r="M92" s="22"/>
+      <c r="N92" s="22"/>
+      <c r="O92" s="22"/>
+      <c r="P92" s="22"/>
+      <c r="Q92" s="22"/>
+      <c r="R92" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -12922,7 +12770,7 @@
   <sheetPr>
     <tabColor theme="8"/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.140625" bestFit="1" customWidth="1"/>
@@ -12949,918 +12797,382 @@
         <v>524</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
-        <v>715</v>
+    <row r="2" spans="1:5" s="10" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="11" t="s">
+        <v>658</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>525</v>
+        <v>659</v>
       </c>
       <c r="B3" t="s">
+        <v>633</v>
+      </c>
+      <c r="C3" t="s">
+        <v>634</v>
+      </c>
+      <c r="D3" t="s">
         <v>526</v>
       </c>
-      <c r="C3" t="s">
-        <v>527</v>
-      </c>
-      <c r="D3" t="s">
-        <v>528</v>
-      </c>
       <c r="E3" t="s">
-        <v>529</v>
+        <v>635</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>530</v>
+        <v>660</v>
       </c>
       <c r="B4" t="s">
+        <v>525</v>
+      </c>
+      <c r="C4" t="s">
+        <v>634</v>
+      </c>
+      <c r="D4" t="s">
         <v>526</v>
       </c>
-      <c r="C4" t="s">
-        <v>531</v>
-      </c>
-      <c r="D4" t="s">
-        <v>528</v>
-      </c>
       <c r="E4" t="s">
-        <v>532</v>
+        <v>636</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>530</v>
+        <v>661</v>
       </c>
       <c r="B5" t="s">
+        <v>633</v>
+      </c>
+      <c r="C5" t="s">
+        <v>634</v>
+      </c>
+      <c r="D5" t="s">
         <v>526</v>
       </c>
-      <c r="C5" t="s">
-        <v>531</v>
-      </c>
-      <c r="D5" t="s">
-        <v>528</v>
-      </c>
       <c r="E5" t="s">
-        <v>533</v>
+        <v>637</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>534</v>
+        <v>662</v>
       </c>
       <c r="B6" t="s">
+        <v>638</v>
+      </c>
+      <c r="C6" t="s">
+        <v>634</v>
+      </c>
+      <c r="D6" t="s">
         <v>526</v>
       </c>
-      <c r="C6" t="s">
-        <v>531</v>
-      </c>
-      <c r="D6" t="s">
-        <v>528</v>
-      </c>
       <c r="E6" t="s">
-        <v>535</v>
+        <v>527</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>536</v>
+        <v>663</v>
       </c>
       <c r="B7" t="s">
-        <v>537</v>
+        <v>639</v>
       </c>
       <c r="C7" t="s">
-        <v>531</v>
+        <v>634</v>
       </c>
       <c r="D7" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="E7" t="s">
-        <v>538</v>
+        <v>527</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>536</v>
+        <v>664</v>
       </c>
       <c r="B8" t="s">
-        <v>537</v>
+        <v>640</v>
       </c>
       <c r="C8" t="s">
-        <v>531</v>
+        <v>641</v>
       </c>
       <c r="D8" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="E8" t="s">
-        <v>539</v>
+        <v>642</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>540</v>
+        <v>665</v>
       </c>
       <c r="B9" t="s">
-        <v>537</v>
+        <v>633</v>
       </c>
       <c r="C9" t="s">
-        <v>531</v>
+        <v>634</v>
       </c>
       <c r="D9" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="E9" t="s">
-        <v>541</v>
+        <v>643</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>542</v>
+        <v>666</v>
       </c>
       <c r="B10" t="s">
+        <v>525</v>
+      </c>
+      <c r="C10" t="s">
+        <v>634</v>
+      </c>
+      <c r="D10" t="s">
         <v>526</v>
       </c>
-      <c r="C10" t="s">
-        <v>531</v>
-      </c>
-      <c r="D10" t="s">
-        <v>528</v>
-      </c>
       <c r="E10" t="s">
-        <v>543</v>
+        <v>644</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>542</v>
+        <v>667</v>
       </c>
       <c r="B11" t="s">
+        <v>633</v>
+      </c>
+      <c r="C11" t="s">
+        <v>634</v>
+      </c>
+      <c r="D11" t="s">
         <v>526</v>
       </c>
-      <c r="C11" t="s">
-        <v>531</v>
-      </c>
-      <c r="D11" t="s">
-        <v>528</v>
-      </c>
       <c r="E11" t="s">
-        <v>544</v>
+        <v>643</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>542</v>
+        <v>668</v>
       </c>
       <c r="B12" t="s">
+        <v>638</v>
+      </c>
+      <c r="C12" t="s">
+        <v>634</v>
+      </c>
+      <c r="D12" t="s">
         <v>526</v>
       </c>
-      <c r="C12" t="s">
-        <v>531</v>
-      </c>
-      <c r="D12" t="s">
-        <v>528</v>
-      </c>
       <c r="E12" t="s">
-        <v>545</v>
+        <v>645</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>546</v>
+        <v>669</v>
       </c>
       <c r="B13" t="s">
+        <v>639</v>
+      </c>
+      <c r="C13" t="s">
+        <v>634</v>
+      </c>
+      <c r="D13" t="s">
         <v>526</v>
       </c>
-      <c r="C13" t="s">
-        <v>531</v>
-      </c>
-      <c r="D13" t="s">
-        <v>528</v>
-      </c>
       <c r="E13" t="s">
-        <v>547</v>
+        <v>645</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>546</v>
+        <v>670</v>
       </c>
       <c r="B14" t="s">
+        <v>640</v>
+      </c>
+      <c r="C14" t="s">
+        <v>646</v>
+      </c>
+      <c r="D14" t="s">
         <v>526</v>
       </c>
-      <c r="C14" t="s">
-        <v>531</v>
-      </c>
-      <c r="D14" t="s">
-        <v>528</v>
-      </c>
       <c r="E14" t="s">
-        <v>548</v>
+        <v>642</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>549</v>
+        <v>671</v>
       </c>
       <c r="B15" t="s">
-        <v>537</v>
+        <v>639</v>
       </c>
       <c r="C15" t="s">
-        <v>531</v>
+        <v>647</v>
       </c>
       <c r="D15" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="E15" t="s">
-        <v>550</v>
+        <v>648</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>551</v>
+        <v>672</v>
       </c>
       <c r="B16" t="s">
-        <v>537</v>
+        <v>525</v>
       </c>
       <c r="C16" t="s">
-        <v>531</v>
+        <v>647</v>
       </c>
       <c r="D16" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="E16" t="s">
-        <v>552</v>
+        <v>649</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>551</v>
+        <v>673</v>
       </c>
       <c r="B17" t="s">
-        <v>537</v>
+        <v>525</v>
       </c>
       <c r="C17" t="s">
-        <v>531</v>
+        <v>650</v>
       </c>
       <c r="D17" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="E17" t="s">
-        <v>553</v>
+        <v>651</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>551</v>
+        <v>674</v>
       </c>
       <c r="B18" t="s">
-        <v>537</v>
+        <v>525</v>
       </c>
       <c r="C18" t="s">
-        <v>531</v>
+        <v>650</v>
       </c>
       <c r="D18" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="E18" t="s">
-        <v>554</v>
+        <v>652</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>551</v>
+        <v>675</v>
       </c>
       <c r="B19" t="s">
-        <v>537</v>
+        <v>653</v>
       </c>
       <c r="C19" t="s">
-        <v>531</v>
+        <v>654</v>
       </c>
       <c r="D19" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="E19" t="s">
-        <v>555</v>
+        <v>655</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>556</v>
+        <v>676</v>
       </c>
       <c r="B20" t="s">
+        <v>639</v>
+      </c>
+      <c r="C20" t="s">
+        <v>647</v>
+      </c>
+      <c r="D20" t="s">
         <v>526</v>
       </c>
-      <c r="C20" t="s">
-        <v>557</v>
-      </c>
-      <c r="D20" t="s">
-        <v>528</v>
-      </c>
       <c r="E20" t="s">
-        <v>529</v>
+        <v>656</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>558</v>
+        <v>677</v>
       </c>
       <c r="B21" t="s">
+        <v>525</v>
+      </c>
+      <c r="C21" t="s">
+        <v>647</v>
+      </c>
+      <c r="D21" t="s">
         <v>526</v>
       </c>
-      <c r="C21" t="s">
-        <v>559</v>
-      </c>
-      <c r="D21" t="s">
-        <v>528</v>
-      </c>
       <c r="E21" t="s">
-        <v>560</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>558</v>
-      </c>
-      <c r="B22" t="s">
-        <v>526</v>
-      </c>
-      <c r="C22" t="s">
-        <v>559</v>
-      </c>
-      <c r="D22" t="s">
-        <v>528</v>
-      </c>
-      <c r="E22" t="s">
-        <v>561</v>
+        <v>657</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>562</v>
-      </c>
-      <c r="B23" t="s">
-        <v>526</v>
-      </c>
-      <c r="C23" t="s">
-        <v>559</v>
-      </c>
-      <c r="D23" t="s">
-        <v>528</v>
-      </c>
-      <c r="E23" t="s">
-        <v>563</v>
-      </c>
+      <c r="A23" s="24" t="s">
+        <v>695</v>
+      </c>
+      <c r="B23" s="23"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="23"/>
+      <c r="E23" s="23"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>562</v>
-      </c>
-      <c r="B24" t="s">
-        <v>526</v>
-      </c>
-      <c r="C24" t="s">
-        <v>559</v>
-      </c>
-      <c r="D24" t="s">
-        <v>528</v>
-      </c>
-      <c r="E24" t="s">
-        <v>564</v>
-      </c>
+      <c r="A24" s="23"/>
+      <c r="B24" s="23"/>
+      <c r="C24" s="23"/>
+      <c r="D24" s="23"/>
+      <c r="E24" s="23"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>562</v>
-      </c>
-      <c r="B25" t="s">
-        <v>526</v>
-      </c>
-      <c r="C25" t="s">
-        <v>559</v>
-      </c>
-      <c r="D25" t="s">
-        <v>528</v>
-      </c>
-      <c r="E25" t="s">
-        <v>565</v>
-      </c>
+      <c r="A25" s="23"/>
+      <c r="B25" s="23"/>
+      <c r="C25" s="23"/>
+      <c r="D25" s="23"/>
+      <c r="E25" s="23"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>566</v>
-      </c>
-      <c r="B26" t="s">
-        <v>526</v>
-      </c>
-      <c r="C26" t="s">
-        <v>559</v>
-      </c>
-      <c r="D26" t="s">
-        <v>528</v>
-      </c>
-      <c r="E26" t="s">
-        <v>567</v>
-      </c>
+      <c r="A26" s="23"/>
+      <c r="B26" s="23"/>
+      <c r="C26" s="23"/>
+      <c r="D26" s="23"/>
+      <c r="E26" s="23"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>568</v>
-      </c>
-      <c r="B27" t="s">
-        <v>537</v>
-      </c>
-      <c r="C27" t="s">
-        <v>559</v>
-      </c>
-      <c r="D27" t="s">
-        <v>528</v>
-      </c>
-      <c r="E27" t="s">
-        <v>569</v>
-      </c>
+      <c r="A27" s="23"/>
+      <c r="B27" s="23"/>
+      <c r="C27" s="23"/>
+      <c r="D27" s="23"/>
+      <c r="E27" s="23"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>568</v>
-      </c>
-      <c r="B28" t="s">
-        <v>537</v>
-      </c>
-      <c r="C28" t="s">
-        <v>559</v>
-      </c>
-      <c r="D28" t="s">
-        <v>528</v>
-      </c>
-      <c r="E28" t="s">
-        <v>570</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>568</v>
-      </c>
-      <c r="B29" t="s">
-        <v>537</v>
-      </c>
-      <c r="C29" t="s">
-        <v>559</v>
-      </c>
-      <c r="D29" t="s">
-        <v>528</v>
-      </c>
-      <c r="E29" t="s">
-        <v>571</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>572</v>
-      </c>
-      <c r="B30" t="s">
-        <v>537</v>
-      </c>
-      <c r="C30" t="s">
-        <v>559</v>
-      </c>
-      <c r="D30" t="s">
-        <v>528</v>
-      </c>
-      <c r="E30" t="s">
-        <v>573</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>572</v>
-      </c>
-      <c r="B31" t="s">
-        <v>537</v>
-      </c>
-      <c r="C31" t="s">
-        <v>559</v>
-      </c>
-      <c r="D31" t="s">
-        <v>528</v>
-      </c>
-      <c r="E31" t="s">
-        <v>574</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>572</v>
-      </c>
-      <c r="B32" t="s">
-        <v>537</v>
-      </c>
-      <c r="C32" t="s">
-        <v>559</v>
-      </c>
-      <c r="D32" t="s">
-        <v>528</v>
-      </c>
-      <c r="E32" t="s">
-        <v>575</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>576</v>
-      </c>
-      <c r="B33" t="s">
-        <v>526</v>
-      </c>
-      <c r="C33" t="s">
-        <v>577</v>
-      </c>
-      <c r="D33" t="s">
-        <v>528</v>
-      </c>
-      <c r="E33" t="s">
-        <v>529</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>578</v>
-      </c>
-      <c r="B34" t="s">
-        <v>526</v>
-      </c>
-      <c r="C34" t="s">
-        <v>579</v>
-      </c>
-      <c r="D34" t="s">
-        <v>528</v>
-      </c>
-      <c r="E34" t="s">
-        <v>529</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>580</v>
-      </c>
-      <c r="B35" t="s">
-        <v>526</v>
-      </c>
-      <c r="C35" t="s">
-        <v>581</v>
-      </c>
-      <c r="D35" t="s">
-        <v>528</v>
-      </c>
-      <c r="E35" t="s">
-        <v>529</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>582</v>
-      </c>
-      <c r="B36" t="s">
-        <v>526</v>
-      </c>
-      <c r="C36" t="s">
-        <v>583</v>
-      </c>
-      <c r="D36" t="s">
-        <v>528</v>
-      </c>
-      <c r="E36" t="s">
-        <v>529</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" s="10" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A37" s="12" t="s">
-        <v>714</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>716</v>
-      </c>
-      <c r="B38" t="s">
-        <v>689</v>
-      </c>
-      <c r="C38" t="s">
-        <v>690</v>
-      </c>
-      <c r="D38" t="s">
-        <v>528</v>
-      </c>
-      <c r="E38" t="s">
-        <v>691</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>717</v>
-      </c>
-      <c r="B39" t="s">
-        <v>526</v>
-      </c>
-      <c r="C39" t="s">
-        <v>690</v>
-      </c>
-      <c r="D39" t="s">
-        <v>528</v>
-      </c>
-      <c r="E39" t="s">
-        <v>692</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>718</v>
-      </c>
-      <c r="B40" t="s">
-        <v>689</v>
-      </c>
-      <c r="C40" t="s">
-        <v>690</v>
-      </c>
-      <c r="D40" t="s">
-        <v>528</v>
-      </c>
-      <c r="E40" t="s">
-        <v>693</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>719</v>
-      </c>
-      <c r="B41" t="s">
-        <v>694</v>
-      </c>
-      <c r="C41" t="s">
-        <v>690</v>
-      </c>
-      <c r="D41" t="s">
-        <v>528</v>
-      </c>
-      <c r="E41" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>720</v>
-      </c>
-      <c r="B42" t="s">
-        <v>695</v>
-      </c>
-      <c r="C42" t="s">
-        <v>690</v>
-      </c>
-      <c r="D42" t="s">
-        <v>528</v>
-      </c>
-      <c r="E42" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>721</v>
-      </c>
-      <c r="B43" t="s">
-        <v>696</v>
-      </c>
-      <c r="C43" t="s">
-        <v>697</v>
-      </c>
-      <c r="D43" t="s">
-        <v>528</v>
-      </c>
-      <c r="E43" t="s">
-        <v>698</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>722</v>
-      </c>
-      <c r="B44" t="s">
-        <v>689</v>
-      </c>
-      <c r="C44" t="s">
-        <v>690</v>
-      </c>
-      <c r="D44" t="s">
-        <v>528</v>
-      </c>
-      <c r="E44" t="s">
-        <v>699</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>723</v>
-      </c>
-      <c r="B45" t="s">
-        <v>526</v>
-      </c>
-      <c r="C45" t="s">
-        <v>690</v>
-      </c>
-      <c r="D45" t="s">
-        <v>528</v>
-      </c>
-      <c r="E45" t="s">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>724</v>
-      </c>
-      <c r="B46" t="s">
-        <v>689</v>
-      </c>
-      <c r="C46" t="s">
-        <v>690</v>
-      </c>
-      <c r="D46" t="s">
-        <v>528</v>
-      </c>
-      <c r="E46" t="s">
-        <v>699</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>725</v>
-      </c>
-      <c r="B47" t="s">
-        <v>694</v>
-      </c>
-      <c r="C47" t="s">
-        <v>690</v>
-      </c>
-      <c r="D47" t="s">
-        <v>528</v>
-      </c>
-      <c r="E47" t="s">
-        <v>701</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>726</v>
-      </c>
-      <c r="B48" t="s">
-        <v>695</v>
-      </c>
-      <c r="C48" t="s">
-        <v>690</v>
-      </c>
-      <c r="D48" t="s">
-        <v>528</v>
-      </c>
-      <c r="E48" t="s">
-        <v>701</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>727</v>
-      </c>
-      <c r="B49" t="s">
-        <v>696</v>
-      </c>
-      <c r="C49" t="s">
-        <v>702</v>
-      </c>
-      <c r="D49" t="s">
-        <v>528</v>
-      </c>
-      <c r="E49" t="s">
-        <v>698</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>728</v>
-      </c>
-      <c r="B50" t="s">
-        <v>695</v>
-      </c>
-      <c r="C50" t="s">
-        <v>703</v>
-      </c>
-      <c r="D50" t="s">
-        <v>528</v>
-      </c>
-      <c r="E50" t="s">
-        <v>704</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>729</v>
-      </c>
-      <c r="B51" t="s">
-        <v>526</v>
-      </c>
-      <c r="C51" t="s">
-        <v>703</v>
-      </c>
-      <c r="D51" t="s">
-        <v>528</v>
-      </c>
-      <c r="E51" t="s">
-        <v>705</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>730</v>
-      </c>
-      <c r="B52" t="s">
-        <v>526</v>
-      </c>
-      <c r="C52" t="s">
-        <v>706</v>
-      </c>
-      <c r="D52" t="s">
-        <v>528</v>
-      </c>
-      <c r="E52" t="s">
-        <v>707</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>731</v>
-      </c>
-      <c r="B53" t="s">
-        <v>526</v>
-      </c>
-      <c r="C53" t="s">
-        <v>706</v>
-      </c>
-      <c r="D53" t="s">
-        <v>528</v>
-      </c>
-      <c r="E53" t="s">
-        <v>708</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>732</v>
-      </c>
-      <c r="B54" t="s">
-        <v>709</v>
-      </c>
-      <c r="C54" t="s">
-        <v>710</v>
-      </c>
-      <c r="D54" t="s">
-        <v>528</v>
-      </c>
-      <c r="E54" t="s">
-        <v>711</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>733</v>
-      </c>
-      <c r="B55" t="s">
-        <v>695</v>
-      </c>
-      <c r="C55" t="s">
-        <v>703</v>
-      </c>
-      <c r="D55" t="s">
-        <v>528</v>
-      </c>
-      <c r="E55" t="s">
-        <v>712</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>734</v>
-      </c>
-      <c r="B56" t="s">
-        <v>526</v>
-      </c>
-      <c r="C56" t="s">
-        <v>703</v>
-      </c>
-      <c r="D56" t="s">
-        <v>528</v>
-      </c>
-      <c r="E56" t="s">
-        <v>713</v>
-      </c>
+      <c r="A28" s="23"/>
+      <c r="B28" s="23"/>
+      <c r="C28" s="23"/>
+      <c r="D28" s="23"/>
+      <c r="E28" s="23"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A23:E28"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -13889,60 +13201,60 @@
   <sheetData>
     <row r="1" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>584</v>
+        <v>528</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>585</v>
+        <v>529</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>586</v>
+        <v>530</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>587</v>
+        <v>531</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>588</v>
+        <v>532</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>589</v>
+        <v>533</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>590</v>
+        <v>534</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>591</v>
+        <v>535</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>592</v>
+        <v>536</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>593</v>
+        <v>537</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>594</v>
+        <v>538</v>
       </c>
     </row>
     <row r="2" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>595</v>
+        <v>539</v>
       </c>
       <c r="C2" s="6">
         <v>0</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>596</v>
+        <v>540</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>597</v>
+        <v>541</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>598</v>
+        <v>542</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>599</v>
+        <v>543</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>600</v>
+        <v>544</v>
       </c>
       <c r="I2" s="6">
         <v>0</v>
@@ -13953,22 +13265,22 @@
     </row>
     <row r="3" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>601</v>
+        <v>545</v>
       </c>
       <c r="C3" s="6">
         <v>0</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>596</v>
+        <v>540</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>597</v>
+        <v>541</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>602</v>
+        <v>546</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>603</v>
+        <v>547</v>
       </c>
       <c r="I3" s="6">
         <v>0</v>
@@ -13977,7 +13289,7 @@
         <v>0</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>604</v>
+        <v>548</v>
       </c>
     </row>
     <row r="4" spans="1:11" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -13988,16 +13300,16 @@
         <v>0</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>605</v>
+        <v>549</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>597</v>
+        <v>541</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>606</v>
+        <v>550</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>607</v>
+        <v>551</v>
       </c>
       <c r="I4" s="7">
         <v>0</v>
@@ -14014,16 +13326,16 @@
         <v>0</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>596</v>
+        <v>540</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>597</v>
+        <v>541</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>602</v>
+        <v>546</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>603</v>
+        <v>547</v>
       </c>
       <c r="I5" s="6">
         <v>0</v>
@@ -14040,16 +13352,16 @@
         <v>0</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>605</v>
+        <v>549</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>597</v>
+        <v>541</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>608</v>
+        <v>552</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>609</v>
+        <v>553</v>
       </c>
       <c r="I6" s="7">
         <v>1</v>
@@ -14058,7 +13370,7 @@
         <v>1</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>610</v>
+        <v>554</v>
       </c>
     </row>
     <row r="7" spans="1:11" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -14069,16 +13381,16 @@
         <v>2</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>605</v>
+        <v>549</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>597</v>
+        <v>541</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>608</v>
+        <v>552</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>609</v>
+        <v>553</v>
       </c>
       <c r="I7" s="7">
         <v>1</v>
@@ -14087,7 +13399,7 @@
         <v>1</v>
       </c>
       <c r="K7" s="7" t="s">
-        <v>611</v>
+        <v>555</v>
       </c>
     </row>
     <row r="8" spans="1:11" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -14098,16 +13410,16 @@
         <v>93</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>596</v>
+        <v>540</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>597</v>
+        <v>541</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>612</v>
+        <v>556</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>613</v>
+        <v>557</v>
       </c>
       <c r="I8" s="7">
         <v>49</v>
@@ -14116,7 +13428,7 @@
         <v>27</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>614</v>
+        <v>558</v>
       </c>
     </row>
     <row r="9" spans="1:11" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -14127,16 +13439,16 @@
         <v>100</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>615</v>
+        <v>559</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>597</v>
+        <v>541</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>616</v>
+        <v>560</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>613</v>
+        <v>557</v>
       </c>
       <c r="I9" s="7">
         <v>64</v>
@@ -14145,7 +13457,7 @@
         <v>35</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>617</v>
+        <v>561</v>
       </c>
     </row>
     <row r="10" spans="1:11" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -14156,16 +13468,16 @@
         <v>93</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>596</v>
+        <v>540</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>597</v>
+        <v>541</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>612</v>
+        <v>556</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>613</v>
+        <v>557</v>
       </c>
       <c r="I10" s="7">
         <v>45</v>
@@ -14174,27 +13486,27 @@
         <v>25</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>618</v>
+        <v>562</v>
       </c>
     </row>
     <row r="11" spans="1:11" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>619</v>
+        <v>563</v>
       </c>
       <c r="C11" s="7">
         <v>0</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>605</v>
+        <v>549</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>597</v>
+        <v>541</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>608</v>
+        <v>552</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>609</v>
+        <v>553</v>
       </c>
       <c r="I11" s="7">
         <v>1</v>
@@ -14203,27 +13515,27 @@
         <v>1</v>
       </c>
       <c r="K11" s="7" t="s">
-        <v>620</v>
+        <v>564</v>
       </c>
     </row>
     <row r="12" spans="1:11" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>621</v>
+        <v>565</v>
       </c>
       <c r="C12" s="7">
         <v>0</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>605</v>
+        <v>549</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>597</v>
+        <v>541</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>608</v>
+        <v>552</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>609</v>
+        <v>553</v>
       </c>
       <c r="I12" s="7">
         <v>1</v>
@@ -14232,27 +13544,27 @@
         <v>1</v>
       </c>
       <c r="K12" s="7" t="s">
-        <v>622</v>
+        <v>566</v>
       </c>
     </row>
     <row r="13" spans="1:11" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>623</v>
+        <v>567</v>
       </c>
       <c r="C13" s="7">
         <v>33</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>605</v>
+        <v>549</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>597</v>
+        <v>541</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>624</v>
+        <v>568</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>625</v>
+        <v>569</v>
       </c>
       <c r="I13" s="7">
         <v>11</v>
@@ -14261,7 +13573,7 @@
         <v>8</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>626</v>
+        <v>570</v>
       </c>
     </row>
     <row r="14" spans="1:11" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -14272,16 +13584,16 @@
         <v>0</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>605</v>
+        <v>549</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>597</v>
+        <v>541</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>608</v>
+        <v>552</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>609</v>
+        <v>553</v>
       </c>
       <c r="I14" s="7">
         <v>1</v>
@@ -14290,27 +13602,27 @@
         <v>1</v>
       </c>
       <c r="K14" s="7" t="s">
-        <v>610</v>
+        <v>554</v>
       </c>
     </row>
     <row r="15" spans="1:11" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>627</v>
+        <v>571</v>
       </c>
       <c r="C15" s="7">
         <v>0</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>605</v>
+        <v>549</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>597</v>
+        <v>541</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>624</v>
+        <v>568</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>625</v>
+        <v>569</v>
       </c>
       <c r="I15" s="7">
         <v>1</v>
@@ -14319,27 +13631,27 @@
         <v>1</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>628</v>
+        <v>572</v>
       </c>
     </row>
     <row r="16" spans="1:11" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
-        <v>629</v>
+        <v>573</v>
       </c>
       <c r="C16" s="7">
         <v>97</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>596</v>
+        <v>540</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>597</v>
+        <v>541</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>612</v>
+        <v>556</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>613</v>
+        <v>557</v>
       </c>
       <c r="I16" s="7">
         <v>60</v>
@@ -14348,30 +13660,30 @@
         <v>27</v>
       </c>
       <c r="K16" s="7" t="s">
-        <v>630</v>
+        <v>574</v>
       </c>
     </row>
     <row r="17" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>631</v>
+        <v>575</v>
       </c>
       <c r="C17" s="6">
         <v>0</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>596</v>
+        <v>540</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>632</v>
+        <v>576</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>633</v>
+        <v>577</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>634</v>
+        <v>578</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>635</v>
+        <v>579</v>
       </c>
       <c r="I17" s="6">
         <v>0</v>
@@ -14382,25 +13694,25 @@
     </row>
     <row r="18" spans="1:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>636</v>
+        <v>580</v>
       </c>
       <c r="C18" s="6">
         <v>0</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>596</v>
+        <v>540</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>632</v>
+        <v>576</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>633</v>
+        <v>577</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>634</v>
+        <v>578</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>637</v>
+        <v>581</v>
       </c>
       <c r="I18" s="6">
         <v>0</v>
@@ -14411,25 +13723,25 @@
     </row>
     <row r="19" spans="1:11" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>638</v>
+        <v>582</v>
       </c>
       <c r="C19" s="7">
         <v>0</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>596</v>
+        <v>540</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>597</v>
+        <v>541</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>639</v>
+        <v>583</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>640</v>
+        <v>584</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>641</v>
+        <v>585</v>
       </c>
       <c r="I19" s="7">
         <v>0</v>
@@ -14446,19 +13758,19 @@
         <v>0</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>596</v>
+        <v>540</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>597</v>
+        <v>541</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>639</v>
+        <v>583</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>640</v>
+        <v>584</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>642</v>
+        <v>586</v>
       </c>
       <c r="I20" s="7">
         <v>0</v>
@@ -14469,22 +13781,22 @@
     </row>
     <row r="21" spans="1:11" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
-        <v>643</v>
+        <v>587</v>
       </c>
       <c r="C21" s="7">
         <v>100</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>615</v>
+        <v>559</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>597</v>
+        <v>541</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>616</v>
+        <v>560</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>613</v>
+        <v>557</v>
       </c>
       <c r="I21" s="7">
         <v>73</v>
@@ -14493,27 +13805,27 @@
         <v>39</v>
       </c>
       <c r="K21" s="7" t="s">
-        <v>644</v>
+        <v>588</v>
       </c>
     </row>
     <row r="22" spans="1:11" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
-        <v>645</v>
+        <v>589</v>
       </c>
       <c r="C22" s="7">
         <v>80</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>596</v>
+        <v>540</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>597</v>
+        <v>541</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>612</v>
+        <v>556</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>613</v>
+        <v>557</v>
       </c>
       <c r="I22" s="7">
         <v>46</v>
@@ -14522,27 +13834,27 @@
         <v>23</v>
       </c>
       <c r="K22" s="7" t="s">
-        <v>646</v>
+        <v>590</v>
       </c>
     </row>
     <row r="23" spans="1:11" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>647</v>
+        <v>591</v>
       </c>
       <c r="C23" s="7">
         <v>100</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>615</v>
+        <v>559</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>597</v>
+        <v>541</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>616</v>
+        <v>560</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>613</v>
+        <v>557</v>
       </c>
       <c r="I23" s="7">
         <v>72</v>
@@ -14551,27 +13863,27 @@
         <v>40</v>
       </c>
       <c r="K23" s="7" t="s">
-        <v>648</v>
+        <v>592</v>
       </c>
     </row>
     <row r="24" spans="1:11" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
-        <v>649</v>
+        <v>593</v>
       </c>
       <c r="C24" s="7">
         <v>100</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>615</v>
+        <v>559</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>597</v>
+        <v>541</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>616</v>
+        <v>560</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>613</v>
+        <v>557</v>
       </c>
       <c r="I24" s="7">
         <v>59</v>
@@ -14580,27 +13892,27 @@
         <v>31</v>
       </c>
       <c r="K24" s="7" t="s">
-        <v>650</v>
+        <v>594</v>
       </c>
     </row>
     <row r="25" spans="1:11" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>651</v>
+        <v>595</v>
       </c>
       <c r="C25" s="7">
         <v>77</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>596</v>
+        <v>540</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>597</v>
+        <v>541</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>612</v>
+        <v>556</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>613</v>
+        <v>557</v>
       </c>
       <c r="I25" s="7">
         <v>39</v>
@@ -14609,26 +13921,26 @@
         <v>21</v>
       </c>
       <c r="K25" s="7" t="s">
-        <v>652</v>
+        <v>596</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B27" s="7" t="s">
-        <v>653</v>
+        <v>597</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>654</v>
+        <v>598</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B28" s="6" t="s">
-        <v>655</v>
+        <v>599</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>656</v>
+        <v>600</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>660</v>
+        <v>604</v>
       </c>
     </row>
   </sheetData>

</xml_diff>